<commit_message>
Actualización automática de noticias - 2026-01-19
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,12 +463,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -478,77 +478,77 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PorJulieth Cicua Caballero</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
+          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
+          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -575,29 +575,29 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
+          <t>https://www.diarioadn.co/seccion/vida</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -607,12 +607,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>PorGabriela Cicero</t>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -634,17 +634,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>PorGabriela Cicero</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -666,25 +666,29 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PorDaniella Mazo González</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -694,19 +698,15 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PorJhon Bernal</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -726,47 +726,51 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>PorJimmy Nomesqui Rivera</t>
+          <t>PorJhon Bernal</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PorJimmy Nomesqui Rivera</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -776,29 +780,25 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>PorJuan Sánchez Romero</t>
-        </is>
-      </c>
+          <t>https://www.alertabogota.com/noticias/local</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -808,12 +808,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -823,29 +823,29 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+          <t>PorJuan Sánchez Romero</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -855,74 +855,106 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>PorDahana Ospina</t>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+          <t>PorDahana Ospina</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Alerta Bogotá</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>2026-01-09</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Infobae</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Barranquilla</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>PorPaula Naranjo</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-01-21
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,12 +463,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -483,24 +483,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>PorJulieth Cicua Caballero</t>
+          <t>PorSantiago Cifuentes Quintero</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -510,77 +510,77 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PorJulieth Cicua Caballero</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
+          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
+          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -607,29 +607,29 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
+          <t>https://www.diarioadn.co/seccion/vida</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -639,12 +639,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>PorGabriela Cicero</t>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -666,17 +666,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>PorGabriela Cicero</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -698,25 +698,29 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PorDaniella Mazo González</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -726,19 +730,15 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PorJhon Bernal</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -775,30 +775,34 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PorJhon Bernal</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -808,29 +812,25 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>PorJuan Sánchez Romero</t>
-        </is>
-      </c>
+          <t>https://www.alertabogota.com/noticias/local</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -840,12 +840,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -855,29 +855,29 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+          <t>PorJuan Sánchez Romero</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -887,74 +887,106 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>PorDahana Ospina</t>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+          <t>PorDahana Ospina</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Alerta Bogotá</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>2026-01-09</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Infobae</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
         <is>
           <t>Barranquilla</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>PorPaula Naranjo</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-01-22
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,12 +463,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -483,24 +483,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>PorSantiago Cifuentes Quintero</t>
+          <t>PorFrederic Dumoulin</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -510,29 +510,29 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>PorJulieth Cicua Caballero</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -542,126 +542,126 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PorSantiago Cifuentes Quintero</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
+          <t>PorJulieth Cicua Caballero</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
+          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -671,44 +671,44 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+          <t>https://www.diarioadn.co/seccion/vida</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>PorGabriela Cicero</t>
+          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -730,25 +730,29 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PorGabriela Cicero</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -758,29 +762,29 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>PorJimmy Nomesqui Rivera</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -790,57 +794,57 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>PorJhon Bernal</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>PorJhon Bernal</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -850,17 +854,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>PorJuan Sánchez Romero</t>
+          <t>PorJimmy Nomesqui Rivera</t>
         </is>
       </c>
     </row>
@@ -872,39 +876,35 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
-        </is>
-      </c>
+          <t>https://www.alertabogota.com/noticias/local</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -919,74 +919,138 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>PorDahana Ospina</t>
+          <t>PorJuan Sánchez Romero</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Sin identificar</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>PorDahana Ospina</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Alerta Bogotá</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>2026-01-09</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Infobae</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
         <is>
           <t>Barranquilla</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>PorPaula Naranjo</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-01-23
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -720,7 +720,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -730,19 +730,15 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PorGabriela Cicero</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -784,7 +780,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -794,15 +790,19 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PorGabriela Cicero</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-01-24
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,12 +463,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -478,17 +478,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>PorFrederic Dumoulin</t>
+          <t>PorPaula Naranjo</t>
         </is>
       </c>
     </row>
@@ -527,12 +527,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -547,24 +547,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>PorSantiago Cifuentes Quintero</t>
+          <t>PorFrederic Dumoulin</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -579,24 +579,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>PorJulieth Cicua Caballero</t>
+          <t>PorSantiago Cifuentes Quintero</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -606,77 +606,77 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PorJulieth Cicua Caballero</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
+          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
+          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -703,42 +703,46 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
+          <t>https://www.diarioadn.co/seccion/vida</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -748,7 +752,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -758,17 +762,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>PorGabriela Cicero</t>
         </is>
       </c>
     </row>
@@ -780,7 +784,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -790,29 +794,29 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>PorGabriela Cicero</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -822,19 +826,15 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>PorJhon Bernal</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -871,30 +871,34 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PorJhon Bernal</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -904,29 +908,25 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>PorJuan Sánchez Romero</t>
-        </is>
-      </c>
+          <t>https://www.alertabogota.com/noticias/local</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -936,12 +936,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -951,29 +951,29 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+          <t>PorJuan Sánchez Romero</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -983,74 +983,106 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>PorDahana Ospina</t>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+          <t>PorDahana Ospina</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Alerta Bogotá</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>2026-01-09</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Infobae</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
         <is>
           <t>Barranquilla</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>PorPaula Naranjo</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-01-25
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,81 +463,77 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
+          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>PorPaula Naranjo</t>
+          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PorDaniella Mazo González</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -547,24 +543,20 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PorFrederic Dumoulin</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -574,29 +566,29 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>PorSantiago Cifuentes Quintero</t>
+          <t>PorPaula Naranjo</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -611,24 +603,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>PorJulieth Cicua Caballero</t>
+          <t>PorFrederic Dumoulin</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -638,62 +630,66 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PorDaniella Mazo González</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
+          <t>PorSantiago Cifuentes Quintero</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -703,148 +699,148 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
+          <t>PorJulieth Cicua Caballero</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>PorGabriela Cicero</t>
+          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://www.diarioadn.co/seccion/vida</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -859,24 +855,20 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>PorJimmy Nomesqui Rivera</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -886,57 +878,61 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>PorJhon Bernal</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>PorGabriela Cicero</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -946,34 +942,34 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>PorJuan Sánchez Romero</t>
+          <t>PorJimmy Nomesqui Rivera</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -983,106 +979,198 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+          <t>PorJhon Bernal</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>PorDahana Ospina</t>
-        </is>
-      </c>
+          <t>https://www.alertabogota.com/noticias/local</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+          <t>PorJuan Sánchez Romero</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Diario ADN</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Sin identificar</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Sin identificar</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>PorDahana Ospina</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Alerta Bogotá</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>2026-01-09</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Infobae</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
         <is>
           <t>Barranquilla</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>PorPaula Naranjo</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-01-26
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,49 +463,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -515,7 +511,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -523,17 +519,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -543,57 +539,57 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>https://www.pulzo.com/nacion/hablo-papa-ninas-envenenadas-con-talio-bogota-PP5011766A</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>“Para mí fue un error”: habló papá de una de las niñas envenenadas con talio</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PorPaula Naranjo</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -603,56 +599,52 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
+          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>PorFrederic Dumoulin</t>
+          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PorDaniella Mazo González</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -662,29 +654,29 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>PorSantiago Cifuentes Quintero</t>
+          <t>PorPaula Naranjo</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -694,29 +686,29 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>PorJulieth Cicua Caballero</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -726,62 +718,66 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PorFrederic Dumoulin</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
+          <t>PorSantiago Cifuentes Quintero</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -791,61 +787,57 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
+          <t>PorJulieth Cicua Caballero</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -855,57 +847,61 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
+          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://www.diarioadn.co/seccion/vida</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -915,24 +911,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>PorGabriela Cicero</t>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -942,29 +938,29 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>PorJimmy Nomesqui Rivera</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -979,39 +975,39 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>PorJhon Bernal</t>
+          <t>PorGabriela Cicero</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -1019,12 +1015,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1039,138 +1035,230 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>PorJuan Sánchez Romero</t>
+          <t>PorJhon Bernal</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+          <t>PorJimmy Nomesqui Rivera</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>PorDahana Ospina</t>
-        </is>
-      </c>
+          <t>https://www.alertabogota.com/noticias/local</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+          <t>PorJuan Sánchez Romero</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Diario ADN</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Sin identificar</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Sin identificar</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>PorDahana Ospina</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Alerta Bogotá</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>2026-01-09</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Infobae</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
         <is>
           <t>Barranquilla</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>PorPaula Naranjo</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-01-27
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,12 +463,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -483,7 +483,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -524,44 +524,40 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/hablo-papa-ninas-envenenadas-con-talio-bogota-PP5011766A</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>“Para mí fue un error”: habló papá de una de las niñas envenenadas con talio</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -571,10 +567,14 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>https://www.pulzo.com/nacion/hablo-papa-ninas-envenenadas-con-talio-bogota-PP5011766A</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>“Para mí fue un error”: habló papá de una de las niñas envenenadas con talio</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -584,12 +584,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -599,14 +599,10 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -616,12 +612,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -631,52 +627,52 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PorPaula Naranjo</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -691,12 +687,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>PorPaula Naranjo</t>
         </is>
       </c>
     </row>
@@ -708,7 +704,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -718,29 +714,29 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>PorFrederic Dumoulin</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -755,24 +751,24 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>PorSantiago Cifuentes Quintero</t>
+          <t>PorFrederic Dumoulin</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -787,24 +783,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>PorJulieth Cicua Caballero</t>
+          <t>PorSantiago Cifuentes Quintero</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -814,77 +810,77 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>PorJulieth Cicua Caballero</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
+          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
+          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
         </is>
       </c>
     </row>
@@ -896,7 +892,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -911,44 +907,44 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
+          <t>https://www.diarioadn.co/seccion/vida</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
         </is>
       </c>
     </row>
@@ -1015,12 +1011,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1030,17 +1026,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>PorJhon Bernal</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1048,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1062,47 +1058,51 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>PorJimmy Nomesqui Rivera</t>
+          <t>PorJhon Bernal</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>PorJimmy Nomesqui Rivera</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1112,29 +1112,25 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>PorJuan Sánchez Romero</t>
-        </is>
-      </c>
+          <t>https://www.alertabogota.com/noticias/local</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1144,12 +1140,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1159,29 +1155,29 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+          <t>PorJuan Sánchez Romero</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1191,74 +1187,106 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>PorDahana Ospina</t>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+          <t>PorDahana Ospina</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Alerta Bogotá</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>2026-01-09</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Infobae</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
         <is>
           <t>Barranquilla</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>PorPaula Naranjo</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-01-29
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,40 +463,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
+          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/inicio</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -506,12 +510,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -579,17 +583,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -599,7 +603,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -612,12 +616,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -627,14 +631,10 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -644,12 +644,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -659,52 +659,52 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
+          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PorPaula Naranjo</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -719,12 +719,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>PorPaula Naranjo</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -746,29 +746,29 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>PorFrederic Dumoulin</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -783,24 +783,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>PorSantiago Cifuentes Quintero</t>
+          <t>PorFrederic Dumoulin</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -815,24 +815,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>PorJulieth Cicua Caballero</t>
+          <t>PorSantiago Cifuentes Quintero</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -842,77 +842,77 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>PorJulieth Cicua Caballero</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
+          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
+          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
         </is>
       </c>
     </row>
@@ -951,17 +951,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -971,12 +971,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+          <t>https://www.diarioadn.co/seccion/vida</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>PorGabriela Cicero</t>
+          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -998,15 +998,19 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>PorGabriela Cicero</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1016,7 +1020,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1026,29 +1030,25 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>PorDaniella Mazo González</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1058,17 +1058,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>PorJhon Bernal</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1090,47 +1090,51 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>PorJimmy Nomesqui Rivera</t>
+          <t>PorJhon Bernal</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>PorJimmy Nomesqui Rivera</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1140,29 +1144,25 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>PorJuan Sánchez Romero</t>
-        </is>
-      </c>
+          <t>https://www.alertabogota.com/noticias/local</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1172,12 +1172,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1187,29 +1187,29 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+          <t>PorJuan Sánchez Romero</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1219,74 +1219,106 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>PorDahana Ospina</t>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+          <t>PorDahana Ospina</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Alerta Bogotá</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>2026-01-09</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Infobae</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
         <is>
           <t>Barranquilla</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>PorPaula Naranjo</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-02-02
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,122 +463,126 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
+          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/inicio</t>
+          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+          <t>PorJhoan Pardo</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
+          <t>1Masacre en Colombia: ataque de sicarios dejó a tres jóvenes muertos en pleno parque</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>https://www.pulzo.com/nacion/masacre-riohacha-ataque-sicarios-deja-tres-muertos-hay-dura-hipotesis-PP5023694A</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Masacre en Colombia: ataque de sicarios dejó a tres jóvenes muertos en pleno parque</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
+          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/inicio</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/hablo-papa-ninas-envenenadas-con-talio-bogota-PP5011766A</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>“Para mí fue un error”: habló papá de una de las niñas envenenadas con talio</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -588,12 +592,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -603,35 +607,39 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>https://www.pulzo.com/nacion/hablo-papa-ninas-envenenadas-con-talio-bogota-PP5011766A</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>“Para mí fue un error”: habló papá de una de las niñas envenenadas con talio</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -639,17 +647,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -659,14 +667,10 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -691,7 +695,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion</t>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -699,76 +703,72 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
+          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>PorPaula Naranjo</t>
+          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>PorDaniella Mazo González</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -778,29 +778,29 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>PorFrederic Dumoulin</t>
+          <t>PorPaula Naranjo</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -810,29 +810,29 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>PorSantiago Cifuentes Quintero</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -847,24 +847,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>PorJulieth Cicua Caballero</t>
+          <t>PorFrederic Dumoulin</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -874,126 +874,126 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PorSantiago Cifuentes Quintero</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
+          <t>PorJulieth Cicua Caballero</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
+          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
+          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1003,42 +1003,46 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+          <t>https://www.diarioadn.co/seccion/vida</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>PorGabriela Cicero</t>
+          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1048,7 +1052,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1058,29 +1062,25 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>PorDaniella Mazo González</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1090,29 +1090,29 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>PorJhon Bernal</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1122,57 +1122,61 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>PorJimmy Nomesqui Rivera</t>
+          <t>PorGabriela Cicero</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>PorJhon Bernal</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1182,17 +1186,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>PorJuan Sánchez Romero</t>
+          <t>PorJimmy Nomesqui Rivera</t>
         </is>
       </c>
     </row>
@@ -1204,39 +1208,35 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
-        </is>
-      </c>
+          <t>https://www.alertabogota.com/noticias/local</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1251,74 +1251,138 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>PorDahana Ospina</t>
+          <t>PorJuan Sánchez Romero</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Sin identificar</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>PorDahana Ospina</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Alerta Bogotá</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>2026-01-09</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Infobae</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
         <is>
           <t>Barranquilla</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>PorPaula Naranjo</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-02-05
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,32 +463,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+          <t>https://www.pulzo.com/nacion/bogota/muertos-bogota-hoy-menor-edad-fue-asesinado-por-no-dejarse-robar-celular-PP5030714</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>PorJhoan Pardo</t>
+          <t>Menor de edad fue asesinado en Bogotá, tras no dejarse robar el celular; recién salía de su casa</t>
         </is>
       </c>
     </row>
@@ -527,94 +527,94 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
+          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/inicio</t>
+          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+          <t>PorJhoan Pardo</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
+          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/inicio</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/hablo-papa-ninas-envenenadas-con-talio-bogota-PP5011766A</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>“Para mí fue un error”: habló papá de una de las niñas envenenadas con talio</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -624,25 +624,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>https://www.pulzo.com/nacion/hablo-papa-ninas-envenenadas-con-talio-bogota-PP5011766A</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>“Para mí fue un error”: habló papá de una de las niñas envenenadas con talio</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -652,7 +656,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
+          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -662,12 +666,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
+          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -675,17 +679,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -695,7 +699,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -708,12 +712,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -723,14 +727,10 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -740,12 +740,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -755,52 +755,52 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>PorPaula Naranjo</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -815,12 +815,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>PorPaula Naranjo</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -842,29 +842,29 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>PorFrederic Dumoulin</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -879,24 +879,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>PorSantiago Cifuentes Quintero</t>
+          <t>PorFrederic Dumoulin</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -911,24 +911,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>PorJulieth Cicua Caballero</t>
+          <t>PorSantiago Cifuentes Quintero</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -938,77 +938,77 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>PorJulieth Cicua Caballero</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
+          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
+          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
         </is>
       </c>
     </row>
@@ -1047,30 +1047,34 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/vida</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1080,7 +1084,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1090,19 +1094,15 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>PorDaniella Mazo González</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1122,29 +1122,29 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>PorGabriela Cicero</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1159,12 +1159,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>PorJhon Bernal</t>
+          <t>PorGabriela Cicero</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1186,47 +1186,51 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>PorJimmy Nomesqui Rivera</t>
+          <t>PorJhon Bernal</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>PorJimmy Nomesqui Rivera</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1236,29 +1240,25 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>PorJuan Sánchez Romero</t>
-        </is>
-      </c>
+          <t>https://www.alertabogota.com/noticias/local</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1268,12 +1268,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1283,29 +1283,29 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+          <t>PorJuan Sánchez Romero</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1315,74 +1315,106 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>PorDahana Ospina</t>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+          <t>PorDahana Ospina</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Alerta Bogotá</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>2026-01-09</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Infobae</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
         <is>
           <t>Barranquilla</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>PorPaula Naranjo</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-02-06
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,12 +463,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -483,24 +483,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/muertos-bogota-hoy-menor-edad-fue-asesinado-por-no-dejarse-robar-celular-PP5030714</t>
+          <t>https://www.pulzo.com/nacion/bogota/cuantos-colegios-han-cerrado-bogota-varios-eran-pupys-con-buenos-icfes-PP5032950</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Menor de edad fue asesinado en Bogotá, tras no dejarse robar el celular; recién salía de su casa</t>
+          <t>Colegios más 'puppys' de Bogotá que han cerrado: fueron 'top' en Icfes y con estudiantes famosos</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1Masacre en Colombia: ataque de sicarios dejó a tres jóvenes muertos en pleno parque</t>
+          <t>1Colegios en Colombia no alcanzan ni el 50 % de estudiantes: les tocará hasta regalar los pupitres</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -515,88 +515,88 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/masacre-riohacha-ataque-sicarios-deja-tres-muertos-hay-dura-hipotesis-PP5023694A</t>
+          <t>https://www.pulzo.com/nacion/cuantos-colegios-han-cerrado-colombia-1-cada-5-no-logra-50-ocupacion-PP5031212</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Masacre en Colombia: ataque de sicarios dejó a tres jóvenes muertos en pleno parque</t>
+          <t>Colegios en Colombia no alcanzan ni el 50 % de estudiantes: les tocará hasta regalar los pupitres</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+          <t>https://www.pulzo.com/nacion/bogota/muertos-bogota-hoy-menor-edad-fue-asesinado-por-no-dejarse-robar-celular-PP5030714</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>PorJhoan Pardo</t>
+          <t>Menor de edad fue asesinado en Bogotá, tras no dejarse robar el celular; recién salía de su casa</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
+          <t>1Masacre en Colombia: ataque de sicarios dejó a tres jóvenes muertos en pleno parque</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/inicio</t>
+          <t>https://www.pulzo.com/nacion/masacre-riohacha-ataque-sicarios-deja-tres-muertos-hay-dura-hipotesis-PP5023694A</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+          <t>Masacre en Colombia: ataque de sicarios dejó a tres jóvenes muertos en pleno parque</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
+          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -606,30 +606,34 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PorJhoan Pardo</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -639,24 +643,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/hablo-papa-ninas-envenenadas-con-talio-bogota-PP5011766A</t>
+          <t>https://www.diarioadn.co/seccion/inicio</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>“Para mí fue un error”: habló papá de una de las niñas envenenadas con talio</t>
+          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -671,7 +675,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -684,12 +688,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -699,35 +703,39 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>https://www.pulzo.com/nacion/hablo-papa-ninas-envenenadas-con-talio-bogota-PP5011766A</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>“Para mí fue un error”: habló papá de una de las niñas envenenadas con talio</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -735,17 +743,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -755,14 +763,10 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -787,7 +791,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion</t>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -795,76 +799,72 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
+          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>PorPaula Naranjo</t>
+          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>PorDaniella Mazo González</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -874,29 +874,29 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>PorFrederic Dumoulin</t>
+          <t>PorPaula Naranjo</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -906,29 +906,29 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>PorSantiago Cifuentes Quintero</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -943,24 +943,24 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>PorJulieth Cicua Caballero</t>
+          <t>PorFrederic Dumoulin</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -970,169 +970,173 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>PorSantiago Cifuentes Quintero</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
+          <t>PorJulieth Cicua Caballero</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
+          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
+          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/vida</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1148,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1154,29 +1158,25 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>PorGabriela Cicero</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1186,29 +1186,29 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>PorJhon Bernal</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1218,57 +1218,61 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>PorJimmy Nomesqui Rivera</t>
+          <t>PorGabriela Cicero</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>PorJhon Bernal</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1278,17 +1282,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>PorJuan Sánchez Romero</t>
+          <t>PorJimmy Nomesqui Rivera</t>
         </is>
       </c>
     </row>
@@ -1300,39 +1304,35 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
-        </is>
-      </c>
+          <t>https://www.alertabogota.com/noticias/local</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1347,74 +1347,138 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>PorDahana Ospina</t>
+          <t>PorJuan Sánchez Romero</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Sin identificar</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>PorDahana Ospina</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Alerta Bogotá</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>2026-01-09</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Infobae</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
         <is>
           <t>Barranquilla</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>PorPaula Naranjo</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-02-07
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,12 +463,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -478,29 +478,29 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/cuantos-colegios-han-cerrado-bogota-varios-eran-pupys-con-buenos-icfes-PP5032950</t>
+          <t>https://www.pulzo.com/nacion/bogota/veterinario-zulma-guzman-pago-domiciliario-que-envio-frambuesas-PP5033639A</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Colegios más 'puppys' de Bogotá que han cerrado: fueron 'top' en Icfes y con estudiantes famosos</t>
+          <t>Nuevo implicado en muerte de niñas con talio: veterinario de Zulma Guzmán le pagó a domiciliario</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1Colegios en Colombia no alcanzan ni el 50 % de estudiantes: les tocará hasta regalar los pupitres</t>
+          <t>1Pelea de jóvenes frente a colegio de Bogotá acabó en tragedia: menor murió por herida con arma</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -510,29 +510,29 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/cuantos-colegios-han-cerrado-colombia-1-cada-5-no-logra-50-ocupacion-PP5031212</t>
+          <t>https://www.pulzo.com/nacion/bogota/rina-afuera-colegio-la-candelaria-bogota-dejo-menor-fallecido-PP5033637A</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Colegios en Colombia no alcanzan ni el 50 % de estudiantes: les tocará hasta regalar los pupitres</t>
+          <t>Pelea de jóvenes frente a colegio de Bogotá acabó en tragedia: menor murió por herida con arma</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1Colegios en Colombia no alcanzan ni el 50 % de estudiantes: les tocará hasta regalar los pupitres</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -542,29 +542,29 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/muertos-bogota-hoy-menor-edad-fue-asesinado-por-no-dejarse-robar-celular-PP5030714</t>
+          <t>https://www.pulzo.com/nacion/cuantos-colegios-han-cerrado-colombia-1-cada-5-no-logra-50-ocupacion-PP5031212</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Menor de edad fue asesinado en Bogotá, tras no dejarse robar el celular; recién salía de su casa</t>
+          <t>Colegios en Colombia no alcanzan ni el 50 % de estudiantes: les tocará hasta regalar los pupitres</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1Masacre en Colombia: ataque de sicarios dejó a tres jóvenes muertos en pleno parque</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -574,126 +574,130 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/masacre-riohacha-ataque-sicarios-deja-tres-muertos-hay-dura-hipotesis-PP5023694A</t>
+          <t>https://www.pulzo.com/nacion/bogota/cuantos-colegios-han-cerrado-bogota-varios-eran-pupys-con-buenos-icfes-PP5032950</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Masacre en Colombia: ataque de sicarios dejó a tres jóvenes muertos en pleno parque</t>
+          <t>Colegios más 'puppys' de Bogotá que han cerrado: fueron 'top' en Icfes y con estudiantes famosos</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+          <t>https://www.pulzo.com/nacion/bogota/muertos-bogota-hoy-menor-edad-fue-asesinado-por-no-dejarse-robar-celular-PP5030714</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>PorJhoan Pardo</t>
+          <t>Menor de edad fue asesinado en Bogotá, tras no dejarse robar el celular; recién salía de su casa</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
+          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/inicio</t>
+          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+          <t>PorJhoan Pardo</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
+          <t>1Masacre en Colombia: ataque de sicarios dejó a tres jóvenes muertos en pleno parque</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
+          <t>https://www.pulzo.com/nacion/masacre-riohacha-ataque-sicarios-deja-tres-muertos-hay-dura-hipotesis-PP5023694A</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Masacre en Colombia: ataque de sicarios dejó a tres jóvenes muertos en pleno parque</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -703,24 +707,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/hablo-papa-ninas-envenenadas-con-talio-bogota-PP5011766A</t>
+          <t>https://www.diarioadn.co/seccion/inicio</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>“Para mí fue un error”: habló papá de una de las niñas envenenadas con talio</t>
+          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -735,7 +739,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -748,12 +752,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -763,35 +767,39 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>https://www.pulzo.com/nacion/hablo-papa-ninas-envenenadas-con-talio-bogota-PP5011766A</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>“Para mí fue un error”: habló papá de una de las niñas envenenadas con talio</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -799,17 +807,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -819,14 +827,10 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -851,7 +855,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion</t>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -859,76 +863,72 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
+          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>PorPaula Naranjo</t>
+          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>PorDaniella Mazo González</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -938,29 +938,29 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>PorFrederic Dumoulin</t>
+          <t>PorPaula Naranjo</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -970,29 +970,29 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>PorSantiago Cifuentes Quintero</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1007,24 +1007,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>PorJulieth Cicua Caballero</t>
+          <t>PorFrederic Dumoulin</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1034,169 +1034,173 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>PorSantiago Cifuentes Quintero</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
+          <t>PorJulieth Cicua Caballero</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
+          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/vida</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1212,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1218,29 +1222,25 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>PorGabriela Cicero</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1250,29 +1250,29 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>PorJhon Bernal</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1282,57 +1282,61 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>PorJimmy Nomesqui Rivera</t>
+          <t>PorGabriela Cicero</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>PorJhon Bernal</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1342,17 +1346,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>PorJuan Sánchez Romero</t>
+          <t>PorJimmy Nomesqui Rivera</t>
         </is>
       </c>
     </row>
@@ -1364,39 +1368,35 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
-        </is>
-      </c>
+          <t>https://www.alertabogota.com/noticias/local</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1411,74 +1411,138 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>PorDahana Ospina</t>
+          <t>PorJuan Sánchez Romero</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Sin identificar</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>PorDahana Ospina</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Alerta Bogotá</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>2026-01-09</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Infobae</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
         <is>
           <t>Barranquilla</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>PorPaula Naranjo</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-02-08
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -960,7 +960,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -970,17 +970,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>PorFrederic Dumoulin</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1002,17 +1002,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>PorFrederic Dumoulin</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1222,15 +1222,19 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>PorDaniella Mazo González</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1240,7 +1244,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1250,17 +1254,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>PorGabriela Cicero</t>
         </is>
       </c>
     </row>
@@ -1272,7 +1276,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1282,19 +1286,15 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>PorGabriela Cicero</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-02-09
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -960,7 +960,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -970,17 +970,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>PorFrederic Dumoulin</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1002,17 +1002,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>PorFrederic Dumoulin</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1222,17 +1222,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>PorGabriela Cicero</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1254,19 +1254,15 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>PorGabriela Cicero</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1276,7 +1272,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1286,15 +1282,19 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>PorDaniella Mazo González</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-02-10
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -960,7 +960,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -970,17 +970,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>PorFrederic Dumoulin</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1002,17 +1002,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>PorFrederic Dumoulin</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1222,19 +1222,15 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>PorGabriela Cicero</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1244,7 +1240,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1254,15 +1250,19 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>PorDaniella Mazo González</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1282,17 +1282,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>PorGabriela Cicero</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-02-11
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -960,7 +960,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -970,17 +970,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>PorFrederic Dumoulin</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1002,17 +1002,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>PorFrederic Dumoulin</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1222,15 +1222,19 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>PorDaniella Mazo González</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1240,7 +1244,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1250,17 +1254,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>PorGabriela Cicero</t>
         </is>
       </c>
     </row>
@@ -1272,7 +1276,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1282,19 +1286,15 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>PorGabriela Cicero</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-02-12
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,17 +463,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -483,12 +483,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/veterinario-zulma-guzman-pago-domiciliario-que-envio-frambuesas-PP5033639A</t>
+          <t>https://www.infobae.com/colombia/2026/02/12/la-falta-de-sueno-deteriora-la-salud-cerebral-y-emocional-desde-la-infancia-60-de-los-ninos-y-adolescentes-no-duerme-las-horas-recomendadas/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Nuevo implicado en muerte de niñas con talio: veterinario de Zulma Guzmán le pagó a domiciliario</t>
+          <t>PorLina Muñoz Medina</t>
         </is>
       </c>
     </row>
@@ -527,12 +527,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1Colegios en Colombia no alcanzan ni el 50 % de estudiantes: les tocará hasta regalar los pupitres</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -542,17 +542,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/cuantos-colegios-han-cerrado-colombia-1-cada-5-no-logra-50-ocupacion-PP5031212</t>
+          <t>https://www.pulzo.com/nacion/bogota/veterinario-zulma-guzman-pago-domiciliario-que-envio-frambuesas-PP5033639A</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Colegios en Colombia no alcanzan ni el 50 % de estudiantes: les tocará hasta regalar los pupitres</t>
+          <t>Nuevo implicado en muerte de niñas con talio: veterinario de Zulma Guzmán le pagó a domiciliario</t>
         </is>
       </c>
     </row>
@@ -591,12 +591,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1Colegios en Colombia no alcanzan ni el 50 % de estudiantes: les tocará hasta regalar los pupitres</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -606,49 +606,49 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/muertos-bogota-hoy-menor-edad-fue-asesinado-por-no-dejarse-robar-celular-PP5030714</t>
+          <t>https://www.pulzo.com/nacion/cuantos-colegios-han-cerrado-colombia-1-cada-5-no-logra-50-ocupacion-PP5031212</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Menor de edad fue asesinado en Bogotá, tras no dejarse robar el celular; recién salía de su casa</t>
+          <t>Colegios en Colombia no alcanzan ni el 50 % de estudiantes: les tocará hasta regalar los pupitres</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+          <t>https://www.pulzo.com/nacion/bogota/muertos-bogota-hoy-menor-edad-fue-asesinado-por-no-dejarse-robar-celular-PP5030714</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>PorJhoan Pardo</t>
+          <t>Menor de edad fue asesinado en Bogotá, tras no dejarse robar el celular; recién salía de su casa</t>
         </is>
       </c>
     </row>
@@ -660,121 +660,121 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1Masacre en Colombia: ataque de sicarios dejó a tres jóvenes muertos en pleno parque</t>
+          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/masacre-riohacha-ataque-sicarios-deja-tres-muertos-hay-dura-hipotesis-PP5023694A</t>
+          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Masacre en Colombia: ataque de sicarios dejó a tres jóvenes muertos en pleno parque</t>
+          <t>PorJhoan Pardo</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
+          <t>1Masacre en Colombia: ataque de sicarios dejó a tres jóvenes muertos en pleno parque</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/inicio</t>
+          <t>https://www.pulzo.com/nacion/masacre-riohacha-ataque-sicarios-deja-tres-muertos-hay-dura-hipotesis-PP5023694A</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+          <t>Masacre en Colombia: ataque de sicarios dejó a tres jóvenes muertos en pleno parque</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
+          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/inicio</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/hablo-papa-ninas-envenenadas-con-talio-bogota-PP5011766A</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>“Para mí fue un error”: habló papá de una de las niñas envenenadas con talio</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -784,25 +784,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>https://www.pulzo.com/nacion/hablo-papa-ninas-envenenadas-con-talio-bogota-PP5011766A</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>“Para mí fue un error”: habló papá de una de las niñas envenenadas con talio</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -812,7 +816,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
+          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -822,12 +826,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
+          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -835,17 +839,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -855,7 +859,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -868,12 +872,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -883,14 +887,10 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -900,12 +900,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -915,52 +915,52 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
+          <t>https://www.pulzo.com/nacion/intencione-zulma-guzman-daria-giro-caso-ninas-envenenadas-bogota-PP5009034A</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Dan versión sobre las verdaderas intenciones de Zulma Guzmán: daría giro a caso de niñas envenenadas</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>PorPaula Naranjo</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -975,12 +975,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>PorPaula Naranjo</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1002,29 +1002,29 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>PorFrederic Dumoulin</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>La viuda del último sha de Irán dijo que quiere regresar: “La juventud y todo el pueblo iraní serán finalmente libres”</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1039,24 +1039,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://www.infobae.com/america/mundo/2026/01/21/la-viuda-del-ultimo-sha-de-iran-dijo-que-quiere-regresar-la-juventud-y-todo-el-pueblo-irani-seran-finalmente-libres/</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>PorSantiago Cifuentes Quintero</t>
+          <t>PorFrederic Dumoulin</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1071,24 +1071,24 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>PorJulieth Cicua Caballero</t>
+          <t>PorSantiago Cifuentes Quintero</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1098,77 +1098,77 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>PorJulieth Cicua Caballero</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
+          <t>https://www.pulzo.com/nacion/que-trata-cambio-estructural-educacion-colombia-por-giro-pae-PP4995431</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
+          <t>Anuncian cambio estructural para educación en Colombia: nueva resolución toca a 550.000 niños</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Por qué tantas personas de 30 siguen actuando como adolescentes al elegir pareja, según expertos en comportamiento</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1195,44 +1195,44 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
+          <t>https://www.diarioadn.co/seccion/vida</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+          <t>Afirman que la madurez emocional no llega sola con los años sino que se construye.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>PorDaniella Mazo González</t>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1254,17 +1254,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>PorGabriela Cicero</t>
+          <t>PorDaniella Mazo González</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1286,25 +1286,29 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>PorGabriela Cicero</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>Menor de edad colombiana tardó seis años para reencontrarse con su mamá en España, pero murió en grave accidente de tránsito</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1314,19 +1318,15 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>PorJhon Bernal</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/15/menor-de-edad-colombiana-tardo-seis-anos-para-reencontrarse-con-su-mama-en-espana-pero-murio-en-grave-accidente-de-transito/</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1346,47 +1346,51 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>PorJimmy Nomesqui Rivera</t>
+          <t>PorJhon Bernal</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>PorJimmy Nomesqui Rivera</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1396,29 +1400,25 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>PorJuan Sánchez Romero</t>
-        </is>
-      </c>
+          <t>https://www.alertabogota.com/noticias/local</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1428,12 +1428,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1443,29 +1443,29 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+          <t>PorJuan Sánchez Romero</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1475,74 +1475,106 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>PorDahana Ospina</t>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Madre denuncia a Karina García por grabar a su hija menor de edad sin autorización durante una transmisión en vivo</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+          <t>https://www.infobae.com/colombia/2026/01/12/madre-denuncia-a-karina-garcia-por-grabar-a-su-hija-menor-de-edad-sin-autorizacion-durante-una-transmision-en-vivo/</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+          <t>PorDahana Ospina</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Alerta Bogotá</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://www.alertabogota.com/noticias/local/estudiantes-respiran-con-el-aumento-del-pasaje-de-transmilenio-no-tendran-que-gastarse-lo-del-almuerzo</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>El incremento en el pasaje no será una barrera para que los estudiantes continúen asistiendo a clases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>2026-01-09</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Infobae</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
         <is>
           <t>Barranquilla</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>PorPaula Naranjo</t>
         </is>

</xml_diff>

<commit_message>
Limpiar resúmenes duplicados en datos históricos (195 de 226)
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2021" uniqueCount="618">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1826" uniqueCount="618">
   <si>
     <t>fecha</t>
   </si>
@@ -2324,9 +2324,6 @@
       <c r="H3" s="2" t="s">
         <v>384</v>
       </c>
-      <c r="I3" t="s">
-        <v>73</v>
-      </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
@@ -2411,9 +2408,6 @@
       <c r="H6" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="I6" t="s">
-        <v>76</v>
-      </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
@@ -2440,9 +2434,6 @@
       <c r="H7" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="I7" t="s">
-        <v>77</v>
-      </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
@@ -2469,9 +2460,6 @@
       <c r="H8" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="I8" t="s">
-        <v>78</v>
-      </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
@@ -2498,9 +2486,6 @@
       <c r="H9" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="I9" t="s">
-        <v>79</v>
-      </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
@@ -2527,9 +2512,6 @@
       <c r="H10" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="I10" t="s">
-        <v>80</v>
-      </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" t="s">
@@ -2556,9 +2538,6 @@
       <c r="H11" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="I11" t="s">
-        <v>81</v>
-      </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" t="s">
@@ -2585,9 +2564,6 @@
       <c r="H12" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="I12" t="s">
-        <v>82</v>
-      </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" t="s">
@@ -2614,9 +2590,6 @@
       <c r="H13" s="2" t="s">
         <v>394</v>
       </c>
-      <c r="I13" t="s">
-        <v>83</v>
-      </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" t="s">
@@ -2643,9 +2616,6 @@
       <c r="H14" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="I14" t="s">
-        <v>84</v>
-      </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" t="s">
@@ -2672,9 +2642,6 @@
       <c r="H15" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="I15" t="s">
-        <v>85</v>
-      </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" t="s">
@@ -2701,9 +2668,6 @@
       <c r="H16" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="I16" t="s">
-        <v>86</v>
-      </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
@@ -2730,9 +2694,6 @@
       <c r="H17" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="I17" t="s">
-        <v>87</v>
-      </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
@@ -2759,9 +2720,6 @@
       <c r="H18" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="I18" t="s">
-        <v>88</v>
-      </c>
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
@@ -2788,9 +2746,6 @@
       <c r="H19" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="I19" t="s">
-        <v>89</v>
-      </c>
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
@@ -2817,9 +2772,6 @@
       <c r="H20" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="I20" t="s">
-        <v>90</v>
-      </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
@@ -2846,9 +2798,6 @@
       <c r="H21" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="I21" t="s">
-        <v>91</v>
-      </c>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" t="s">
@@ -2875,9 +2824,6 @@
       <c r="H22" s="2" t="s">
         <v>403</v>
       </c>
-      <c r="I22" t="s">
-        <v>92</v>
-      </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" t="s">
@@ -2904,9 +2850,6 @@
       <c r="H23" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="I23" t="s">
-        <v>93</v>
-      </c>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" t="s">
@@ -2933,9 +2876,6 @@
       <c r="H24" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="I24" t="s">
-        <v>94</v>
-      </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" t="s">
@@ -2962,9 +2902,6 @@
       <c r="H25" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="I25" t="s">
-        <v>95</v>
-      </c>
     </row>
     <row r="26" spans="1:9">
       <c r="A26" t="s">
@@ -2991,9 +2928,6 @@
       <c r="H26" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="I26" t="s">
-        <v>96</v>
-      </c>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" t="s">
@@ -3075,9 +3009,6 @@
       <c r="H29" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="I29" t="s">
-        <v>99</v>
-      </c>
     </row>
     <row r="30" spans="1:9">
       <c r="A30" t="s">
@@ -3104,9 +3035,6 @@
       <c r="H30" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="I30" t="s">
-        <v>100</v>
-      </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" t="s">
@@ -3133,9 +3061,6 @@
       <c r="H31" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="I31" t="s">
-        <v>101</v>
-      </c>
     </row>
     <row r="32" spans="1:9">
       <c r="A32" t="s">
@@ -3191,9 +3116,6 @@
       <c r="H33" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="I33" t="s">
-        <v>103</v>
-      </c>
     </row>
     <row r="34" spans="1:9">
       <c r="A34" t="s">
@@ -3249,9 +3171,6 @@
       <c r="H35" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="I35" t="s">
-        <v>105</v>
-      </c>
     </row>
     <row r="36" spans="1:9">
       <c r="A36" t="s">
@@ -3278,9 +3197,6 @@
       <c r="H36" s="2" t="s">
         <v>417</v>
       </c>
-      <c r="I36" t="s">
-        <v>106</v>
-      </c>
     </row>
     <row r="37" spans="1:9">
       <c r="A37" t="s">
@@ -3307,9 +3223,6 @@
       <c r="H37" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="I37" t="s">
-        <v>107</v>
-      </c>
     </row>
     <row r="38" spans="1:9">
       <c r="A38" t="s">
@@ -3336,9 +3249,6 @@
       <c r="H38" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="I38" t="s">
-        <v>93</v>
-      </c>
     </row>
     <row r="39" spans="1:9">
       <c r="A39" t="s">
@@ -3365,9 +3275,6 @@
       <c r="H39" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="I39" t="s">
-        <v>108</v>
-      </c>
     </row>
     <row r="40" spans="1:9">
       <c r="A40" t="s">
@@ -3394,9 +3301,6 @@
       <c r="H40" s="2" t="s">
         <v>421</v>
       </c>
-      <c r="I40" t="s">
-        <v>105</v>
-      </c>
     </row>
     <row r="41" spans="1:9">
       <c r="A41" t="s">
@@ -3423,9 +3327,6 @@
       <c r="H41" s="2" t="s">
         <v>422</v>
       </c>
-      <c r="I41" t="s">
-        <v>109</v>
-      </c>
     </row>
     <row r="42" spans="1:9">
       <c r="A42" t="s">
@@ -3452,9 +3353,6 @@
       <c r="H42" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="I42" t="s">
-        <v>110</v>
-      </c>
     </row>
     <row r="43" spans="1:9">
       <c r="A43" t="s">
@@ -3481,9 +3379,6 @@
       <c r="H43" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="I43" t="s">
-        <v>111</v>
-      </c>
     </row>
     <row r="44" spans="1:9">
       <c r="A44" t="s">
@@ -3510,9 +3405,6 @@
       <c r="H44" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="I44" t="s">
-        <v>112</v>
-      </c>
     </row>
     <row r="45" spans="1:9">
       <c r="A45" t="s">
@@ -3539,9 +3431,6 @@
       <c r="H45" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="I45" t="s">
-        <v>113</v>
-      </c>
     </row>
     <row r="46" spans="1:9">
       <c r="A46" t="s">
@@ -3568,9 +3457,6 @@
       <c r="H46" s="2" t="s">
         <v>427</v>
       </c>
-      <c r="I46" t="s">
-        <v>114</v>
-      </c>
     </row>
     <row r="47" spans="1:9">
       <c r="A47" t="s">
@@ -3597,9 +3483,6 @@
       <c r="H47" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="I47" t="s">
-        <v>115</v>
-      </c>
     </row>
     <row r="48" spans="1:9">
       <c r="A48" t="s">
@@ -3626,11 +3509,8 @@
       <c r="H48" s="2" t="s">
         <v>429</v>
       </c>
-      <c r="I48" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9">
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49" t="s">
         <v>21</v>
       </c>
@@ -3655,11 +3535,8 @@
       <c r="H49" s="2" t="s">
         <v>430</v>
       </c>
-      <c r="I49" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9">
+    </row>
+    <row r="50" spans="1:8">
       <c r="A50" t="s">
         <v>21</v>
       </c>
@@ -3684,11 +3561,8 @@
       <c r="H50" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="I50" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9">
+    </row>
+    <row r="51" spans="1:8">
       <c r="A51" t="s">
         <v>21</v>
       </c>
@@ -3713,11 +3587,8 @@
       <c r="H51" s="2" t="s">
         <v>432</v>
       </c>
-      <c r="I51" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9">
+    </row>
+    <row r="52" spans="1:8">
       <c r="A52" t="s">
         <v>21</v>
       </c>
@@ -3742,11 +3613,8 @@
       <c r="H52" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="I52" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9">
+    </row>
+    <row r="53" spans="1:8">
       <c r="A53" t="s">
         <v>22</v>
       </c>
@@ -3771,11 +3639,8 @@
       <c r="H53" s="2" t="s">
         <v>434</v>
       </c>
-      <c r="I53" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9">
+    </row>
+    <row r="54" spans="1:8">
       <c r="A54" t="s">
         <v>22</v>
       </c>
@@ -3800,11 +3665,8 @@
       <c r="H54" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="I54" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9">
+    </row>
+    <row r="55" spans="1:8">
       <c r="A55" t="s">
         <v>22</v>
       </c>
@@ -3829,11 +3691,8 @@
       <c r="H55" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="I55" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9">
+    </row>
+    <row r="56" spans="1:8">
       <c r="A56" t="s">
         <v>22</v>
       </c>
@@ -3858,11 +3717,8 @@
       <c r="H56" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="I56" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9">
+    </row>
+    <row r="57" spans="1:8">
       <c r="A57" t="s">
         <v>22</v>
       </c>
@@ -3887,11 +3743,8 @@
       <c r="H57" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="I57" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9">
+    </row>
+    <row r="58" spans="1:8">
       <c r="A58" t="s">
         <v>23</v>
       </c>
@@ -3916,11 +3769,8 @@
       <c r="H58" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="I58" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9">
+    </row>
+    <row r="59" spans="1:8">
       <c r="A59" t="s">
         <v>23</v>
       </c>
@@ -3945,11 +3795,8 @@
       <c r="H59" s="2" t="s">
         <v>440</v>
       </c>
-      <c r="I59" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9">
+    </row>
+    <row r="60" spans="1:8">
       <c r="A60" t="s">
         <v>23</v>
       </c>
@@ -3974,11 +3821,8 @@
       <c r="H60" s="2" t="s">
         <v>441</v>
       </c>
-      <c r="I60" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9">
+    </row>
+    <row r="61" spans="1:8">
       <c r="A61" t="s">
         <v>23</v>
       </c>
@@ -4003,11 +3847,8 @@
       <c r="H61" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="I61" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9">
+    </row>
+    <row r="62" spans="1:8">
       <c r="A62" t="s">
         <v>24</v>
       </c>
@@ -4032,11 +3873,8 @@
       <c r="H62" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="I62" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9">
+    </row>
+    <row r="63" spans="1:8">
       <c r="A63" t="s">
         <v>24</v>
       </c>
@@ -4061,11 +3899,8 @@
       <c r="H63" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="I63" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9">
+    </row>
+    <row r="64" spans="1:8">
       <c r="A64" t="s">
         <v>24</v>
       </c>
@@ -4089,9 +3924,6 @@
       </c>
       <c r="H64" s="2" t="s">
         <v>445</v>
-      </c>
-      <c r="I64" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -4119,9 +3951,6 @@
       <c r="H65" s="2" t="s">
         <v>446</v>
       </c>
-      <c r="I65" t="s">
-        <v>131</v>
-      </c>
     </row>
     <row r="66" spans="1:9">
       <c r="A66" t="s">
@@ -4174,9 +4003,6 @@
       <c r="H67" s="2" t="s">
         <v>448</v>
       </c>
-      <c r="I67" t="s">
-        <v>133</v>
-      </c>
     </row>
     <row r="68" spans="1:9">
       <c r="A68" t="s">
@@ -4203,9 +4029,6 @@
       <c r="H68" s="2" t="s">
         <v>449</v>
       </c>
-      <c r="I68" t="s">
-        <v>134</v>
-      </c>
     </row>
     <row r="69" spans="1:9">
       <c r="A69" t="s">
@@ -4232,9 +4055,6 @@
       <c r="H69" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="I69" t="s">
-        <v>135</v>
-      </c>
     </row>
     <row r="70" spans="1:9">
       <c r="A70" t="s">
@@ -4261,9 +4081,6 @@
       <c r="H70" s="2" t="s">
         <v>451</v>
       </c>
-      <c r="I70" t="s">
-        <v>136</v>
-      </c>
     </row>
     <row r="71" spans="1:9">
       <c r="A71" t="s">
@@ -4290,9 +4107,6 @@
       <c r="H71" s="2" t="s">
         <v>452</v>
       </c>
-      <c r="I71" t="s">
-        <v>137</v>
-      </c>
     </row>
     <row r="72" spans="1:9">
       <c r="A72" t="s">
@@ -4319,9 +4133,6 @@
       <c r="H72" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="I72" t="s">
-        <v>138</v>
-      </c>
     </row>
     <row r="73" spans="1:9">
       <c r="A73" t="s">
@@ -4348,9 +4159,6 @@
       <c r="H73" s="2" t="s">
         <v>454</v>
       </c>
-      <c r="I73" t="s">
-        <v>139</v>
-      </c>
     </row>
     <row r="74" spans="1:9">
       <c r="A74" t="s">
@@ -4377,9 +4185,6 @@
       <c r="H74" s="2" t="s">
         <v>455</v>
       </c>
-      <c r="I74" t="s">
-        <v>140</v>
-      </c>
     </row>
     <row r="75" spans="1:9">
       <c r="A75" t="s">
@@ -4406,9 +4211,6 @@
       <c r="H75" s="2" t="s">
         <v>456</v>
       </c>
-      <c r="I75" t="s">
-        <v>141</v>
-      </c>
     </row>
     <row r="76" spans="1:9">
       <c r="A76" t="s">
@@ -4435,9 +4237,6 @@
       <c r="H76" s="2" t="s">
         <v>457</v>
       </c>
-      <c r="I76" t="s">
-        <v>142</v>
-      </c>
     </row>
     <row r="77" spans="1:9">
       <c r="A77" t="s">
@@ -4464,9 +4263,6 @@
       <c r="H77" s="2" t="s">
         <v>458</v>
       </c>
-      <c r="I77" t="s">
-        <v>143</v>
-      </c>
     </row>
     <row r="78" spans="1:9">
       <c r="A78" t="s">
@@ -4493,9 +4289,6 @@
       <c r="H78" s="2" t="s">
         <v>459</v>
       </c>
-      <c r="I78" t="s">
-        <v>144</v>
-      </c>
     </row>
     <row r="79" spans="1:9">
       <c r="A79" t="s">
@@ -4551,11 +4344,8 @@
       <c r="H80" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="I80" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="81" spans="1:9">
+    </row>
+    <row r="81" spans="1:8">
       <c r="A81" t="s">
         <v>30</v>
       </c>
@@ -4580,11 +4370,8 @@
       <c r="H81" s="2" t="s">
         <v>462</v>
       </c>
-      <c r="I81" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="82" spans="1:9">
+    </row>
+    <row r="82" spans="1:8">
       <c r="A82" t="s">
         <v>30</v>
       </c>
@@ -4609,11 +4396,8 @@
       <c r="H82" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="I82" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="83" spans="1:9">
+    </row>
+    <row r="83" spans="1:8">
       <c r="A83" t="s">
         <v>31</v>
       </c>
@@ -4639,7 +4423,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="84" spans="1:9">
+    <row r="84" spans="1:8">
       <c r="A84" t="s">
         <v>31</v>
       </c>
@@ -4664,11 +4448,8 @@
       <c r="H84" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="I84" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="85" spans="1:9">
+    </row>
+    <row r="85" spans="1:8">
       <c r="A85" t="s">
         <v>31</v>
       </c>
@@ -4693,11 +4474,8 @@
       <c r="H85" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="I85" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="86" spans="1:9">
+    </row>
+    <row r="86" spans="1:8">
       <c r="A86" t="s">
         <v>31</v>
       </c>
@@ -4722,11 +4500,8 @@
       <c r="H86" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="I86" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="87" spans="1:9">
+    </row>
+    <row r="87" spans="1:8">
       <c r="A87" t="s">
         <v>31</v>
       </c>
@@ -4751,11 +4526,8 @@
       <c r="H87" s="2" t="s">
         <v>468</v>
       </c>
-      <c r="I87" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="88" spans="1:9">
+    </row>
+    <row r="88" spans="1:8">
       <c r="A88" t="s">
         <v>31</v>
       </c>
@@ -4780,11 +4552,8 @@
       <c r="H88" s="2" t="s">
         <v>469</v>
       </c>
-      <c r="I88" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="89" spans="1:9">
+    </row>
+    <row r="89" spans="1:8">
       <c r="A89" t="s">
         <v>32</v>
       </c>
@@ -4809,11 +4578,8 @@
       <c r="H89" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="I89" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="90" spans="1:9">
+    </row>
+    <row r="90" spans="1:8">
       <c r="A90" t="s">
         <v>32</v>
       </c>
@@ -4838,11 +4604,8 @@
       <c r="H90" s="2" t="s">
         <v>471</v>
       </c>
-      <c r="I90" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="91" spans="1:9">
+    </row>
+    <row r="91" spans="1:8">
       <c r="A91" t="s">
         <v>32</v>
       </c>
@@ -4867,11 +4630,8 @@
       <c r="H91" s="2" t="s">
         <v>472</v>
       </c>
-      <c r="I91" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="92" spans="1:9">
+    </row>
+    <row r="92" spans="1:8">
       <c r="A92" t="s">
         <v>32</v>
       </c>
@@ -4897,7 +4657,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="93" spans="1:9">
+    <row r="93" spans="1:8">
       <c r="A93" t="s">
         <v>32</v>
       </c>
@@ -4922,11 +4682,8 @@
       <c r="H93" s="2" t="s">
         <v>474</v>
       </c>
-      <c r="I93" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="94" spans="1:9">
+    </row>
+    <row r="94" spans="1:8">
       <c r="A94" t="s">
         <v>32</v>
       </c>
@@ -4952,7 +4709,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="95" spans="1:9">
+    <row r="95" spans="1:8">
       <c r="A95" t="s">
         <v>32</v>
       </c>
@@ -4977,11 +4734,8 @@
       <c r="H95" s="2" t="s">
         <v>476</v>
       </c>
-      <c r="I95" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="96" spans="1:9">
+    </row>
+    <row r="96" spans="1:8">
       <c r="A96" t="s">
         <v>33</v>
       </c>
@@ -5006,11 +4760,8 @@
       <c r="H96" s="2" t="s">
         <v>477</v>
       </c>
-      <c r="I96" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="97" spans="1:9">
+    </row>
+    <row r="97" spans="1:8">
       <c r="A97" t="s">
         <v>33</v>
       </c>
@@ -5036,7 +4787,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="98" spans="1:9">
+    <row r="98" spans="1:8">
       <c r="A98" t="s">
         <v>33</v>
       </c>
@@ -5061,11 +4812,8 @@
       <c r="H98" s="2" t="s">
         <v>479</v>
       </c>
-      <c r="I98" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="99" spans="1:9">
+    </row>
+    <row r="99" spans="1:8">
       <c r="A99" t="s">
         <v>34</v>
       </c>
@@ -5090,11 +4838,8 @@
       <c r="H99" s="2" t="s">
         <v>480</v>
       </c>
-      <c r="I99" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="100" spans="1:9">
+    </row>
+    <row r="100" spans="1:8">
       <c r="A100" t="s">
         <v>34</v>
       </c>
@@ -5119,11 +4864,8 @@
       <c r="H100" s="2" t="s">
         <v>481</v>
       </c>
-      <c r="I100" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="101" spans="1:9">
+    </row>
+    <row r="101" spans="1:8">
       <c r="A101" t="s">
         <v>34</v>
       </c>
@@ -5149,7 +4891,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="102" spans="1:9">
+    <row r="102" spans="1:8">
       <c r="A102" t="s">
         <v>35</v>
       </c>
@@ -5174,11 +4916,8 @@
       <c r="H102" s="2" t="s">
         <v>483</v>
       </c>
-      <c r="I102" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="103" spans="1:9">
+    </row>
+    <row r="103" spans="1:8">
       <c r="A103" t="s">
         <v>35</v>
       </c>
@@ -5203,11 +4942,8 @@
       <c r="H103" s="2" t="s">
         <v>484</v>
       </c>
-      <c r="I103" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="104" spans="1:9">
+    </row>
+    <row r="104" spans="1:8">
       <c r="A104" t="s">
         <v>35</v>
       </c>
@@ -5232,11 +4968,8 @@
       <c r="H104" s="2" t="s">
         <v>485</v>
       </c>
-      <c r="I104" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="105" spans="1:9">
+    </row>
+    <row r="105" spans="1:8">
       <c r="A105" t="s">
         <v>35</v>
       </c>
@@ -5261,11 +4994,8 @@
       <c r="H105" s="2" t="s">
         <v>486</v>
       </c>
-      <c r="I105" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="106" spans="1:9">
+    </row>
+    <row r="106" spans="1:8">
       <c r="A106" t="s">
         <v>36</v>
       </c>
@@ -5290,11 +5020,8 @@
       <c r="H106" s="2" t="s">
         <v>487</v>
       </c>
-      <c r="I106" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="107" spans="1:9">
+    </row>
+    <row r="107" spans="1:8">
       <c r="A107" t="s">
         <v>36</v>
       </c>
@@ -5319,11 +5046,8 @@
       <c r="H107" s="2" t="s">
         <v>488</v>
       </c>
-      <c r="I107" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="108" spans="1:9">
+    </row>
+    <row r="108" spans="1:8">
       <c r="A108" t="s">
         <v>36</v>
       </c>
@@ -5348,11 +5072,8 @@
       <c r="H108" s="2" t="s">
         <v>489</v>
       </c>
-      <c r="I108" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="109" spans="1:9">
+    </row>
+    <row r="109" spans="1:8">
       <c r="A109" t="s">
         <v>36</v>
       </c>
@@ -5377,11 +5098,8 @@
       <c r="H109" s="2" t="s">
         <v>490</v>
       </c>
-      <c r="I109" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="110" spans="1:9">
+    </row>
+    <row r="110" spans="1:8">
       <c r="A110" t="s">
         <v>36</v>
       </c>
@@ -5406,11 +5124,8 @@
       <c r="H110" s="2" t="s">
         <v>491</v>
       </c>
-      <c r="I110" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="111" spans="1:9">
+    </row>
+    <row r="111" spans="1:8">
       <c r="A111" t="s">
         <v>36</v>
       </c>
@@ -5435,11 +5150,8 @@
       <c r="H111" s="2" t="s">
         <v>492</v>
       </c>
-      <c r="I111" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="112" spans="1:9">
+    </row>
+    <row r="112" spans="1:8">
       <c r="A112" t="s">
         <v>36</v>
       </c>
@@ -5464,11 +5176,8 @@
       <c r="H112" s="2" t="s">
         <v>493</v>
       </c>
-      <c r="I112" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="113" spans="1:9">
+    </row>
+    <row r="113" spans="1:8">
       <c r="A113" t="s">
         <v>36</v>
       </c>
@@ -5494,7 +5203,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="114" spans="1:9">
+    <row r="114" spans="1:8">
       <c r="A114" t="s">
         <v>37</v>
       </c>
@@ -5519,11 +5228,8 @@
       <c r="H114" s="2" t="s">
         <v>495</v>
       </c>
-      <c r="I114" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="115" spans="1:9">
+    </row>
+    <row r="115" spans="1:8">
       <c r="A115" t="s">
         <v>37</v>
       </c>
@@ -5548,11 +5254,8 @@
       <c r="H115" s="2" t="s">
         <v>496</v>
       </c>
-      <c r="I115" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="116" spans="1:9">
+    </row>
+    <row r="116" spans="1:8">
       <c r="A116" t="s">
         <v>37</v>
       </c>
@@ -5578,7 +5281,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="117" spans="1:9">
+    <row r="117" spans="1:8">
       <c r="A117" t="s">
         <v>37</v>
       </c>
@@ -5603,11 +5306,8 @@
       <c r="H117" s="2" t="s">
         <v>498</v>
       </c>
-      <c r="I117" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="118" spans="1:9">
+    </row>
+    <row r="118" spans="1:8">
       <c r="A118" t="s">
         <v>37</v>
       </c>
@@ -5632,11 +5332,8 @@
       <c r="H118" s="2" t="s">
         <v>499</v>
       </c>
-      <c r="I118" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="119" spans="1:9">
+    </row>
+    <row r="119" spans="1:8">
       <c r="A119" t="s">
         <v>37</v>
       </c>
@@ -5661,11 +5358,8 @@
       <c r="H119" s="2" t="s">
         <v>500</v>
       </c>
-      <c r="I119" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="120" spans="1:9">
+    </row>
+    <row r="120" spans="1:8">
       <c r="A120" t="s">
         <v>37</v>
       </c>
@@ -5690,11 +5384,8 @@
       <c r="H120" s="2" t="s">
         <v>501</v>
       </c>
-      <c r="I120" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="121" spans="1:9">
+    </row>
+    <row r="121" spans="1:8">
       <c r="A121" t="s">
         <v>37</v>
       </c>
@@ -5719,11 +5410,8 @@
       <c r="H121" s="2" t="s">
         <v>502</v>
       </c>
-      <c r="I121" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="122" spans="1:9">
+    </row>
+    <row r="122" spans="1:8">
       <c r="A122" t="s">
         <v>37</v>
       </c>
@@ -5748,11 +5436,8 @@
       <c r="H122" s="2" t="s">
         <v>503</v>
       </c>
-      <c r="I122" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="123" spans="1:9">
+    </row>
+    <row r="123" spans="1:8">
       <c r="A123" t="s">
         <v>38</v>
       </c>
@@ -5777,11 +5462,8 @@
       <c r="H123" s="2" t="s">
         <v>504</v>
       </c>
-      <c r="I123" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="124" spans="1:9">
+    </row>
+    <row r="124" spans="1:8">
       <c r="A124" t="s">
         <v>39</v>
       </c>
@@ -5807,7 +5489,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="125" spans="1:9">
+    <row r="125" spans="1:8">
       <c r="A125" t="s">
         <v>40</v>
       </c>
@@ -5832,11 +5514,8 @@
       <c r="H125" s="2" t="s">
         <v>506</v>
       </c>
-      <c r="I125" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="126" spans="1:9">
+    </row>
+    <row r="126" spans="1:8">
       <c r="A126" t="s">
         <v>40</v>
       </c>
@@ -5862,7 +5541,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="127" spans="1:9">
+    <row r="127" spans="1:8">
       <c r="A127" t="s">
         <v>41</v>
       </c>
@@ -5887,11 +5566,8 @@
       <c r="H127" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="I127" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="128" spans="1:9">
+    </row>
+    <row r="128" spans="1:8">
       <c r="A128" t="s">
         <v>41</v>
       </c>
@@ -5915,9 +5591,6 @@
       </c>
       <c r="H128" s="2" t="s">
         <v>509</v>
-      </c>
-      <c r="I128" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="129" spans="1:9">
@@ -5945,9 +5618,6 @@
       <c r="H129" s="2" t="s">
         <v>510</v>
       </c>
-      <c r="I129" t="s">
-        <v>194</v>
-      </c>
     </row>
     <row r="130" spans="1:9">
       <c r="A130" t="s">
@@ -5974,9 +5644,6 @@
       <c r="H130" s="2" t="s">
         <v>511</v>
       </c>
-      <c r="I130" t="s">
-        <v>195</v>
-      </c>
     </row>
     <row r="131" spans="1:9">
       <c r="A131" t="s">
@@ -6003,9 +5670,6 @@
       <c r="H131" s="2" t="s">
         <v>512</v>
       </c>
-      <c r="I131" t="s">
-        <v>196</v>
-      </c>
     </row>
     <row r="132" spans="1:9">
       <c r="A132" t="s">
@@ -6032,9 +5696,6 @@
       <c r="H132" s="2" t="s">
         <v>513</v>
       </c>
-      <c r="I132" t="s">
-        <v>197</v>
-      </c>
     </row>
     <row r="133" spans="1:9">
       <c r="A133" t="s">
@@ -6119,9 +5780,6 @@
       <c r="H135" s="2" t="s">
         <v>516</v>
       </c>
-      <c r="I135" t="s">
-        <v>200</v>
-      </c>
     </row>
     <row r="136" spans="1:9">
       <c r="A136" t="s">
@@ -6148,9 +5806,6 @@
       <c r="H136" s="2" t="s">
         <v>517</v>
       </c>
-      <c r="I136" t="s">
-        <v>201</v>
-      </c>
     </row>
     <row r="137" spans="1:9">
       <c r="A137" t="s">
@@ -6278,9 +5933,6 @@
       <c r="H141" s="2" t="s">
         <v>521</v>
       </c>
-      <c r="I141" t="s">
-        <v>206</v>
-      </c>
     </row>
     <row r="142" spans="1:9">
       <c r="A142" t="s">
@@ -6307,9 +5959,6 @@
       <c r="H142" s="2" t="s">
         <v>522</v>
       </c>
-      <c r="I142" t="s">
-        <v>207</v>
-      </c>
     </row>
     <row r="143" spans="1:9">
       <c r="A143" t="s">
@@ -6336,9 +5985,6 @@
       <c r="H143" s="2" t="s">
         <v>523</v>
       </c>
-      <c r="I143" t="s">
-        <v>208</v>
-      </c>
     </row>
     <row r="144" spans="1:9">
       <c r="A144" t="s">
@@ -6365,11 +6011,8 @@
       <c r="H144" s="2" t="s">
         <v>524</v>
       </c>
-      <c r="I144" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="145" spans="1:9">
+    </row>
+    <row r="145" spans="1:8">
       <c r="A145" t="s">
         <v>43</v>
       </c>
@@ -6394,11 +6037,8 @@
       <c r="H145" s="2" t="s">
         <v>525</v>
       </c>
-      <c r="I145" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="146" spans="1:9">
+    </row>
+    <row r="146" spans="1:8">
       <c r="A146" t="s">
         <v>43</v>
       </c>
@@ -6423,11 +6063,8 @@
       <c r="H146" s="2" t="s">
         <v>526</v>
       </c>
-      <c r="I146" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="147" spans="1:9">
+    </row>
+    <row r="147" spans="1:8">
       <c r="A147" t="s">
         <v>43</v>
       </c>
@@ -6452,11 +6089,8 @@
       <c r="H147" s="2" t="s">
         <v>527</v>
       </c>
-      <c r="I147" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="148" spans="1:9">
+    </row>
+    <row r="148" spans="1:8">
       <c r="A148" t="s">
         <v>44</v>
       </c>
@@ -6481,11 +6115,8 @@
       <c r="H148" s="2" t="s">
         <v>528</v>
       </c>
-      <c r="I148" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="149" spans="1:9">
+    </row>
+    <row r="149" spans="1:8">
       <c r="A149" t="s">
         <v>44</v>
       </c>
@@ -6510,11 +6141,8 @@
       <c r="H149" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="I149" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="150" spans="1:9">
+    </row>
+    <row r="150" spans="1:8">
       <c r="A150" t="s">
         <v>44</v>
       </c>
@@ -6539,11 +6167,8 @@
       <c r="H150" s="2" t="s">
         <v>530</v>
       </c>
-      <c r="I150" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="151" spans="1:9">
+    </row>
+    <row r="151" spans="1:8">
       <c r="A151" t="s">
         <v>44</v>
       </c>
@@ -6568,11 +6193,8 @@
       <c r="H151" s="2" t="s">
         <v>531</v>
       </c>
-      <c r="I151" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="152" spans="1:9">
+    </row>
+    <row r="152" spans="1:8">
       <c r="A152" t="s">
         <v>44</v>
       </c>
@@ -6597,11 +6219,8 @@
       <c r="H152" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="I152" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="153" spans="1:9">
+    </row>
+    <row r="153" spans="1:8">
       <c r="A153" t="s">
         <v>44</v>
       </c>
@@ -6626,11 +6245,8 @@
       <c r="H153" s="2" t="s">
         <v>533</v>
       </c>
-      <c r="I153" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="154" spans="1:9">
+    </row>
+    <row r="154" spans="1:8">
       <c r="A154" t="s">
         <v>44</v>
       </c>
@@ -6655,11 +6271,8 @@
       <c r="H154" s="2" t="s">
         <v>534</v>
       </c>
-      <c r="I154" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="155" spans="1:9">
+    </row>
+    <row r="155" spans="1:8">
       <c r="A155" t="s">
         <v>44</v>
       </c>
@@ -6684,11 +6297,8 @@
       <c r="H155" s="2" t="s">
         <v>535</v>
       </c>
-      <c r="I155" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="156" spans="1:9">
+    </row>
+    <row r="156" spans="1:8">
       <c r="A156" t="s">
         <v>44</v>
       </c>
@@ -6714,7 +6324,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="157" spans="1:9">
+    <row r="157" spans="1:8">
       <c r="A157" t="s">
         <v>44</v>
       </c>
@@ -6740,7 +6350,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="158" spans="1:9">
+    <row r="158" spans="1:8">
       <c r="A158" t="s">
         <v>44</v>
       </c>
@@ -6765,11 +6375,8 @@
       <c r="H158" s="2" t="s">
         <v>538</v>
       </c>
-      <c r="I158" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="159" spans="1:9">
+    </row>
+    <row r="159" spans="1:8">
       <c r="A159" t="s">
         <v>45</v>
       </c>
@@ -6795,7 +6402,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="160" spans="1:9">
+    <row r="160" spans="1:8">
       <c r="A160" t="s">
         <v>45</v>
       </c>
@@ -6819,9 +6426,6 @@
       </c>
       <c r="H160" s="2" t="s">
         <v>540</v>
-      </c>
-      <c r="I160" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="161" spans="1:9">
@@ -6875,9 +6479,6 @@
       <c r="H162" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="I162" t="s">
-        <v>227</v>
-      </c>
     </row>
     <row r="163" spans="1:9">
       <c r="A163" t="s">
@@ -6959,9 +6560,6 @@
       <c r="H165" s="2" t="s">
         <v>545</v>
       </c>
-      <c r="I165" t="s">
-        <v>230</v>
-      </c>
     </row>
     <row r="166" spans="1:9">
       <c r="A166" t="s">
@@ -6988,9 +6586,6 @@
       <c r="H166" s="2" t="s">
         <v>546</v>
       </c>
-      <c r="I166" t="s">
-        <v>231</v>
-      </c>
     </row>
     <row r="167" spans="1:9">
       <c r="A167" t="s">
@@ -7043,9 +6638,6 @@
       <c r="H168" s="2" t="s">
         <v>548</v>
       </c>
-      <c r="I168" t="s">
-        <v>233</v>
-      </c>
     </row>
     <row r="169" spans="1:9">
       <c r="A169" t="s">
@@ -7072,9 +6664,6 @@
       <c r="H169" s="2" t="s">
         <v>549</v>
       </c>
-      <c r="I169" t="s">
-        <v>234</v>
-      </c>
     </row>
     <row r="170" spans="1:9">
       <c r="A170" t="s">
@@ -7101,9 +6690,6 @@
       <c r="H170" s="2" t="s">
         <v>550</v>
       </c>
-      <c r="I170" t="s">
-        <v>235</v>
-      </c>
     </row>
     <row r="171" spans="1:9">
       <c r="A171" t="s">
@@ -7130,9 +6716,6 @@
       <c r="H171" s="2" t="s">
         <v>551</v>
       </c>
-      <c r="I171" t="s">
-        <v>236</v>
-      </c>
     </row>
     <row r="172" spans="1:9">
       <c r="A172" t="s">
@@ -7159,9 +6742,6 @@
       <c r="H172" s="2" t="s">
         <v>552</v>
       </c>
-      <c r="I172" t="s">
-        <v>237</v>
-      </c>
     </row>
     <row r="173" spans="1:9">
       <c r="A173" t="s">
@@ -7188,9 +6768,6 @@
       <c r="H173" s="2" t="s">
         <v>553</v>
       </c>
-      <c r="I173" t="s">
-        <v>238</v>
-      </c>
     </row>
     <row r="174" spans="1:9">
       <c r="A174" t="s">
@@ -7217,9 +6794,6 @@
       <c r="H174" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="I174" t="s">
-        <v>239</v>
-      </c>
     </row>
     <row r="175" spans="1:9">
       <c r="A175" t="s">
@@ -7246,9 +6820,6 @@
       <c r="H175" s="2" t="s">
         <v>555</v>
       </c>
-      <c r="I175" t="s">
-        <v>240</v>
-      </c>
     </row>
     <row r="176" spans="1:9">
       <c r="A176" t="s">
@@ -7275,11 +6846,8 @@
       <c r="H176" s="2" t="s">
         <v>556</v>
       </c>
-      <c r="I176" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="177" spans="1:9">
+    </row>
+    <row r="177" spans="1:8">
       <c r="A177" t="s">
         <v>54</v>
       </c>
@@ -7304,11 +6872,8 @@
       <c r="H177" s="2" t="s">
         <v>557</v>
       </c>
-      <c r="I177" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="178" spans="1:9">
+    </row>
+    <row r="178" spans="1:8">
       <c r="A178" t="s">
         <v>54</v>
       </c>
@@ -7333,11 +6898,8 @@
       <c r="H178" s="2" t="s">
         <v>558</v>
       </c>
-      <c r="I178" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="179" spans="1:9">
+    </row>
+    <row r="179" spans="1:8">
       <c r="A179" t="s">
         <v>54</v>
       </c>
@@ -7362,11 +6924,8 @@
       <c r="H179" s="2" t="s">
         <v>559</v>
       </c>
-      <c r="I179" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="180" spans="1:9">
+    </row>
+    <row r="180" spans="1:8">
       <c r="A180" t="s">
         <v>55</v>
       </c>
@@ -7391,11 +6950,8 @@
       <c r="H180" s="2" t="s">
         <v>560</v>
       </c>
-      <c r="I180" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="181" spans="1:9">
+    </row>
+    <row r="181" spans="1:8">
       <c r="A181" t="s">
         <v>55</v>
       </c>
@@ -7420,11 +6976,8 @@
       <c r="H181" s="2" t="s">
         <v>561</v>
       </c>
-      <c r="I181" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="182" spans="1:9">
+    </row>
+    <row r="182" spans="1:8">
       <c r="A182" t="s">
         <v>55</v>
       </c>
@@ -7449,11 +7002,8 @@
       <c r="H182" s="2" t="s">
         <v>562</v>
       </c>
-      <c r="I182" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="183" spans="1:9">
+    </row>
+    <row r="183" spans="1:8">
       <c r="A183" t="s">
         <v>55</v>
       </c>
@@ -7478,11 +7028,8 @@
       <c r="H183" s="2" t="s">
         <v>563</v>
       </c>
-      <c r="I183" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="184" spans="1:9">
+    </row>
+    <row r="184" spans="1:8">
       <c r="A184" t="s">
         <v>55</v>
       </c>
@@ -7507,11 +7054,8 @@
       <c r="H184" s="2" t="s">
         <v>564</v>
       </c>
-      <c r="I184" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="185" spans="1:9">
+    </row>
+    <row r="185" spans="1:8">
       <c r="A185" t="s">
         <v>56</v>
       </c>
@@ -7536,11 +7080,8 @@
       <c r="H185" s="2" t="s">
         <v>565</v>
       </c>
-      <c r="I185" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="186" spans="1:9">
+    </row>
+    <row r="186" spans="1:8">
       <c r="A186" t="s">
         <v>57</v>
       </c>
@@ -7565,11 +7106,8 @@
       <c r="H186" s="2" t="s">
         <v>566</v>
       </c>
-      <c r="I186" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="187" spans="1:9">
+    </row>
+    <row r="187" spans="1:8">
       <c r="A187" t="s">
         <v>57</v>
       </c>
@@ -7594,11 +7132,8 @@
       <c r="H187" s="2" t="s">
         <v>567</v>
       </c>
-      <c r="I187" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="188" spans="1:9">
+    </row>
+    <row r="188" spans="1:8">
       <c r="A188" t="s">
         <v>58</v>
       </c>
@@ -7623,11 +7158,8 @@
       <c r="H188" s="2" t="s">
         <v>568</v>
       </c>
-      <c r="I188" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="189" spans="1:9">
+    </row>
+    <row r="189" spans="1:8">
       <c r="A189" t="s">
         <v>58</v>
       </c>
@@ -7652,11 +7184,8 @@
       <c r="H189" s="2" t="s">
         <v>569</v>
       </c>
-      <c r="I189" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="190" spans="1:9">
+    </row>
+    <row r="190" spans="1:8">
       <c r="A190" t="s">
         <v>59</v>
       </c>
@@ -7681,11 +7210,8 @@
       <c r="H190" s="2" t="s">
         <v>570</v>
       </c>
-      <c r="I190" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="191" spans="1:9">
+    </row>
+    <row r="191" spans="1:8">
       <c r="A191" t="s">
         <v>59</v>
       </c>
@@ -7710,11 +7236,8 @@
       <c r="H191" s="2" t="s">
         <v>571</v>
       </c>
-      <c r="I191" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="192" spans="1:9">
+    </row>
+    <row r="192" spans="1:8">
       <c r="A192" t="s">
         <v>60</v>
       </c>
@@ -7739,11 +7262,8 @@
       <c r="H192" s="2" t="s">
         <v>572</v>
       </c>
-      <c r="I192" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="193" spans="1:9">
+    </row>
+    <row r="193" spans="1:8">
       <c r="A193" t="s">
         <v>61</v>
       </c>
@@ -7768,11 +7288,8 @@
       <c r="H193" s="2" t="s">
         <v>573</v>
       </c>
-      <c r="I193" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="194" spans="1:9">
+    </row>
+    <row r="194" spans="1:8">
       <c r="A194" t="s">
         <v>61</v>
       </c>
@@ -7797,11 +7314,8 @@
       <c r="H194" s="2" t="s">
         <v>574</v>
       </c>
-      <c r="I194" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="195" spans="1:9">
+    </row>
+    <row r="195" spans="1:8">
       <c r="A195" t="s">
         <v>62</v>
       </c>
@@ -7826,11 +7340,8 @@
       <c r="H195" s="2" t="s">
         <v>575</v>
       </c>
-      <c r="I195" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="196" spans="1:9">
+    </row>
+    <row r="196" spans="1:8">
       <c r="A196" t="s">
         <v>63</v>
       </c>
@@ -7855,11 +7366,8 @@
       <c r="H196" s="2" t="s">
         <v>576</v>
       </c>
-      <c r="I196" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="197" spans="1:9">
+    </row>
+    <row r="197" spans="1:8">
       <c r="A197" t="s">
         <v>64</v>
       </c>
@@ -7884,11 +7392,8 @@
       <c r="H197" s="2" t="s">
         <v>577</v>
       </c>
-      <c r="I197" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="198" spans="1:9">
+    </row>
+    <row r="198" spans="1:8">
       <c r="A198" t="s">
         <v>64</v>
       </c>
@@ -7913,11 +7418,8 @@
       <c r="H198" s="2" t="s">
         <v>578</v>
       </c>
-      <c r="I198" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="199" spans="1:9">
+    </row>
+    <row r="199" spans="1:8">
       <c r="A199" t="s">
         <v>65</v>
       </c>
@@ -7942,11 +7444,8 @@
       <c r="H199" s="2" t="s">
         <v>579</v>
       </c>
-      <c r="I199" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="200" spans="1:9">
+    </row>
+    <row r="200" spans="1:8">
       <c r="A200" t="s">
         <v>66</v>
       </c>
@@ -7971,11 +7470,8 @@
       <c r="H200" s="2" t="s">
         <v>580</v>
       </c>
-      <c r="I200" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="201" spans="1:9">
+    </row>
+    <row r="201" spans="1:8">
       <c r="A201" t="s">
         <v>67</v>
       </c>
@@ -8000,11 +7496,8 @@
       <c r="H201" s="2" t="s">
         <v>581</v>
       </c>
-      <c r="I201" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="202" spans="1:9">
+    </row>
+    <row r="202" spans="1:8">
       <c r="A202" t="s">
         <v>67</v>
       </c>
@@ -8029,11 +7522,8 @@
       <c r="H202" s="2" t="s">
         <v>582</v>
       </c>
-      <c r="I202" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="203" spans="1:9">
+    </row>
+    <row r="203" spans="1:8">
       <c r="A203" t="s">
         <v>67</v>
       </c>
@@ -8058,11 +7548,8 @@
       <c r="H203" s="2" t="s">
         <v>583</v>
       </c>
-      <c r="I203" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="204" spans="1:9">
+    </row>
+    <row r="204" spans="1:8">
       <c r="A204" t="s">
         <v>67</v>
       </c>
@@ -8087,11 +7574,8 @@
       <c r="H204" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="I204" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="205" spans="1:9">
+    </row>
+    <row r="205" spans="1:8">
       <c r="A205" t="s">
         <v>67</v>
       </c>
@@ -8116,11 +7600,8 @@
       <c r="H205" s="2" t="s">
         <v>585</v>
       </c>
-      <c r="I205" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="206" spans="1:9">
+    </row>
+    <row r="206" spans="1:8">
       <c r="A206" t="s">
         <v>67</v>
       </c>
@@ -8145,11 +7626,8 @@
       <c r="H206" s="2" t="s">
         <v>586</v>
       </c>
-      <c r="I206" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="207" spans="1:9">
+    </row>
+    <row r="207" spans="1:8">
       <c r="A207" t="s">
         <v>68</v>
       </c>
@@ -8174,11 +7652,8 @@
       <c r="H207" s="2" t="s">
         <v>587</v>
       </c>
-      <c r="I207" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="208" spans="1:9">
+    </row>
+    <row r="208" spans="1:8">
       <c r="A208" t="s">
         <v>68</v>
       </c>
@@ -8203,11 +7678,8 @@
       <c r="H208" s="2" t="s">
         <v>588</v>
       </c>
-      <c r="I208" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="209" spans="1:9">
+    </row>
+    <row r="209" spans="1:8">
       <c r="A209" t="s">
         <v>68</v>
       </c>
@@ -8232,11 +7704,8 @@
       <c r="H209" s="2" t="s">
         <v>589</v>
       </c>
-      <c r="I209" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="210" spans="1:9">
+    </row>
+    <row r="210" spans="1:8">
       <c r="A210" t="s">
         <v>68</v>
       </c>
@@ -8261,11 +7730,8 @@
       <c r="H210" s="2" t="s">
         <v>590</v>
       </c>
-      <c r="I210" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="211" spans="1:9">
+    </row>
+    <row r="211" spans="1:8">
       <c r="A211" t="s">
         <v>68</v>
       </c>
@@ -8290,11 +7756,8 @@
       <c r="H211" s="2" t="s">
         <v>591</v>
       </c>
-      <c r="I211" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="212" spans="1:9">
+    </row>
+    <row r="212" spans="1:8">
       <c r="A212" t="s">
         <v>68</v>
       </c>
@@ -8319,11 +7782,8 @@
       <c r="H212" s="2" t="s">
         <v>592</v>
       </c>
-      <c r="I212" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="213" spans="1:9">
+    </row>
+    <row r="213" spans="1:8">
       <c r="A213" t="s">
         <v>68</v>
       </c>
@@ -8348,11 +7808,8 @@
       <c r="H213" s="2" t="s">
         <v>593</v>
       </c>
-      <c r="I213" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="214" spans="1:9">
+    </row>
+    <row r="214" spans="1:8">
       <c r="A214" t="s">
         <v>69</v>
       </c>
@@ -8377,11 +7834,8 @@
       <c r="H214" s="2" t="s">
         <v>594</v>
       </c>
-      <c r="I214" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="215" spans="1:9">
+    </row>
+    <row r="215" spans="1:8">
       <c r="A215" t="s">
         <v>69</v>
       </c>
@@ -8406,11 +7860,8 @@
       <c r="H215" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="I215" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="216" spans="1:9">
+    </row>
+    <row r="216" spans="1:8">
       <c r="A216" t="s">
         <v>69</v>
       </c>
@@ -8435,11 +7886,8 @@
       <c r="H216" s="2" t="s">
         <v>596</v>
       </c>
-      <c r="I216" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="217" spans="1:9">
+    </row>
+    <row r="217" spans="1:8">
       <c r="A217" t="s">
         <v>70</v>
       </c>
@@ -8464,11 +7912,8 @@
       <c r="H217" s="2" t="s">
         <v>597</v>
       </c>
-      <c r="I217" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="218" spans="1:9">
+    </row>
+    <row r="218" spans="1:8">
       <c r="A218" t="s">
         <v>70</v>
       </c>
@@ -8493,11 +7938,8 @@
       <c r="H218" s="2" t="s">
         <v>598</v>
       </c>
-      <c r="I218" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="219" spans="1:9">
+    </row>
+    <row r="219" spans="1:8">
       <c r="A219" t="s">
         <v>70</v>
       </c>
@@ -8522,11 +7964,8 @@
       <c r="H219" s="2" t="s">
         <v>599</v>
       </c>
-      <c r="I219" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="220" spans="1:9">
+    </row>
+    <row r="220" spans="1:8">
       <c r="A220" t="s">
         <v>71</v>
       </c>
@@ -8551,11 +7990,8 @@
       <c r="H220" s="2" t="s">
         <v>600</v>
       </c>
-      <c r="I220" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="221" spans="1:9">
+    </row>
+    <row r="221" spans="1:8">
       <c r="A221" t="s">
         <v>71</v>
       </c>
@@ -8580,11 +8016,8 @@
       <c r="H221" s="2" t="s">
         <v>601</v>
       </c>
-      <c r="I221" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="222" spans="1:9">
+    </row>
+    <row r="222" spans="1:8">
       <c r="A222" t="s">
         <v>71</v>
       </c>
@@ -8609,11 +8042,8 @@
       <c r="H222" s="2" t="s">
         <v>602</v>
       </c>
-      <c r="I222" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="223" spans="1:9">
+    </row>
+    <row r="223" spans="1:8">
       <c r="A223" t="s">
         <v>71</v>
       </c>
@@ -8638,11 +8068,8 @@
       <c r="H223" s="2" t="s">
         <v>603</v>
       </c>
-      <c r="I223" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="224" spans="1:9">
+    </row>
+    <row r="224" spans="1:8">
       <c r="A224" t="s">
         <v>71</v>
       </c>
@@ -8667,11 +8094,8 @@
       <c r="H224" s="2" t="s">
         <v>604</v>
       </c>
-      <c r="I224" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="225" spans="1:9">
+    </row>
+    <row r="225" spans="1:8">
       <c r="A225" t="s">
         <v>71</v>
       </c>
@@ -8696,11 +8120,8 @@
       <c r="H225" s="2" t="s">
         <v>605</v>
       </c>
-      <c r="I225" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="226" spans="1:9">
+    </row>
+    <row r="226" spans="1:8">
       <c r="A226" t="s">
         <v>71</v>
       </c>
@@ -8725,11 +8146,8 @@
       <c r="H226" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="I226" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="227" spans="1:9">
+    </row>
+    <row r="227" spans="1:8">
       <c r="A227" t="s">
         <v>71</v>
       </c>
@@ -8753,9 +8171,6 @@
       </c>
       <c r="H227" s="2" t="s">
         <v>607</v>
-      </c>
-      <c r="I227" t="s">
-        <v>288</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-03-12
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I92"/>
+  <dimension ref="A1:I94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -573,7 +573,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
+          <t>Estudiantes de colegios públicos en Bogotá que tendrían que reponer clase el sábado</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -588,22 +588,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
+          <t>https://www.pulzo.com/nacion/bogota/estudiantes-colegios-publicos-bogota-que-tendrian-que-reponer-clase-PP5091931A</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -611,17 +611,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
+          <t>La travesía del gigante telescopio que Rodolfo Llinás le regaló al histórico Observatorio de la Universidad Nacional</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -636,44 +636,44 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
+          <t>https://www.las2orillas.co/la-travesia-del-gigante-telescopio-que-rodolfo-llinas-le-regalo-al-historico-observatorio-de-la-universidad-nacional/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
+          <t>En medio del paro de la Nacional, el cientifico donó su telescopio personal, el más grande instalado en Colombia, ahora al servicio de estudiantes e investigadoresEl artículoLa travesía del gigante telescopio que Rodolfo Llinás le regaló al...</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
+          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -683,24 +683,20 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -710,42 +706,42 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
+          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Valledupar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
+          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
         </is>
       </c>
     </row>
@@ -757,42 +753,42 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Prosperidad Social inicia entrega de transferencia monetaria de Jóvenes en Paz</t>
+          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-inicia-entrega-de-transferencia-monetaria-de-jovenes-en-paz/</t>
+          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Esta transferencia corresponde al ciclo 1 de 2026. Más de 12.000 jóvenes en el país recibirán los recursos. Bogotá D. C., 24 de febrero de 2026. Prosperidad Social realizará este 27 de febrero la transferencia monetaria condicionada para los...</t>
+          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
         </is>
       </c>
     </row>
@@ -804,7 +800,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
+          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -819,27 +815,27 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
+          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
         </is>
       </c>
     </row>
@@ -851,42 +847,42 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
+          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
+          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
         </is>
       </c>
     </row>
@@ -898,17 +894,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
+          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -918,22 +914,22 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Valledupar</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
+          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
         </is>
       </c>
     </row>
@@ -945,42 +941,42 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
+          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
+          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
         </is>
       </c>
     </row>
@@ -992,17 +988,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
+          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1012,39 +1008,39 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
+          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
+          <t>Prosperidad Social inicia entrega de transferencia monetaria de Jóvenes en Paz</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1054,7 +1050,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1069,71 +1065,71 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-inicia-entrega-de-transferencia-monetaria-de-jovenes-en-paz/</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
+          <t>Esta transferencia corresponde al ciclo 1 de 2026. Más de 12.000 jóvenes en el país recibirán los recursos. Bogotá D. C., 24 de febrero de 2026. Prosperidad Social realizará este 27 de febrero la transferencia monetaria condicionada para los...</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
+          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
+          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
+          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
+          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1163,24 +1159,24 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
+          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
+          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1195,7 +1191,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1210,34 +1206,34 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
+          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
+          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1257,59 +1253,59 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
+          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
+          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
+          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
         </is>
       </c>
     </row>
@@ -1321,64 +1317,64 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
+          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/cultura</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
+          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
+          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1388,7 +1384,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1398,67 +1394,71 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
+          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+          <t>https://www.diarioadn.co/seccion/cultura</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Adam Mosseri, director de Instagram, desmiente la existencia de “la adicción clínica” a las redes sociales</t>
+          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1473,12 +1473,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1488,57 +1488,57 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/tecno/2026/02/12/adam-mosseri-director-de-instagram-desmiente-la-existencia-de-la-adiccion-clinica-a-las-redes-sociales/</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>El directivo admitió que ciertas funciones de la app como los filtros digitales generan riesgos sobre la imagen corporal y el bienestar de los usuarios jóvenes</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
+          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
+          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1578,10 +1578,14 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1591,12 +1595,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
+          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1611,24 +1615,20 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1681,12 +1681,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
+          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1701,20 +1701,24 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
+          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1724,7 +1728,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
+          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1754,71 +1758,63 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
+          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>Adam Mosseri, director de Instagram, desmiente la existencia de “la adicción clínica” a las redes sociales</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1833,45 +1829,49 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr"/>
+          <t>https://www.infobae.com/tecno/2026/02/12/adam-mosseri-director-de-instagram-desmiente-la-existencia-de-la-adiccion-clinica-a-las-redes-sociales/</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>El directivo admitió que ciertas funciones de la app como los filtros digitales generan riesgos sobre la imagen corporal y el bienestar de los usuarios jóvenes</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1891,20 +1891,24 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1919,7 +1923,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1934,7 +1938,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
@@ -1942,12 +1946,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1962,22 +1966,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
@@ -1985,12 +1989,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
+          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2010,17 +2014,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -2028,22 +2032,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
+          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2053,39 +2057,35 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
+          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
@@ -2123,17 +2123,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
+          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2143,20 +2143,24 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2166,12 +2170,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
+          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2181,12 +2185,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2196,29 +2200,25 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/inicio</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
+          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2228,7 +2228,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2243,20 +2243,24 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/inicio</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
+          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2271,22 +2275,22 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -2294,12 +2298,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
+          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2329,7 +2333,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -2337,12 +2341,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2357,7 +2361,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2372,7 +2376,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -2380,17 +2384,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2400,7 +2404,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2415,7 +2419,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -2423,12 +2427,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2443,22 +2447,22 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
+          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -2466,32 +2470,32 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Estados Unidos reclama a Colombia ante ONU el incremento de reclutamiento de menores de edad - El Espectador</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2501,7 +2505,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxPVFRDQXk2WVcwQVhLTmljT1B4akFGM3ozQlBvc3QyOHJua1BfT1hxRnFJY212eFowWTVTdVBmTHN6d2REcXc5VGVuUmw1LWsxNWxOeW82UzBPaVQ3azZfQVNSb0pUTHFqTHdGVWJXS2Z5YmVSbXZJSXd4dzdTamNXdUtqMTRwVDV4MF9acHJFX1pTZ19NVVNvLWdNb1Y1d0FzZlN2dWVMamlvVlNCN01ZS2MxZDh1M250d2tsNEVpc2NYRUJXcE9KYk0yd1FHU3BiNUtFOENRdWZ4ZHdsR0l2cFRFMEpKTGYtaUk4dmhuRjhyaVU3RDYxbUpCUzjSAZACQVVfeXFMTmxJSVphakhMc1dSdUhqdDJFZW00OTIwT0NRNndiZGNtLWROVW1NZFFHWHhTMzVYb3N6aHRBV1NObF94cEVSeHZMOWpPTW1oVXdGeDloRU9uSWpIUXNldU1qY2lUM3dNWnhwMUNESWVTUy1SNGYzZkM0Nk1ORE9zQkNkdzc1MnJpUldVTnhKeUsycE1rcGdwMi1SN3F4bkZUdHZGNUJWT1RLeS1ZMFJUVkdmOXpHcnpId0N2QW9oOEVsbkYyVU9xbUtnTEVBdW1kNnlOY2wwVGVUY1dCc3N5WkQ5ZTBRUTFKSndYUU4zYVU2aUc1cUlsLUt4d3B6OTZ4Xzl0cC0tMFAwQ0hwM2JWUC0?oc=5</t>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -2509,12 +2513,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2544,7 +2548,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -2595,12 +2599,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2615,7 +2619,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2630,7 +2634,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -2638,32 +2642,32 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>Estados Unidos reclama a Colombia ante ONU el incremento de reclutamiento de menores de edad - El Espectador</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2673,7 +2677,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxPVFRDQXk2WVcwQVhLTmljT1B4akFGM3ozQlBvc3QyOHJua1BfT1hxRnFJY212eFowWTVTdVBmTHN6d2REcXc5VGVuUmw1LWsxNWxOeW82UzBPaVQ3azZfQVNSb0pUTHFqTHdGVWJXS2Z5YmVSbXZJSXd4dzdTamNXdUtqMTRwVDV4MF9acHJFX1pTZ19NVVNvLWdNb1Y1d0FzZlN2dWVMamlvVlNCN01ZS2MxZDh1M250d2tsNEVpc2NYRUJXcE9KYk0yd1FHU3BiNUtFOENRdWZ4ZHdsR0l2cFRFMEpKTGYtaUk4dmhuRjhyaVU3RDYxbUpCUzjSAZACQVVfeXFMTmxJSVphakhMc1dSdUhqdDJFZW00OTIwT0NRNndiZGNtLWROVW1NZFFHWHhTMzVYb3N6aHRBV1NObF94cEVSeHZMOWpPTW1oVXdGeDloRU9uSWpIUXNldU1qY2lUM3dNWnhwMUNESWVTUy1SNGYzZkM0Nk1ORE9zQkNkdzc1MnJpUldVTnhKeUsycE1rcGdwMi1SN3F4bkZUdHZGNUJWT1RLeS1ZMFJUVkdmOXpHcnpId0N2QW9oOEVsbkYyVU9xbUtnTEVBdW1kNnlOY2wwVGVUY1dCc3N5WkQ5ZTBRUTFKSndYUU4zYVU2aUc1cUlsLUt4d3B6OTZ4Xzl0cC0tMFAwQ0hwM2JWUC0?oc=5</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -2681,12 +2685,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>En el regreso a clases, el sueño insuficiente en adolescentes duplica el riesgo de problemas de atención y conducta - Infobae</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2706,7 +2710,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2716,7 +2720,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNTjNaNDNPUHFZYzdoUlNIaUJZbGlqb2JPZndHd3Rad0F4VGwtRHFFQXdzaEIzRWN3bndOTjhsa0JReEtYS1B3TWN5ZVhaRG1RZGtxTkVDVVI2TWV0aTFxTC1KZUJfT2NDZEpIc0tLckJjMmhEOHZvZjVHaEhGRDB2c2NxSmw5SUJpVi0tUlVaZDI1cDgyY1p5QzVRMTlMQ0NOMlkxNGlad243SzF0TFJXZ3RNRGtRY0xtSW5VSnNZaHZCYUJWWG83RzBEZEY4dUFZYUxtLTlqVGx0bWVjbk9vMzFBS0o2LUlyTXNLb3M3ZzbSAYsCQVVfeXFMTTZoYWJjUTZubmFSQjVXNzlCZkdxTkhLby1HTG1iUmdWVVNSMGZpM3EwNkd3U3NSaVhDZWJJeHpQcC1KbUlUWjhFMERwZVBmRXM5NnJVNFQ2RmFDZmNSaXlkOG5tYWhlZlFydUw5X0xVZGkxWmVIM0tuVmd4eHBOMF9SSExuc2tzQ2stNU9kdjlCemxvZTV4MUlVbElWT3dmYmVSYXE0c0VUQTRUTGtYVDZ1SmRKU0R6Z3ZlTEExQmVMa0RDRHl2ZVlvUmVTQWl3aVJJM3hrQU5rMlpLVUYzOUNjOVBDZmVzdWtoeFdqT3JLaUdGY2JOaUw0MnJyQXVNMTQ4Wl9JNHBaYjdv?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -2729,7 +2733,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2749,7 +2753,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2759,7 +2763,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -2767,12 +2771,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>En el regreso a clases, el sueño insuficiente en adolescentes duplica el riesgo de problemas de atención y conducta - Infobae</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2787,7 +2791,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2802,7 +2806,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNTjNaNDNPUHFZYzdoUlNIaUJZbGlqb2JPZndHd3Rad0F4VGwtRHFFQXdzaEIzRWN3bndOTjhsa0JReEtYS1B3TWN5ZVhaRG1RZGtxTkVDVVI2TWV0aTFxTC1KZUJfT2NDZEpIc0tLckJjMmhEOHZvZjVHaEhGRDB2c2NxSmw5SUJpVi0tUlVaZDI1cDgyY1p5QzVRMTlMQ0NOMlkxNGlad243SzF0TFJXZ3RNRGtRY0xtSW5VSnNZaHZCYUJWWG83RzBEZEY4dUFZYUxtLTlqVGx0bWVjbk9vMzFBS0o2LUlyTXNLb3M3ZzbSAYsCQVVfeXFMTTZoYWJjUTZubmFSQjVXNzlCZkdxTkhLby1HTG1iUmdWVVNSMGZpM3EwNkd3U3NSaVhDZWJJeHpQcC1KbUlUWjhFMERwZVBmRXM5NnJVNFQ2RmFDZmNSaXlkOG5tYWhlZlFydUw5X0xVZGkxWmVIM0tuVmd4eHBOMF9SSExuc2tzQ2stNU9kdjlCemxvZTV4MUlVbElWT3dmYmVSYXE0c0VUQTRUTGtYVDZ1SmRKU0R6Z3ZlTEExQmVMa0RDRHl2ZVlvUmVTQWl3aVJJM3hrQU5rMlpLVUYzOUNjOVBDZmVzdWtoeFdqT3JLaUdGY2JOaUw0MnJyQXVNMTQ4Wl9JNHBaYjdv?oc=5</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -2810,12 +2814,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2835,17 +2839,17 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -2853,27 +2857,27 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2888,7 +2892,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -2896,17 +2900,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2921,71 +2925,63 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Casas de Juventud lanzan nuevos Semilleros Distritales para potenciar el talento juvenil en Bogotá</t>
+          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#f8686f5026</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>•Bogotá abre la convocatoria a semilleros gratuitos en artes, deporte y cultura urbana, dirigidos a jóvenes entre 14 y 28 años de todas las localidades, como una estrategia distrital para fortalecer la expresión, la participación y el desarrollo de...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2995,42 +2991,42 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
         </is>
       </c>
     </row>
@@ -3042,40 +3038,44 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Corte Constitucional fijó nuevos criterios para el manejo de conflictos escolares entre menores de edad - Infobae</t>
+          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOOVhMdnBkeXFCaTNlNTNGX2ZaTGxqVnB0b2FIZ0owQTl3LXFiUldIQ2FhOFJZeGdEa3FJTjRoMkxuTHFYNFFBTTVMakFUY0tob051TWxCOVluajg1d24tdWRxM256TTFndk9FSUQ5b2FpNGY3U3ZxQ00za1JhYThoamVHUnBRVUdySkNHNzFhU1JFQ0JsLVJ1N0ZZLU1EdE5tcUViVXluc2hTWm0zblFKcWxXdW9mVDZic1FTWXpyS1NLTWNaZmlEMXZ1T0xoYVR4U2xwZjVycEtkOE1EQlBYLUtn0gH8AUFVX3lxTFB1aVQ2NGIzQ0hhVm54dGlrb0Q4WWtXUVFrdVA0N2dyVEMzWXN3T1p1QmlVZm4wQzdXZmJnZU5TcjlLSFFGTEZwODlYU0FmTU5ra0wtOEhuUWJVMWh5eXlqVEg2WGhHM2tMOVZwMkxTM25vZUFtRHA0S3JjQ1l3RElwVE8wWjRZSWhCcE5Ib1gwWXVpZ09TM2dvOVc5bzBFbFRWdmtYNUZSTzR3T1VrU1I1V25nLWlDSWsxRVJWUmczUFo2Z2lQNTBhOTR4MzhKZDc4YjJxSXJoaU5OU016NGdDX3JtTXp4dVNBTXozV09XSUhRaTJ0ckJvMS00Vw?oc=5</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3085,7 +3085,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
+          <t>Corte Constitucional fijó nuevos criterios para el manejo de conflictos escolares entre menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3100,12 +3100,12 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3115,7 +3115,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOOVhMdnBkeXFCaTNlNTNGX2ZaTGxqVnB0b2FIZ0owQTl3LXFiUldIQ2FhOFJZeGdEa3FJTjRoMkxuTHFYNFFBTTVMakFUY0tob051TWxCOVluajg1d24tdWRxM256TTFndk9FSUQ5b2FpNGY3U3ZxQ00za1JhYThoamVHUnBRVUdySkNHNzFhU1JFQ0JsLVJ1N0ZZLU1EdE5tcUViVXluc2hTWm0zblFKcWxXdW9mVDZic1FTWXpyS1NLTWNaZmlEMXZ1T0xoYVR4U2xwZjVycEtkOE1EQlBYLUtn0gH8AUFVX3lxTFB1aVQ2NGIzQ0hhVm54dGlrb0Q4WWtXUVFrdVA0N2dyVEMzWXN3T1p1QmlVZm4wQzdXZmJnZU5TcjlLSFFGTEZwODlYU0FmTU5ra0wtOEhuUWJVMWh5eXlqVEg2WGhHM2tMOVZwMkxTM25vZUFtRHA0S3JjQ1l3RElwVE8wWjRZSWhCcE5Ib1gwWXVpZ09TM2dvOVc5bzBFbFRWdmtYNUZSTzR3T1VrU1I1V25nLWlDSWsxRVJWUmczUFo2Z2lQNTBhOTR4MzhKZDc4YjJxSXJoaU5OU016NGdDX3JtTXp4dVNBTXozV09XSUhRaTJ0ckJvMS00Vw?oc=5</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -3123,12 +3123,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3143,12 +3143,12 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -3166,27 +3166,27 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Casas de Juventud lanzan nuevos Semilleros Distritales para potenciar el talento juvenil en Bogotá</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3201,20 +3201,24 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#f8686f5026</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>•Bogotá abre la convocatoria a semilleros gratuitos en artes, deporte y cultura urbana, dirigidos a jóvenes entre 14 y 28 años de todas las localidades, como una estrategia distrital para fortalecer la expresión, la participación y el desarrollo de...</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3229,12 +3233,12 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3244,7 +3248,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -3252,12 +3256,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3272,22 +3276,22 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -3300,7 +3304,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
+          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3320,7 +3324,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3330,7 +3334,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -3343,7 +3347,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3358,22 +3362,22 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -3386,7 +3390,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3401,22 +3405,22 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -3424,17 +3428,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3449,17 +3453,17 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -3467,17 +3471,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3487,12 +3491,12 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3502,14 +3506,10 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3519,12 +3519,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3534,22 +3534,22 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
+          <t>https://www.alertabogota.com/noticias/local</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -3557,17 +3557,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3577,12 +3577,12 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Barranquilla</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3592,30 +3592,34 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3635,7 +3639,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -3643,32 +3647,32 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
+          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3678,7 +3682,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
@@ -3686,32 +3690,32 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
+          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3721,7 +3725,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -3729,32 +3733,32 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
+          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3764,7 +3768,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
         </is>
       </c>
       <c r="I75" t="inlineStr"/>
@@ -3772,12 +3776,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
+          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3797,7 +3801,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3807,7 +3811,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
         </is>
       </c>
       <c r="I76" t="inlineStr"/>
@@ -3815,27 +3819,27 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
+          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3850,7 +3854,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
@@ -3858,17 +3862,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
+          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Noticias Caracol</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -3878,7 +3882,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3893,7 +3897,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -3901,27 +3905,27 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
+          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3936,7 +3940,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -3944,17 +3948,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
+          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Noticias Caracol</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3964,22 +3968,22 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -3987,12 +3991,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
+          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4012,7 +4016,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4022,7 +4026,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -4030,27 +4034,27 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
+          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Política pública</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -4065,71 +4069,63 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2025-11-13</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
+          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2025-11-07</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
+          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4144,7 +4140,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Política pública</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -4159,24 +4155,24 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
+          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2025-10-16</t>
+          <t>2025-11-13</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
+          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4191,7 +4187,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -4206,24 +4202,24 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
+          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2025-10-09</t>
+          <t>2025-11-07</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
+          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4238,7 +4234,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -4253,24 +4249,24 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
+          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2025-09-23</t>
+          <t>2025-10-16</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
+          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4300,24 +4296,24 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2025-09-19</t>
+          <t>2025-10-09</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
+          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -4347,24 +4343,24 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
+          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2025-09-13</t>
+          <t>2025-09-23</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
+          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -4394,24 +4390,24 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2025-09-19</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -4426,7 +4422,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -4441,24 +4437,24 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2025-09-09</t>
+          <t>2025-09-13</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4488,57 +4484,151 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2025-09-09</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
           <t>2025-09-06</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="B94" t="inlineStr">
         <is>
           <t>El Frailejón abre sus puertas: Usme estrena nueva Casa de la Juventud</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
+      <c r="C94" t="inlineStr">
         <is>
           <t>SDIS - Juventud</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr">
+      <c r="D94" t="inlineStr">
         <is>
           <t>institucional</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr">
+      <c r="E94" t="inlineStr">
         <is>
           <t>Otra</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr">
+      <c r="F94" t="inlineStr">
         <is>
           <t>Bogotá</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr">
+      <c r="G94" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr">
+      <c r="H94" t="inlineStr">
         <is>
           <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c7eca5d4bd</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr">
+      <c r="I94" t="inlineStr">
         <is>
           <t>• Aunque ya existía una Casa de la Juventud en Usme, la sede se traslada y reinaugura para ofrecer mejores condiciones, ampliar servicios y fortalecer la atención a los jóvenes. • La reapertura se desarrolló con el acompañamiento de la Plataforma...</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-03-13
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I94"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,22 +478,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
+          <t>Abren 200 becas para jóvenes del Pacífico que lideren proyectos en sus territorios</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -503,7 +503,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -513,29 +513,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abren-200-becas-para-jovenes-del-pacifico-que-lideren-proyectos-en-sus-territorios/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
+          <t>El programa DALE lidera Pacífico ofrecerá formación, mentorías y acompañamiento a jóvenes que impulsen iniciativas comunitarias en litoral.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
+          <t>Figura de Independiente Medellín dedicó su gol en la clasificación del equipo en la Copa Libertadores a una persona que “está en tratamiento”</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -545,12 +545,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -560,10 +560,14 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/13/figura-de-independiente-medellin-dedico-su-gol-en-la-clasificacion-del-equipo-en-la-copa-libertadores-a-una-persona-que-esta-en-tratamiento/</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>El equipo dirigido por Alejandro Restrepo venció 2-1 a Juventud de Uruguay ante 12.000 hinchas y clasificó a la fase de grupos, donde acompañará a Deportes Tolima, Junior y Santa Fe en el torneo continental</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -573,7 +577,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Estudiantes de colegios públicos en Bogotá que tendrían que reponer clase el sábado</t>
+          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -588,22 +592,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/estudiantes-colegios-publicos-bogota-que-tendrian-que-reponer-clase-PP5091931A</t>
+          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -616,12 +620,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La travesía del gigante telescopio que Rodolfo Llinás le regaló al histórico Observatorio de la Universidad Nacional</t>
+          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -646,14 +650,10 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-travesia-del-gigante-telescopio-que-rodolfo-llinas-le-regalo-al-historico-observatorio-de-la-universidad-nacional/</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>En medio del paro de la Nacional, el cientifico donó su telescopio personal, el más grande instalado en Colombia, ahora al servicio de estudiantes e investigadoresEl artículoLa travesía del gigante telescopio que Rodolfo Llinás le regaló al...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -663,12 +663,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
+          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -678,12 +678,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -693,72 +693,76 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
+          <t>La travesía del gigante telescopio que Rodolfo Llinás le regaló al histórico Observatorio de la Universidad Nacional</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
+          <t>https://www.las2orillas.co/la-travesia-del-gigante-telescopio-que-rodolfo-llinas-le-regalo-al-historico-observatorio-de-la-universidad-nacional/</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
+          <t>En medio del paro de la Nacional, el cientifico donó su telescopio personal, el más grande instalado en Colombia, ahora al servicio de estudiantes e investigadoresEl artículoLa travesía del gigante telescopio que Rodolfo Llinás le regaló al...</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
+          <t>Estudiantes de colegios públicos en Bogotá que tendrían que reponer clase el sábado</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -773,24 +777,20 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/bogota/estudiantes-colegios-publicos-bogota-que-tendrian-que-reponer-clase-PP5091931A</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
+          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -815,27 +815,27 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
+          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
         </is>
       </c>
     </row>
@@ -847,42 +847,42 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
+          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
+          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
+          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
         </is>
       </c>
     </row>
@@ -894,12 +894,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
+          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -909,12 +909,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Valledupar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -924,12 +924,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
+          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
+          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
+          <t>Prosperidad Social inicia entrega de transferencia monetaria de Jóvenes en Paz</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -971,12 +971,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-inicia-entrega-de-transferencia-monetaria-de-jovenes-en-paz/</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
+          <t>Esta transferencia corresponde al ciclo 1 de 2026. Más de 12.000 jóvenes en el país recibirán los recursos. Bogotá D. C., 24 de febrero de 2026. Prosperidad Social realizará este 27 de febrero la transferencia monetaria condicionada para los...</t>
         </is>
       </c>
     </row>
@@ -988,42 +988,42 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
+          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
+          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Prosperidad Social inicia entrega de transferencia monetaria de Jóvenes en Paz</t>
+          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1065,12 +1065,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-inicia-entrega-de-transferencia-monetaria-de-jovenes-en-paz/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Esta transferencia corresponde al ciclo 1 de 2026. Más de 12.000 jóvenes en el país recibirán los recursos. Bogotá D. C., 24 de febrero de 2026. Prosperidad Social realizará este 27 de febrero la transferencia monetaria condicionada para los...</t>
+          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
         </is>
       </c>
     </row>
@@ -1082,12 +1082,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
+          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1097,91 +1097,91 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
+          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
+          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Valledupar</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
+          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
+          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1206,24 +1206,24 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
+          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
+          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1253,24 +1253,24 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
+          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
+          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1300,34 +1300,34 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
+          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
+          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1347,59 +1347,59 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
+          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
+          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
+          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
         </is>
       </c>
     </row>
@@ -1411,64 +1411,64 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
+          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/cultura</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
+          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
+          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1488,87 +1488,91 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
+          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+          <t>https://www.diarioadn.co/seccion/cultura</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
+          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1578,39 +1582,35 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
+          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1625,10 +1625,14 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1638,7 +1642,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas</t>
+          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1668,7 +1672,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/12/la-falta-de-sueno-deteriora-la-salud-cerebral-y-emocional-desde-la-infancia-60-de-los-ninos-y-adolescentes-no-duerme-las-horas-recomendadas/</t>
+          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -1681,7 +1685,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
+          <t>Adam Mosseri, director de Instagram, desmiente la existencia de “la adicción clínica” a las redes sociales</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1696,12 +1700,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1711,12 +1715,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
+          <t>https://www.infobae.com/tecno/2026/02/12/adam-mosseri-director-de-instagram-desmiente-la-existencia-de-la-adiccion-clinica-a-las-redes-sociales/</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
+          <t>El directivo admitió que ciertas funciones de la app como los filtros digitales generan riesgos sobre la imagen corporal y el bienestar de los usuarios jóvenes</t>
         </is>
       </c>
     </row>
@@ -1728,27 +1732,27 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
+          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1758,10 +1762,14 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr"/>
+          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1771,22 +1779,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
+          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1801,7 +1809,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -1814,7 +1822,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Adam Mosseri, director de Instagram, desmiente la existencia de “la adicción clínica” a las redes sociales</t>
+          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1844,39 +1852,35 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/tecno/2026/02/12/adam-mosseri-director-de-instagram-desmiente-la-existencia-de-la-adiccion-clinica-a-las-redes-sociales/</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>El directivo admitió que ciertas funciones de la app como los filtros digitales generan riesgos sobre la imagen corporal y el bienestar de los usuarios jóvenes</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/02/12/la-falta-de-sueno-deteriora-la-salud-cerebral-y-emocional-desde-la-infancia-60-de-los-ninos-y-adolescentes-no-duerme-las-horas-recomendadas/</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
+          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1891,77 +1895,77 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1981,20 +1985,24 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2009,7 +2017,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2024,7 +2032,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -2032,12 +2040,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2052,22 +2060,22 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
@@ -2075,12 +2083,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
+          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2100,17 +2108,17 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
@@ -2118,22 +2126,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
+          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2143,39 +2151,35 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
+          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2190,7 +2194,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2200,7 +2204,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -2213,42 +2217,42 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
+          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/inicio</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
         </is>
       </c>
     </row>
@@ -2260,12 +2264,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
+          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2290,7 +2294,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -2298,12 +2302,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
+          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2318,12 +2322,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2333,7 +2337,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -2341,17 +2345,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
+          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2361,35 +2365,39 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/inicio</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
+          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2419,7 +2427,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -2427,12 +2435,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2447,7 +2455,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2462,7 +2470,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -2470,17 +2478,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2490,7 +2498,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2505,7 +2513,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -2513,12 +2521,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2533,22 +2541,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
+          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -2556,17 +2564,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Estados Unidos hizo llamado de atención a Colombia ante la ONU por aumento de reclutamiento de menores de edad:“Dudas sobre impunidad al terrorismo” - Infobae</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2576,12 +2584,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2591,7 +2599,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgJBVV95cUxNNFJLRzNtTGZtU1ZCaVUxbGR1QUhBMzV5eFVUT2w4TWZVZnNfYmNMX1IydEVyYnhGT3ZJcDZMaG85R0RUUU9LaEsxT0hyYTFEcy1lNmVTMTA4TWlTbzJ2NmJNbTdxTXZQeUVsczJGMTdSZVlYVHlwblhqeG53UzZ5QkhsMVFyTWRORUQtOUNJMXFBSzJiNkZGQjJSZ1lvcWdfUHFTN1duQjJvcWVyMEZIZE01OGMyakhIQk5WbkROZlpIaDg5UHJRLWdEWVVSRlN4N21hNlhvemlncnlCZlNsM1BvYlJrX2hnUEpmREFCT1pzWS14YmtLMzNHWk1ndnN1NVE5YUdaajNmelBLZEViNEFHNHdjbFhqZEHSAbQCQVVfeXFMTXBsTHJ3d1N1RXh4WFdBdjAtMVFYcEJTV2xwd0xHZERGQVlHNXNvcW5hYmdpN09Wd1ljMjR4RjNSRWMxMl8xMmN5TzN2XzQzUDhCdlJ2WjdNSklzMG1yRzI5YnRnRDFhYWo3Wi1wOEdNbHE4UElzU2FGN3Z2b29XX0Z0bXBDczQzbE1oRE9zVjk1VG9OMzZSNlhsbjlFZUp4em84bGxJSTJyRG8yOWlvUkxPZkhVT0picHVCXzRRX2dhY1VTTWlJcUFYRnVBQzV0ck10YkktYXVpSE5uNm40U1lneGt5c0p5VUNzYnl0NEpqWmVLUE5UcWxOT1BJbnFDZmJRSG9XaTYyMXhqT3dhekhSUDBLSnh6dGxBNFNNYzktYTdZMmxmZm13bXhDd2x3Y0tvWkM?oc=5</t>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -2599,12 +2607,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2634,7 +2642,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -2647,22 +2655,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Estados Unidos reclama a Colombia ante ONU el incremento de reclutamiento de menores de edad - El Espectador</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2677,7 +2685,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxPVFRDQXk2WVcwQVhLTmljT1B4akFGM3ozQlBvc3QyOHJua1BfT1hxRnFJY212eFowWTVTdVBmTHN6d2REcXc5VGVuUmw1LWsxNWxOeW82UzBPaVQ3azZfQVNSb0pUTHFqTHdGVWJXS2Z5YmVSbXZJSXd4dzdTamNXdUtqMTRwVDV4MF9acHJFX1pTZ19NVVNvLWdNb1Y1d0FzZlN2dWVMamlvVlNCN01ZS2MxZDh1M250d2tsNEVpc2NYRUJXcE9KYk0yd1FHU3BiNUtFOENRdWZ4ZHdsR0l2cFRFMEpKTGYtaUk4dmhuRjhyaVU3RDYxbUpCUzjSAZACQVVfeXFMTmxJSVphakhMc1dSdUhqdDJFZW00OTIwT0NRNndiZGNtLWROVW1NZFFHWHhTMzVYb3N6aHRBV1NObF94cEVSeHZMOWpPTW1oVXdGeDloRU9uSWpIUXNldU1qY2lUM3dNWnhwMUNESWVTUy1SNGYzZkM0Nk1ORE9zQkNkdzc1MnJpUldVTnhKeUsycE1rcGdwMi1SN3F4bkZUdHZGNUJWT1RLeS1ZMFJUVkdmOXpHcnpId0N2QW9oOEVsbkYyVU9xbUtnTEVBdW1kNnlOY2wwVGVUY1dCc3N5WkQ5ZTBRUTFKSndYUU4zYVU2aUc1cUlsLUt4d3B6OTZ4Xzl0cC0tMFAwQ0hwM2JWUC0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -2685,27 +2693,27 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Estados Unidos reclama a Colombia ante ONU el incremento de reclutamiento de menores de edad - El Espectador</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2720,7 +2728,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxPVFRDQXk2WVcwQVhLTmljT1B4akFGM3ozQlBvc3QyOHJua1BfT1hxRnFJY212eFowWTVTdVBmTHN6d2REcXc5VGVuUmw1LWsxNWxOeW82UzBPaVQ3azZfQVNSb0pUTHFqTHdGVWJXS2Z5YmVSbXZJSXd4dzdTamNXdUtqMTRwVDV4MF9acHJFX1pTZ19NVVNvLWdNb1Y1d0FzZlN2dWVMamlvVlNCN01ZS2MxZDh1M250d2tsNEVpc2NYRUJXcE9KYk0yd1FHU3BiNUtFOENRdWZ4ZHdsR0l2cFRFMEpKTGYtaUk4dmhuRjhyaVU3RDYxbUpCUzjSAZACQVVfeXFMTmxJSVphakhMc1dSdUhqdDJFZW00OTIwT0NRNndiZGNtLWROVW1NZFFHWHhTMzVYb3N6aHRBV1NObF94cEVSeHZMOWpPTW1oVXdGeDloRU9uSWpIUXNldU1qY2lUM3dNWnhwMUNESWVTUy1SNGYzZkM0Nk1ORE9zQkNkdzc1MnJpUldVTnhKeUsycE1rcGdwMi1SN3F4bkZUdHZGNUJWT1RLeS1ZMFJUVkdmOXpHcnpId0N2QW9oOEVsbkYyVU9xbUtnTEVBdW1kNnlOY2wwVGVUY1dCc3N5WkQ5ZTBRUTFKSndYUU4zYVU2aUc1cUlsLUt4d3B6OTZ4Xzl0cC0tMFAwQ0hwM2JWUC0?oc=5</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -2728,12 +2736,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>Estados Unidos hizo llamado de atención a Colombia ante la ONU por aumento de reclutamiento de menores de edad:“Dudas sobre impunidad al terrorismo” - Infobae</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2748,12 +2756,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2763,7 +2771,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://news.google.com/rss/articles/CBMimgJBVV95cUxNNFJLRzNtTGZtU1ZCaVUxbGR1QUhBMzV5eFVUT2w4TWZVZnNfYmNMX1IydEVyYnhGT3ZJcDZMaG85R0RUUU9LaEsxT0hyYTFEcy1lNmVTMTA4TWlTbzJ2NmJNbTdxTXZQeUVsczJGMTdSZVlYVHlwblhqeG53UzZ5QkhsMVFyTWRORUQtOUNJMXFBSzJiNkZGQjJSZ1lvcWdfUHFTN1duQjJvcWVyMEZIZE01OGMyakhIQk5WbkROZlpIaDg5UHJRLWdEWVVSRlN4N21hNlhvemlncnlCZlNsM1BvYlJrX2hnUEpmREFCT1pzWS14YmtLMzNHWk1ndnN1NVE5YUdaajNmelBLZEViNEFHNHdjbFhqZEHSAbQCQVVfeXFMTXBsTHJ3d1N1RXh4WFdBdjAtMVFYcEJTV2xwd0xHZERGQVlHNXNvcW5hYmdpN09Wd1ljMjR4RjNSRWMxMl8xMmN5TzN2XzQzUDhCdlJ2WjdNSklzMG1yRzI5YnRnRDFhYWo3Wi1wOEdNbHE4UElzU2FGN3Z2b29XX0Z0bXBDczQzbE1oRE9zVjk1VG9OMzZSNlhsbjlFZUp4em84bGxJSTJyRG8yOWlvUkxPZkhVT0picHVCXzRRX2dhY1VTTWlJcUFYRnVBQzV0ck10YkktYXVpSE5uNm40U1lneGt5c0p5VUNzYnl0NEpqWmVLUE5UcWxOT1BJbnFDZmJRSG9XaTYyMXhqT3dhekhSUDBLSnh6dGxBNFNNYzktYTdZMmxmZm13bXhDd2x3Y0tvWkM?oc=5</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -2771,12 +2779,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>En el regreso a clases, el sueño insuficiente en adolescentes duplica el riesgo de problemas de atención y conducta - Infobae</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2796,7 +2804,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2806,7 +2814,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNTjNaNDNPUHFZYzdoUlNIaUJZbGlqb2JPZndHd3Rad0F4VGwtRHFFQXdzaEIzRWN3bndOTjhsa0JReEtYS1B3TWN5ZVhaRG1RZGtxTkVDVVI2TWV0aTFxTC1KZUJfT2NDZEpIc0tLckJjMmhEOHZvZjVHaEhGRDB2c2NxSmw5SUJpVi0tUlVaZDI1cDgyY1p5QzVRMTlMQ0NOMlkxNGlad243SzF0TFJXZ3RNRGtRY0xtSW5VSnNZaHZCYUJWWG83RzBEZEY4dUFZYUxtLTlqVGx0bWVjbk9vMzFBS0o2LUlyTXNLb3M3ZzbSAYsCQVVfeXFMTTZoYWJjUTZubmFSQjVXNzlCZkdxTkhLby1HTG1iUmdWVVNSMGZpM3EwNkd3U3NSaVhDZWJJeHpQcC1KbUlUWjhFMERwZVBmRXM5NnJVNFQ2RmFDZmNSaXlkOG5tYWhlZlFydUw5X0xVZGkxWmVIM0tuVmd4eHBOMF9SSExuc2tzQ2stNU9kdjlCemxvZTV4MUlVbElWT3dmYmVSYXE0c0VUQTRUTGtYVDZ1SmRKU0R6Z3ZlTEExQmVMa0RDRHl2ZVlvUmVTQWl3aVJJM3hrQU5rMlpLVUYzOUNjOVBDZmVzdWtoeFdqT3JLaUdGY2JOaUw0MnJyQXVNMTQ4Wl9JNHBaYjdv?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -2819,7 +2827,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2839,7 +2847,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2849,7 +2857,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -2857,12 +2865,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>En el regreso a clases, el sueño insuficiente en adolescentes duplica el riesgo de problemas de atención y conducta - Infobae</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2877,7 +2885,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2892,7 +2900,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNTjNaNDNPUHFZYzdoUlNIaUJZbGlqb2JPZndHd3Rad0F4VGwtRHFFQXdzaEIzRWN3bndOTjhsa0JReEtYS1B3TWN5ZVhaRG1RZGtxTkVDVVI2TWV0aTFxTC1KZUJfT2NDZEpIc0tLckJjMmhEOHZvZjVHaEhGRDB2c2NxSmw5SUJpVi0tUlVaZDI1cDgyY1p5QzVRMTlMQ0NOMlkxNGlad243SzF0TFJXZ3RNRGtRY0xtSW5VSnNZaHZCYUJWWG83RzBEZEY4dUFZYUxtLTlqVGx0bWVjbk9vMzFBS0o2LUlyTXNLb3M3ZzbSAYsCQVVfeXFMTTZoYWJjUTZubmFSQjVXNzlCZkdxTkhLby1HTG1iUmdWVVNSMGZpM3EwNkd3U3NSaVhDZWJJeHpQcC1KbUlUWjhFMERwZVBmRXM5NnJVNFQ2RmFDZmNSaXlkOG5tYWhlZlFydUw5X0xVZGkxWmVIM0tuVmd4eHBOMF9SSExuc2tzQ2stNU9kdjlCemxvZTV4MUlVbElWT3dmYmVSYXE0c0VUQTRUTGtYVDZ1SmRKU0R6Z3ZlTEExQmVMa0RDRHl2ZVlvUmVTQWl3aVJJM3hrQU5rMlpLVUYzOUNjOVBDZmVzdWtoeFdqT3JLaUdGY2JOaUw0MnJyQXVNMTQ4Wl9JNHBaYjdv?oc=5</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -2900,12 +2908,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2925,17 +2933,17 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -2943,27 +2951,27 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2978,7 +2986,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -2986,17 +2994,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3011,71 +3019,63 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
+          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3085,12 +3085,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Corte Constitucional fijó nuevos criterios para el manejo de conflictos escolares entre menores de edad - Infobae</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3115,10 +3115,14 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOOVhMdnBkeXFCaTNlNTNGX2ZaTGxqVnB0b2FIZ0owQTl3LXFiUldIQ2FhOFJZeGdEa3FJTjRoMkxuTHFYNFFBTTVMakFUY0tob051TWxCOVluajg1d24tdWRxM256TTFndk9FSUQ5b2FpNGY3U3ZxQ00za1JhYThoamVHUnBRVUdySkNHNzFhU1JFQ0JsLVJ1N0ZZLU1EdE5tcUViVXluc2hTWm0zblFKcWxXdW9mVDZic1FTWXpyS1NLTWNaZmlEMXZ1T0xoYVR4U2xwZjVycEtkOE1EQlBYLUtn0gH8AUFVX3lxTFB1aVQ2NGIzQ0hhVm54dGlrb0Q4WWtXUVFrdVA0N2dyVEMzWXN3T1p1QmlVZm4wQzdXZmJnZU5TcjlLSFFGTEZwODlYU0FmTU5ra0wtOEhuUWJVMWh5eXlqVEg2WGhHM2tMOVZwMkxTM25vZUFtRHA0S3JjQ1l3RElwVE8wWjRZSWhCcE5Ib1gwWXVpZ09TM2dvOVc5bzBFbFRWdmtYNUZSTzR3T1VrU1I1V25nLWlDSWsxRVJWUmczUFo2Z2lQNTBhOTR4MzhKZDc4YjJxSXJoaU5OU016NGdDX3JtTXp4dVNBTXozV09XSUhRaTJ0ckJvMS00Vw?oc=5</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3128,7 +3132,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
+          <t>Corte Constitucional fijó nuevos criterios para el manejo de conflictos escolares entre menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3143,12 +3147,12 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3158,7 +3162,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOOVhMdnBkeXFCaTNlNTNGX2ZaTGxqVnB0b2FIZ0owQTl3LXFiUldIQ2FhOFJZeGdEa3FJTjRoMkxuTHFYNFFBTTVMakFUY0tob051TWxCOVluajg1d24tdWRxM256TTFndk9FSUQ5b2FpNGY3U3ZxQ00za1JhYThoamVHUnBRVUdySkNHNzFhU1JFQ0JsLVJ1N0ZZLU1EdE5tcUViVXluc2hTWm0zblFKcWxXdW9mVDZic1FTWXpyS1NLTWNaZmlEMXZ1T0xoYVR4U2xwZjVycEtkOE1EQlBYLUtn0gH8AUFVX3lxTFB1aVQ2NGIzQ0hhVm54dGlrb0Q4WWtXUVFrdVA0N2dyVEMzWXN3T1p1QmlVZm4wQzdXZmJnZU5TcjlLSFFGTEZwODlYU0FmTU5ra0wtOEhuUWJVMWh5eXlqVEg2WGhHM2tMOVZwMkxTM25vZUFtRHA0S3JjQ1l3RElwVE8wWjRZSWhCcE5Ib1gwWXVpZ09TM2dvOVc5bzBFbFRWdmtYNUZSTzR3T1VrU1I1V25nLWlDSWsxRVJWUmczUFo2Z2lQNTBhOTR4MzhKZDc4YjJxSXJoaU5OU016NGdDX3JtTXp4dVNBTXozV09XSUhRaTJ0ckJvMS00Vw?oc=5</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -3171,112 +3175,112 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Casas de Juventud lanzan nuevos Semilleros Distritales para potenciar el talento juvenil en Bogotá</t>
+          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#f8686f5026</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>•Bogotá abre la convocatoria a semilleros gratuitos en artes, deporte y cultura urbana, dirigidos a jóvenes entre 14 y 28 años de todas las localidades, como una estrategia distrital para fortalecer la expresión, la participación y el desarrollo de...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Casas de Juventud lanzan nuevos Semilleros Distritales para potenciar el talento juvenil en Bogotá</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#f8686f5026</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>•Bogotá abre la convocatoria a semilleros gratuitos en artes, deporte y cultura urbana, dirigidos a jóvenes entre 14 y 28 años de todas las localidades, como una estrategia distrital para fortalecer la expresión, la participación y el desarrollo de...</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3291,20 +3295,24 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3324,7 +3332,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3334,7 +3342,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -3342,12 +3350,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3362,22 +3370,22 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -3390,7 +3398,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3410,17 +3418,17 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -3433,7 +3441,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3448,22 +3456,22 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -3476,7 +3484,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3491,12 +3499,12 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3506,7 +3514,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -3514,17 +3522,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3539,17 +3547,17 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -3557,17 +3565,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3577,12 +3585,12 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3592,14 +3600,10 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3609,12 +3613,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3624,22 +3628,22 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
+          <t>https://www.alertabogota.com/noticias/local</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -3647,17 +3651,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3667,12 +3671,12 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Barranquilla</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3682,30 +3686,34 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3725,7 +3733,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -3733,32 +3741,32 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
+          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3768,7 +3776,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
       <c r="I75" t="inlineStr"/>
@@ -3776,32 +3784,32 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
+          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3811,7 +3819,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
         </is>
       </c>
       <c r="I76" t="inlineStr"/>
@@ -3819,32 +3827,32 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
+          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3854,7 +3862,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
@@ -3862,12 +3870,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
+          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3887,7 +3895,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3897,7 +3905,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -3905,27 +3913,27 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
+          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3940,7 +3948,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -3948,17 +3956,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
+          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Noticias Caracol</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3968,7 +3976,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3983,7 +3991,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -3991,27 +3999,27 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
+          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -4026,7 +4034,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -4034,17 +4042,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
+          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Noticias Caracol</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4054,22 +4062,22 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
         </is>
       </c>
       <c r="I82" t="inlineStr"/>
@@ -4077,12 +4085,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
+          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -4102,7 +4110,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -4112,7 +4120,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
@@ -4120,27 +4128,27 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
+          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Política pública</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -4155,71 +4163,63 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2025-11-13</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
+          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2025-11-07</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
+          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4234,7 +4234,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Política pública</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -4249,24 +4249,24 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
+          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2025-10-16</t>
+          <t>2025-11-13</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
+          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4281,7 +4281,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -4296,24 +4296,24 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
+          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2025-10-09</t>
+          <t>2025-11-07</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
+          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -4328,7 +4328,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -4343,24 +4343,24 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
+          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2025-09-23</t>
+          <t>2025-10-16</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
+          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -4390,24 +4390,24 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2025-09-19</t>
+          <t>2025-10-09</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
+          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -4437,24 +4437,24 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
+          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2025-09-13</t>
+          <t>2025-09-23</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
+          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4484,24 +4484,24 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2025-09-19</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -4531,24 +4531,24 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2025-09-09</t>
+          <t>2025-09-13</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4578,57 +4578,151 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2025-09-09</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
           <t>2025-09-06</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B96" t="inlineStr">
         <is>
           <t>El Frailejón abre sus puertas: Usme estrena nueva Casa de la Juventud</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
+      <c r="C96" t="inlineStr">
         <is>
           <t>SDIS - Juventud</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="D96" t="inlineStr">
         <is>
           <t>institucional</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr">
+      <c r="E96" t="inlineStr">
         <is>
           <t>Otra</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr">
+      <c r="F96" t="inlineStr">
         <is>
           <t>Bogotá</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr">
+      <c r="G96" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr">
+      <c r="H96" t="inlineStr">
         <is>
           <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c7eca5d4bd</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr">
+      <c r="I96" t="inlineStr">
         <is>
           <t>• Aunque ya existía una Casa de la Juventud en Usme, la sede se traslada y reinaugura para ofrecer mejores condiciones, ampliar servicios y fortalecer la atención a los jóvenes. • La reapertura se desarrolló con el acompañamiento de la Plataforma...</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-03-14
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I96"/>
+  <dimension ref="A1:I100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,32 +478,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Abren 200 becas para jóvenes del Pacífico que lideren proyectos en sus territorios</t>
+          <t>Los therian: un fenómeno que alarma</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -513,29 +513,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/abren-200-becas-para-jovenes-del-pacifico-que-lideren-proyectos-en-sus-territorios/</t>
+          <t>https://www.las2orillas.co/los-therian-un-fenomeno-que-alarma/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>El programa DALE lidera Pacífico ofrecerá formación, mentorías y acompañamiento a jóvenes que impulsen iniciativas comunitarias en litoral.</t>
+          <t>Cuando la identificación con un animal es persistente. se recomienda orientación psicológica para ayudar al joven en el desarrollo de una identidad saludableEl artículoLos therian: un fenómeno que alarmafue publicado originalmente enLas2orillas.co:...</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Figura de Independiente Medellín dedicó su gol en la clasificación del equipo en la Copa Libertadores a una persona que “está en tratamiento”</t>
+          <t>Con $86 mil millones de regalías, Bolívar construirá universidad en Montes de María y otros dos proyectos educativos</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -545,12 +545,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -560,29 +560,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/13/figura-de-independiente-medellin-dedico-su-gol-en-la-clasificacion-del-equipo-en-la-copa-libertadores-a-una-persona-que-esta-en-tratamiento/</t>
+          <t>https://www.las2orillas.co/con-86-mil-millones-de-regalias-bolivar-construira-universidad-en-montes-de-maria-y-otros-dos-proyectos-educativos/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>El equipo dirigido por Alejandro Restrepo venció 2-1 a Juventud de Uruguay ante 12.000 hinchas y clasificó a la fase de grupos, donde acompañará a Deportes Tolima, Junior y Santa Fe en el torneo continental</t>
+          <t>Los proyectos impulsados por Yamil Arana buscan, entre otras cosas, abrir más de 4 mil cupos para jóvenes de una región que durante años fue escenario de conflictoEl artículoCon $86 mil millones de regalías, Bolívar construirá universidad en Montes...</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
+          <t>Pese a todo, la IA podría potenciar el criterio político de la juventud</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -592,12 +592,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -607,25 +607,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
+          <t>https://www.lasillavacia.com/red-de-expertos/red-de-democracia-y-tecnologia/pese-a-todo-la-ia-podria-potenciar-el-criterio-politico-de-la-juventud/</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Aunque la IA genera inquietudes en el ámbito educativo, también puede formar la conciencia política e histórica entre la juventud.The postPese a todo, la IA podría potenciar el criterio político de la juventudappeared first onLa Silla Vacía.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
+          <t>Murió el influencer colombiano Alejo Little a los 33 años: estos fueron los quebrantos de salud que presentó en los últimos meses</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -635,7 +639,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -650,20 +654,24 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/03/14/murio-el-influencer-colombiano-alejo-little-a-los-33-anos-estos-fueron-los-quebrantos-de-salud-que-presento-en-los-ultimos-meses/</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>El creador de contenido compartió experiencias sobre el acoso escolar y promovió la aceptación personal a través de sus redes sociales y charlas en instituciones educativas</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
+          <t>Figura de Independiente Medellín dedicó su gol en la clasificación del equipo en la Copa Libertadores a una persona que “está en tratamiento”</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -678,12 +686,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -693,34 +701,34 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/13/figura-de-independiente-medellin-dedico-su-gol-en-la-clasificacion-del-equipo-en-la-copa-libertadores-a-una-persona-que-esta-en-tratamiento/</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
+          <t>El equipo dirigido por Alejandro Restrepo venció 2-1 a Juventud de Uruguay ante 12.000 hinchas y clasificó a la fase de grupos, donde acompañará a Deportes Tolima, Junior y Santa Fe en el torneo continental</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>La travesía del gigante telescopio que Rodolfo Llinás le regaló al histórico Observatorio de la Universidad Nacional</t>
+          <t>Abren 200 becas para jóvenes del Pacífico que lideren proyectos en sus territorios</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -730,7 +738,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -740,12 +748,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-travesia-del-gigante-telescopio-que-rodolfo-llinas-le-regalo-al-historico-observatorio-de-la-universidad-nacional/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abren-200-becas-para-jovenes-del-pacifico-que-lideren-proyectos-en-sus-territorios/</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>En medio del paro de la Nacional, el cientifico donó su telescopio personal, el más grande instalado en Colombia, ahora al servicio de estudiantes e investigadoresEl artículoLa travesía del gigante telescopio que Rodolfo Llinás le regaló al...</t>
+          <t>El programa DALE lidera Pacífico ofrecerá formación, mentorías y acompañamiento a jóvenes que impulsen iniciativas comunitarias en litoral.</t>
         </is>
       </c>
     </row>
@@ -795,17 +803,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
+          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -815,12 +823,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -830,29 +838,25 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
+          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -877,24 +881,20 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
+          <t>La travesía del gigante telescopio que Rodolfo Llinás le regaló al histórico Observatorio de la Universidad Nacional</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -924,59 +924,59 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
+          <t>https://www.las2orillas.co/la-travesia-del-gigante-telescopio-que-rodolfo-llinas-le-regalo-al-historico-observatorio-de-la-universidad-nacional/</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
+          <t>En medio del paro de la Nacional, el cientifico donó su telescopio personal, el más grande instalado en Colombia, ahora al servicio de estudiantes e investigadoresEl artículoLa travesía del gigante telescopio que Rodolfo Llinás le regaló al...</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Prosperidad Social inicia entrega de transferencia monetaria de Jóvenes en Paz</t>
+          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-inicia-entrega-de-transferencia-monetaria-de-jovenes-en-paz/</t>
+          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Esta transferencia corresponde al ciclo 1 de 2026. Más de 12.000 jóvenes en el país recibirán los recursos. Bogotá D. C., 24 de febrero de 2026. Prosperidad Social realizará este 27 de febrero la transferencia monetaria condicionada para los...</t>
+          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
         </is>
       </c>
     </row>
@@ -1035,42 +1035,42 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
+          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
+          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
+          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
         </is>
       </c>
     </row>
@@ -1082,22 +1082,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
+          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1112,12 +1112,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
+          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1129,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
+          <t>Prosperidad Social inicia entrega de transferencia monetaria de Jóvenes en Paz</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1149,22 +1149,22 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Valledupar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-inicia-entrega-de-transferencia-monetaria-de-jovenes-en-paz/</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
+          <t>Esta transferencia corresponde al ciclo 1 de 2026. Más de 12.000 jóvenes en el país recibirán los recursos. Bogotá D. C., 24 de febrero de 2026. Prosperidad Social realizará este 27 de febrero la transferencia monetaria condicionada para los...</t>
         </is>
       </c>
     </row>
@@ -1176,106 +1176,106 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
+          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
+          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
+          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
+          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
+          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
+          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1300,86 +1300,86 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
+          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
+          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Valledupar</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
+          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
+          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1394,34 +1394,34 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
+          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
+          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1441,213 +1441,217 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
+          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
+          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
+          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
+          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/cultura</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
+          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
+          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
+          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
+          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1657,7 +1661,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1672,67 +1676,71 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/cultura</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Adam Mosseri, director de Instagram, desmiente la existencia de “la adicción clínica” a las redes sociales</t>
+          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/tecno/2026/02/12/adam-mosseri-director-de-instagram-desmiente-la-existencia-de-la-adiccion-clinica-a-las-redes-sociales/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>El directivo admitió que ciertas funciones de la app como los filtros digitales generan riesgos sobre la imagen corporal y el bienestar de los usuarios jóvenes</t>
+          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
+          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1747,12 +1755,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1762,57 +1770,57 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
+          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1822,12 +1830,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas</t>
+          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1837,22 +1845,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/12/la-falta-de-sueno-deteriora-la-salud-cerebral-y-emocional-desde-la-infancia-60-de-los-ninos-y-adolescentes-no-duerme-las-horas-recomendadas/</t>
+          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -1865,40 +1873,44 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
+          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1908,7 +1920,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
+          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1938,71 +1950,67 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
+          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
+          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
+          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2017,22 +2025,22 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -2040,12 +2048,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>Adam Mosseri, director de Instagram, desmiente la existencia de “la adicción clínica” a las redes sociales</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2060,35 +2068,39 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr"/>
+          <t>https://www.infobae.com/tecno/2026/02/12/adam-mosseri-director-de-instagram-desmiente-la-existencia-de-la-adiccion-clinica-a-las-redes-sociales/</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>El directivo admitió que ciertas funciones de la app como los filtros digitales generan riesgos sobre la imagen corporal y el bienestar de los usuarios jóvenes</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
+          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2103,22 +2115,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/02/12/la-falta-de-sueno-deteriora-la-salud-cerebral-y-emocional-desde-la-infancia-60-de-los-ninos-y-adolescentes-no-duerme-las-horas-recomendadas/</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
@@ -2126,55 +2138,59 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
+          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2189,22 +2205,22 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -2212,27 +2228,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2247,29 +2263,25 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
+          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2284,17 +2296,17 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -2302,12 +2314,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
+          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2327,7 +2339,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2337,7 +2349,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -2345,17 +2357,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
+          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2365,12 +2377,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2380,72 +2392,72 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/inicio</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
+          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
+          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2455,22 +2467,22 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -2478,12 +2490,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
+          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2498,12 +2510,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2513,7 +2525,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -2521,17 +2533,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
+          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2541,40 +2553,44 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/inicio</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2584,7 +2600,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2599,7 +2615,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -2607,12 +2623,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2627,22 +2643,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -2650,12 +2666,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
+          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2675,7 +2691,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2685,7 +2701,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -2693,42 +2709,42 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Estados Unidos reclama a Colombia ante ONU el incremento de reclutamiento de menores de edad - El Espectador</t>
+          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxPVFRDQXk2WVcwQVhLTmljT1B4akFGM3ozQlBvc3QyOHJua1BfT1hxRnFJY212eFowWTVTdVBmTHN6d2REcXc5VGVuUmw1LWsxNWxOeW82UzBPaVQ3azZfQVNSb0pUTHFqTHdGVWJXS2Z5YmVSbXZJSXd4dzdTamNXdUtqMTRwVDV4MF9acHJFX1pTZ19NVVNvLWdNb1Y1d0FzZlN2dWVMamlvVlNCN01ZS2MxZDh1M250d2tsNEVpc2NYRUJXcE9KYk0yd1FHU3BiNUtFOENRdWZ4ZHdsR0l2cFRFMEpKTGYtaUk4dmhuRjhyaVU3RDYxbUpCUzjSAZACQVVfeXFMTmxJSVphakhMc1dSdUhqdDJFZW00OTIwT0NRNndiZGNtLWROVW1NZFFHWHhTMzVYb3N6aHRBV1NObF94cEVSeHZMOWpPTW1oVXdGeDloRU9uSWpIUXNldU1qY2lUM3dNWnhwMUNESWVTUy1SNGYzZkM0Nk1ORE9zQkNkdzc1MnJpUldVTnhKeUsycE1rcGdwMi1SN3F4bkZUdHZGNUJWT1RLeS1ZMFJUVkdmOXpHcnpId0N2QW9oOEVsbkYyVU9xbUtnTEVBdW1kNnlOY2wwVGVUY1dCc3N5WkQ5ZTBRUTFKSndYUU4zYVU2aUc1cUlsLUt4d3B6OTZ4Xzl0cC0tMFAwQ0hwM2JWUC0?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -2736,17 +2752,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Estados Unidos hizo llamado de atención a Colombia ante la ONU por aumento de reclutamiento de menores de edad:“Dudas sobre impunidad al terrorismo” - Infobae</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2756,12 +2772,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2771,7 +2787,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgJBVV95cUxNNFJLRzNtTGZtU1ZCaVUxbGR1QUhBMzV5eFVUT2w4TWZVZnNfYmNMX1IydEVyYnhGT3ZJcDZMaG85R0RUUU9LaEsxT0hyYTFEcy1lNmVTMTA4TWlTbzJ2NmJNbTdxTXZQeUVsczJGMTdSZVlYVHlwblhqeG53UzZ5QkhsMVFyTWRORUQtOUNJMXFBSzJiNkZGQjJSZ1lvcWdfUHFTN1duQjJvcWVyMEZIZE01OGMyakhIQk5WbkROZlpIaDg5UHJRLWdEWVVSRlN4N21hNlhvemlncnlCZlNsM1BvYlJrX2hnUEpmREFCT1pzWS14YmtLMzNHWk1ndnN1NVE5YUdaajNmelBLZEViNEFHNHdjbFhqZEHSAbQCQVVfeXFMTXBsTHJ3d1N1RXh4WFdBdjAtMVFYcEJTV2xwd0xHZERGQVlHNXNvcW5hYmdpN09Wd1ljMjR4RjNSRWMxMl8xMmN5TzN2XzQzUDhCdlJ2WjdNSklzMG1yRzI5YnRnRDFhYWo3Wi1wOEdNbHE4UElzU2FGN3Z2b29XX0Z0bXBDczQzbE1oRE9zVjk1VG9OMzZSNlhsbjlFZUp4em84bGxJSTJyRG8yOWlvUkxPZkhVT0picHVCXzRRX2dhY1VTTWlJcUFYRnVBQzV0ck10YkktYXVpSE5uNm40U1lneGt5c0p5VUNzYnl0NEpqWmVLUE5UcWxOT1BJbnFDZmJRSG9XaTYyMXhqT3dhekhSUDBLSnh6dGxBNFNNYzktYTdZMmxmZm13bXhDd2x3Y0tvWkM?oc=5</t>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -2779,12 +2795,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2799,7 +2815,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2814,7 +2830,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -2822,32 +2838,32 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>Estados Unidos reclama a Colombia ante ONU el incremento de reclutamiento de menores de edad - El Espectador</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2857,7 +2873,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxPVFRDQXk2WVcwQVhLTmljT1B4akFGM3ozQlBvc3QyOHJua1BfT1hxRnFJY212eFowWTVTdVBmTHN6d2REcXc5VGVuUmw1LWsxNWxOeW82UzBPaVQ3azZfQVNSb0pUTHFqTHdGVWJXS2Z5YmVSbXZJSXd4dzdTamNXdUtqMTRwVDV4MF9acHJFX1pTZ19NVVNvLWdNb1Y1d0FzZlN2dWVMamlvVlNCN01ZS2MxZDh1M250d2tsNEVpc2NYRUJXcE9KYk0yd1FHU3BiNUtFOENRdWZ4ZHdsR0l2cFRFMEpKTGYtaUk4dmhuRjhyaVU3RDYxbUpCUzjSAZACQVVfeXFMTmxJSVphakhMc1dSdUhqdDJFZW00OTIwT0NRNndiZGNtLWROVW1NZFFHWHhTMzVYb3N6aHRBV1NObF94cEVSeHZMOWpPTW1oVXdGeDloRU9uSWpIUXNldU1qY2lUM3dNWnhwMUNESWVTUy1SNGYzZkM0Nk1ORE9zQkNkdzc1MnJpUldVTnhKeUsycE1rcGdwMi1SN3F4bkZUdHZGNUJWT1RLeS1ZMFJUVkdmOXpHcnpId0N2QW9oOEVsbkYyVU9xbUtnTEVBdW1kNnlOY2wwVGVUY1dCc3N5WkQ5ZTBRUTFKSndYUU4zYVU2aUc1cUlsLUt4d3B6OTZ4Xzl0cC0tMFAwQ0hwM2JWUC0?oc=5</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -2865,12 +2881,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>En el regreso a clases, el sueño insuficiente en adolescentes duplica el riesgo de problemas de atención y conducta - Infobae</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2885,12 +2901,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2900,7 +2916,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNTjNaNDNPUHFZYzdoUlNIaUJZbGlqb2JPZndHd3Rad0F4VGwtRHFFQXdzaEIzRWN3bndOTjhsa0JReEtYS1B3TWN5ZVhaRG1RZGtxTkVDVVI2TWV0aTFxTC1KZUJfT2NDZEpIc0tLckJjMmhEOHZvZjVHaEhGRDB2c2NxSmw5SUJpVi0tUlVaZDI1cDgyY1p5QzVRMTlMQ0NOMlkxNGlad243SzF0TFJXZ3RNRGtRY0xtSW5VSnNZaHZCYUJWWG83RzBEZEY4dUFZYUxtLTlqVGx0bWVjbk9vMzFBS0o2LUlyTXNLb3M3ZzbSAYsCQVVfeXFMTTZoYWJjUTZubmFSQjVXNzlCZkdxTkhLby1HTG1iUmdWVVNSMGZpM3EwNkd3U3NSaVhDZWJJeHpQcC1KbUlUWjhFMERwZVBmRXM5NnJVNFQ2RmFDZmNSaXlkOG5tYWhlZlFydUw5X0xVZGkxWmVIM0tuVmd4eHBOMF9SSExuc2tzQ2stNU9kdjlCemxvZTV4MUlVbElWT3dmYmVSYXE0c0VUQTRUTGtYVDZ1SmRKU0R6Z3ZlTEExQmVMa0RDRHl2ZVlvUmVTQWl3aVJJM3hrQU5rMlpLVUYzOUNjOVBDZmVzdWtoeFdqT3JLaUdGY2JOaUw0MnJyQXVNMTQ4Wl9JNHBaYjdv?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -2908,12 +2924,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
+          <t>Estados Unidos hizo llamado de atención a Colombia ante la ONU por aumento de reclutamiento de menores de edad:“Dudas sobre impunidad al terrorismo” - Infobae</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2928,7 +2944,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2943,7 +2959,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgJBVV95cUxNNFJLRzNtTGZtU1ZCaVUxbGR1QUhBMzV5eFVUT2w4TWZVZnNfYmNMX1IydEVyYnhGT3ZJcDZMaG85R0RUUU9LaEsxT0hyYTFEcy1lNmVTMTA4TWlTbzJ2NmJNbTdxTXZQeUVsczJGMTdSZVlYVHlwblhqeG53UzZ5QkhsMVFyTWRORUQtOUNJMXFBSzJiNkZGQjJSZ1lvcWdfUHFTN1duQjJvcWVyMEZIZE01OGMyakhIQk5WbkROZlpIaDg5UHJRLWdEWVVSRlN4N21hNlhvemlncnlCZlNsM1BvYlJrX2hnUEpmREFCT1pzWS14YmtLMzNHWk1ndnN1NVE5YUdaajNmelBLZEViNEFHNHdjbFhqZEHSAbQCQVVfeXFMTXBsTHJ3d1N1RXh4WFdBdjAtMVFYcEJTV2xwd0xHZERGQVlHNXNvcW5hYmdpN09Wd1ljMjR4RjNSRWMxMl8xMmN5TzN2XzQzUDhCdlJ2WjdNSklzMG1yRzI5YnRnRDFhYWo3Wi1wOEdNbHE4UElzU2FGN3Z2b29XX0Z0bXBDczQzbE1oRE9zVjk1VG9OMzZSNlhsbjlFZUp4em84bGxJSTJyRG8yOWlvUkxPZkhVT0picHVCXzRRX2dhY1VTTWlJcUFYRnVBQzV0ck10YkktYXVpSE5uNm40U1lneGt5c0p5VUNzYnl0NEpqWmVLUE5UcWxOT1BJbnFDZmJRSG9XaTYyMXhqT3dhekhSUDBLSnh6dGxBNFNNYzktYTdZMmxmZm13bXhDd2x3Y0tvWkM?oc=5</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -2951,12 +2967,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2971,12 +2987,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2986,7 +3002,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -2994,12 +3010,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>En el regreso a clases, el sueño insuficiente en adolescentes duplica el riesgo de problemas de atención y conducta - Infobae</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3019,17 +3035,17 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNTjNaNDNPUHFZYzdoUlNIaUJZbGlqb2JPZndHd3Rad0F4VGwtRHFFQXdzaEIzRWN3bndOTjhsa0JReEtYS1B3TWN5ZVhaRG1RZGtxTkVDVVI2TWV0aTFxTC1KZUJfT2NDZEpIc0tLckJjMmhEOHZvZjVHaEhGRDB2c2NxSmw5SUJpVi0tUlVaZDI1cDgyY1p5QzVRMTlMQ0NOMlkxNGlad243SzF0TFJXZ3RNRGtRY0xtSW5VSnNZaHZCYUJWWG83RzBEZEY4dUFZYUxtLTlqVGx0bWVjbk9vMzFBS0o2LUlyTXNLb3M3ZzbSAYsCQVVfeXFMTTZoYWJjUTZubmFSQjVXNzlCZkdxTkhLby1HTG1iUmdWVVNSMGZpM3EwNkd3U3NSaVhDZWJJeHpQcC1KbUlUWjhFMERwZVBmRXM5NnJVNFQ2RmFDZmNSaXlkOG5tYWhlZlFydUw5X0xVZGkxWmVIM0tuVmd4eHBOMF9SSExuc2tzQ2stNU9kdjlCemxvZTV4MUlVbElWT3dmYmVSYXE0c0VUQTRUTGtYVDZ1SmRKU0R6Z3ZlTEExQmVMa0RDRHl2ZVlvUmVTQWl3aVJJM3hrQU5rMlpLVUYzOUNjOVBDZmVzdWtoeFdqT3JLaUdGY2JOaUw0MnJyQXVNMTQ4Wl9JNHBaYjdv?oc=5</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -3037,32 +3053,32 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3072,7 +3088,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -3080,17 +3096,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3115,24 +3131,20 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Corte Constitucional fijó nuevos criterios para el manejo de conflictos escolares entre menores de edad - Infobae</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3147,7 +3159,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3162,7 +3174,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOOVhMdnBkeXFCaTNlNTNGX2ZaTGxqVnB0b2FIZ0owQTl3LXFiUldIQ2FhOFJZeGdEa3FJTjRoMkxuTHFYNFFBTTVMakFUY0tob051TWxCOVluajg1d24tdWRxM256TTFndk9FSUQ5b2FpNGY3U3ZxQ00za1JhYThoamVHUnBRVUdySkNHNzFhU1JFQ0JsLVJ1N0ZZLU1EdE5tcUViVXluc2hTWm0zblFKcWxXdW9mVDZic1FTWXpyS1NLTWNaZmlEMXZ1T0xoYVR4U2xwZjVycEtkOE1EQlBYLUtn0gH8AUFVX3lxTFB1aVQ2NGIzQ0hhVm54dGlrb0Q4WWtXUVFrdVA0N2dyVEMzWXN3T1p1QmlVZm4wQzdXZmJnZU5TcjlLSFFGTEZwODlYU0FmTU5ra0wtOEhuUWJVMWh5eXlqVEg2WGhHM2tMOVZwMkxTM25vZUFtRHA0S3JjQ1l3RElwVE8wWjRZSWhCcE5Ib1gwWXVpZ09TM2dvOVc5bzBFbFRWdmtYNUZSTzR3T1VrU1I1V25nLWlDSWsxRVJWUmczUFo2Z2lQNTBhOTR4MzhKZDc4YjJxSXJoaU5OU016NGdDX3JtTXp4dVNBTXozV09XSUhRaTJ0ckJvMS00Vw?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -3170,12 +3182,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3190,22 +3202,22 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -3213,49 +3225,45 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Casas de Juventud lanzan nuevos Semilleros Distritales para potenciar el talento juvenil en Bogotá</t>
+          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#f8686f5026</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>•Bogotá abre la convocatoria a semilleros gratuitos en artes, deporte y cultura urbana, dirigidos a jóvenes entre 14 y 28 años de todas las localidades, como una estrategia distrital para fortalecer la expresión, la participación y el desarrollo de...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3265,59 +3273,55 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
+          <t>Corte Constitucional fijó nuevos criterios para el manejo de conflictos escolares entre menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOOVhMdnBkeXFCaTNlNTNGX2ZaTGxqVnB0b2FIZ0owQTl3LXFiUldIQ2FhOFJZeGdEa3FJTjRoMkxuTHFYNFFBTTVMakFUY0tob051TWxCOVluajg1d24tdWRxM256TTFndk9FSUQ5b2FpNGY3U3ZxQ00za1JhYThoamVHUnBRVUdySkNHNzFhU1JFQ0JsLVJ1N0ZZLU1EdE5tcUViVXluc2hTWm0zblFKcWxXdW9mVDZic1FTWXpyS1NLTWNaZmlEMXZ1T0xoYVR4U2xwZjVycEtkOE1EQlBYLUtn0gH8AUFVX3lxTFB1aVQ2NGIzQ0hhVm54dGlrb0Q4WWtXUVFrdVA0N2dyVEMzWXN3T1p1QmlVZm4wQzdXZmJnZU5TcjlLSFFGTEZwODlYU0FmTU5ra0wtOEhuUWJVMWh5eXlqVEg2WGhHM2tMOVZwMkxTM25vZUFtRHA0S3JjQ1l3RElwVE8wWjRZSWhCcE5Ib1gwWXVpZ09TM2dvOVc5bzBFbFRWdmtYNUZSTzR3T1VrU1I1V25nLWlDSWsxRVJWUmczUFo2Z2lQNTBhOTR4MzhKZDc4YjJxSXJoaU5OU016NGdDX3JtTXp4dVNBTXozV09XSUhRaTJ0ckJvMS00Vw?oc=5</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3327,7 +3331,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3342,20 +3346,24 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3370,22 +3378,22 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -3393,70 +3401,74 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
+          <t>Casas de Juventud lanzan nuevos Semilleros Distritales para potenciar el talento juvenil en Bogotá</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3471,20 +3483,24 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#f8686f5026</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>•Bogotá abre la convocatoria a semilleros gratuitos en artes, deporte y cultura urbana, dirigidos a jóvenes entre 14 y 28 años de todas las localidades, como una estrategia distrital para fortalecer la expresión, la participación y el desarrollo de...</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3499,22 +3515,22 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -3522,12 +3538,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3557,7 +3573,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -3570,7 +3586,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3585,7 +3601,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3600,7 +3616,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
@@ -3608,17 +3624,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3628,7 +3644,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3643,7 +3659,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -3651,17 +3667,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3671,7 +3687,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3686,24 +3702,20 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3718,7 +3730,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3733,7 +3745,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -3741,12 +3753,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
+          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3761,12 +3773,12 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Barranquilla</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3776,7 +3788,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
         </is>
       </c>
       <c r="I75" t="inlineStr"/>
@@ -3784,42 +3796,42 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
+          <t>https://www.alertabogota.com/noticias/local</t>
         </is>
       </c>
       <c r="I76" t="inlineStr"/>
@@ -3827,22 +3839,22 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3852,7 +3864,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3862,20 +3874,24 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3890,12 +3906,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3905,7 +3921,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -3913,12 +3929,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
+          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3933,12 +3949,12 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3948,7 +3964,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -3956,27 +3972,27 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
+          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3991,7 +4007,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -3999,12 +4015,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
+          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4019,12 +4035,12 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4034,7 +4050,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -4042,17 +4058,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
+          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Noticias Caracol</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4062,12 +4078,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4077,7 +4093,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
         </is>
       </c>
       <c r="I82" t="inlineStr"/>
@@ -4085,12 +4101,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
+          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -4120,7 +4136,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
@@ -4128,12 +4144,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
+          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4153,17 +4169,17 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
@@ -4171,32 +4187,32 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
+          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4206,7 +4222,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -4214,121 +4230,113 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
+          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Noticias Caracol</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Política pública</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2025-11-13</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
+          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2025-11-07</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
+          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -4343,71 +4351,63 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2025-10-16</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
+          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2025-10-09</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
+          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Política pública</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -4437,24 +4437,24 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
+          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2025-09-23</t>
+          <t>2025-11-13</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
+          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4469,7 +4469,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4484,24 +4484,24 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
+          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2025-09-19</t>
+          <t>2025-11-07</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
+          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -4531,24 +4531,24 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
+          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2025-09-13</t>
+          <t>2025-10-16</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
+          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4578,24 +4578,24 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2025-10-09</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4625,24 +4625,24 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2025-09-09</t>
+          <t>2025-09-23</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4672,57 +4672,245 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
+          <t>2025-09-19</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2025-09-09</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
           <t>2025-09-06</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B100" t="inlineStr">
         <is>
           <t>El Frailejón abre sus puertas: Usme estrena nueva Casa de la Juventud</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C100" t="inlineStr">
         <is>
           <t>SDIS - Juventud</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="D100" t="inlineStr">
         <is>
           <t>institucional</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
+      <c r="E100" t="inlineStr">
         <is>
           <t>Otra</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr">
+      <c r="F100" t="inlineStr">
         <is>
           <t>Bogotá</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr">
+      <c r="G100" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr">
+      <c r="H100" t="inlineStr">
         <is>
           <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c7eca5d4bd</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr">
+      <c r="I100" t="inlineStr">
         <is>
           <t>• Aunque ya existía una Casa de la Juventud en Usme, la sede se traslada y reinaugura para ofrecer mejores condiciones, ampliar servicios y fortalecer la atención a los jóvenes. • La reapertura se desarrolló con el acompañamiento de la Plataforma...</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-03-15
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I100"/>
+  <dimension ref="A1:I103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,12 +478,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Los therian: un fenómeno que alarma</t>
+          <t>Compensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo lograron?</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -498,7 +498,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -513,44 +513,44 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/los-therian-un-fenomeno-que-alarma/</t>
+          <t>https://www.las2orillas.co/compensar-firmo-un-sorprendente-acuerdo-con-una-de-las-mejores-ligas-de-futbol-del-mundo-quienes-lo-lograron/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Cuando la identificación con un animal es persistente. se recomienda orientación psicológica para ayudar al joven en el desarrollo de una identidad saludableEl artículoLos therian: un fenómeno que alarmafue publicado originalmente enLas2orillas.co:...</t>
+          <t>La Liga española acepto hacer una alianza con la solida caja de copensacion familiar para fortalecer la formación de jóvenes talentosEl artículoCompensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo...</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Con $86 mil millones de regalías, Bolívar construirá universidad en Montes de María y otros dos proyectos educativos</t>
+          <t>Hallan el cuerpo de una adolescente en vivienda de Sahagún, Córdoba; autoridades investigan</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -560,39 +560,39 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/con-86-mil-millones-de-regalias-bolivar-construira-universidad-en-montes-de-maria-y-otros-dos-proyectos-educativos/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/hallan-el-cuerpo-de-una-menor-en-una-vivienda-de-sahagun-cordoba-autoridades-investigan/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Los proyectos impulsados por Yamil Arana buscan, entre otras cosas, abrir más de 4 mil cupos para jóvenes de una región que durante años fue escenario de conflictoEl artículoCon $86 mil millones de regalías, Bolívar construirá universidad en Montes...</t>
+          <t>En lo que va de este año, este sería el tercer caso de una mujer asesinada en el municipio y el cuarto en el departamento.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pese a todo, la IA podría potenciar el criterio político de la juventud</t>
+          <t>Dos jóvenes fueron detenidos por presunta extorsión en Santo Tomás, Atlántico</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -607,12 +607,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/red-de-expertos/red-de-democracia-y-tecnologia/pese-a-todo-la-ia-podria-potenciar-el-criterio-politico-de-la-juventud/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/dos-jovenes-fueron-detenidos-por-presunta-extorsion-en-santo-tomas-atlantico/</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Aunque la IA genera inquietudes en el ámbito educativo, también puede formar la conciencia política e histórica entre la juventud.The postPese a todo, la IA podría potenciar el criterio político de la juventudappeared first onLa Silla Vacía.</t>
+          <t>La investigación señala que los implicados habrían intimidado a un conductor de furgón.</t>
         </is>
       </c>
     </row>
@@ -624,12 +624,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Murió el influencer colombiano Alejo Little a los 33 años: estos fueron los quebrantos de salud que presentó en los últimos meses</t>
+          <t>Con $86 mil millones de regalías, Bolívar construirá universidad en Montes de María y otros dos proyectos educativos</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -654,29 +654,29 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/14/murio-el-influencer-colombiano-alejo-little-a-los-33-anos-estos-fueron-los-quebrantos-de-salud-que-presento-en-los-ultimos-meses/</t>
+          <t>https://www.las2orillas.co/con-86-mil-millones-de-regalias-bolivar-construira-universidad-en-montes-de-maria-y-otros-dos-proyectos-educativos/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>El creador de contenido compartió experiencias sobre el acoso escolar y promovió la aceptación personal a través de sus redes sociales y charlas en instituciones educativas</t>
+          <t>Los proyectos impulsados por Yamil Arana buscan, entre otras cosas, abrir más de 4 mil cupos para jóvenes de una región que durante años fue escenario de conflictoEl artículoCon $86 mil millones de regalías, Bolívar construirá universidad en Montes...</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Figura de Independiente Medellín dedicó su gol en la clasificación del equipo en la Copa Libertadores a una persona que “está en tratamiento”</t>
+          <t>Los therian: un fenómeno que alarma</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -686,12 +686,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -701,39 +701,39 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/13/figura-de-independiente-medellin-dedico-su-gol-en-la-clasificacion-del-equipo-en-la-copa-libertadores-a-una-persona-que-esta-en-tratamiento/</t>
+          <t>https://www.las2orillas.co/los-therian-un-fenomeno-que-alarma/</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>El equipo dirigido por Alejandro Restrepo venció 2-1 a Juventud de Uruguay ante 12.000 hinchas y clasificó a la fase de grupos, donde acompañará a Deportes Tolima, Junior y Santa Fe en el torneo continental</t>
+          <t>Cuando la identificación con un animal es persistente. se recomienda orientación psicológica para ayudar al joven en el desarrollo de una identidad saludableEl artículoLos therian: un fenómeno que alarmafue publicado originalmente enLas2orillas.co:...</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Abren 200 becas para jóvenes del Pacífico que lideren proyectos en sus territorios</t>
+          <t>Pese a todo, la IA podría potenciar el criterio político de la juventud</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -748,29 +748,29 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/abren-200-becas-para-jovenes-del-pacifico-que-lideren-proyectos-en-sus-territorios/</t>
+          <t>https://www.lasillavacia.com/red-de-expertos/red-de-democracia-y-tecnologia/pese-a-todo-la-ia-podria-potenciar-el-criterio-politico-de-la-juventud/</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>El programa DALE lidera Pacífico ofrecerá formación, mentorías y acompañamiento a jóvenes que impulsen iniciativas comunitarias en litoral.</t>
+          <t>Aunque la IA genera inquietudes en el ámbito educativo, también puede formar la conciencia política e histórica entre la juventud.The postPese a todo, la IA podría potenciar el criterio político de la juventudappeared first onLa Silla Vacía.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Estudiantes de colegios públicos en Bogotá que tendrían que reponer clase el sábado</t>
+          <t>Murió el influencer colombiano Alejo Little a los 33 años: estos fueron los quebrantos de salud que presentó en los últimos meses</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -780,55 +780,59 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/estudiantes-colegios-publicos-bogota-que-tendrian-que-reponer-clase-PP5091931A</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/03/14/murio-el-influencer-colombiano-alejo-little-a-los-33-anos-estos-fueron-los-quebrantos-de-salud-que-presento-en-los-ultimos-meses/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>El creador de contenido compartió experiencias sobre el acoso escolar y promovió la aceptación personal a través de sus redes sociales y charlas en instituciones educativas</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
+          <t>Abren 200 becas para jóvenes del Pacífico que lideren proyectos en sus territorios</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -838,25 +842,29 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abren-200-becas-para-jovenes-del-pacifico-que-lideren-proyectos-en-sus-territorios/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>El programa DALE lidera Pacífico ofrecerá formación, mentorías y acompañamiento a jóvenes que impulsen iniciativas comunitarias en litoral.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
+          <t>Figura de Independiente Medellín dedicó su gol en la clasificación del equipo en la Copa Libertadores a una persona que “está en tratamiento”</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -866,12 +874,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -881,10 +889,14 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/13/figura-de-independiente-medellin-dedico-su-gol-en-la-clasificacion-del-equipo-en-la-copa-libertadores-a-una-persona-que-esta-en-tratamiento/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>El equipo dirigido por Alejandro Restrepo venció 2-1 a Juventud de Uruguay ante 12.000 hinchas y clasificó a la fase de grupos, donde acompañará a Deportes Tolima, Junior y Santa Fe en el torneo continental</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -894,12 +906,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>La travesía del gigante telescopio que Rodolfo Llinás le regaló al histórico Observatorio de la Universidad Nacional</t>
+          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -914,7 +926,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -924,12 +936,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-travesia-del-gigante-telescopio-que-rodolfo-llinas-le-regalo-al-historico-observatorio-de-la-universidad-nacional/</t>
+          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>En medio del paro de la Nacional, el cientifico donó su telescopio personal, el más grande instalado en Colombia, ahora al servicio de estudiantes e investigadoresEl artículoLa travesía del gigante telescopio que Rodolfo Llinás le regaló al...</t>
+          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
         </is>
       </c>
     </row>
@@ -941,12 +953,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
+          <t>Estudiantes de colegios públicos en Bogotá que tendrían que reponer clase el sábado</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -961,86 +973,82 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/bogota/estudiantes-colegios-publicos-bogota-que-tendrian-que-reponer-clase-PP5091931A</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
+          <t>La travesía del gigante telescopio que Rodolfo Llinás le regaló al histórico Observatorio de la Universidad Nacional</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
+          <t>https://www.las2orillas.co/la-travesia-del-gigante-telescopio-que-rodolfo-llinas-le-regalo-al-historico-observatorio-de-la-universidad-nacional/</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
+          <t>En medio del paro de la Nacional, el cientifico donó su telescopio personal, el más grande instalado en Colombia, ahora al servicio de estudiantes e investigadoresEl artículoLa travesía del gigante telescopio que Rodolfo Llinás le regaló al...</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
+          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1065,61 +1073,53 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
+          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Prosperidad Social inicia entrega de transferencia monetaria de Jóvenes en Paz</t>
+          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1159,12 +1159,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-inicia-entrega-de-transferencia-monetaria-de-jovenes-en-paz/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Esta transferencia corresponde al ciclo 1 de 2026. Más de 12.000 jóvenes en el país recibirán los recursos. Bogotá D. C., 24 de febrero de 2026. Prosperidad Social realizará este 27 de febrero la transferencia monetaria condicionada para los...</t>
+          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
         </is>
       </c>
     </row>
@@ -1176,42 +1176,42 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
+          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
+          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
         </is>
       </c>
     </row>
@@ -1223,17 +1223,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
+          <t>Prosperidad Social inicia entrega de transferencia monetaria de Jóvenes en Paz</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1243,22 +1243,22 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-inicia-entrega-de-transferencia-monetaria-de-jovenes-en-paz/</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
+          <t>Esta transferencia corresponde al ciclo 1 de 2026. Más de 12.000 jóvenes en el país recibirán los recursos. Bogotá D. C., 24 de febrero de 2026. Prosperidad Social realizará este 27 de febrero la transferencia monetaria condicionada para los...</t>
         </is>
       </c>
     </row>
@@ -1270,42 +1270,42 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
+          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
+          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
+          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
+          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Valledupar</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1347,12 +1347,12 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
+          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
         </is>
       </c>
     </row>
@@ -1364,22 +1364,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
+          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1394,81 +1394,81 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
+          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
+          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Valledupar</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
+          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
+          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1488,34 +1488,34 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
+          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
+          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1525,34 +1525,34 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
+          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
+          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
+          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1582,133 +1582,133 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
+          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
+          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
+          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
+          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/cultura</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
+          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
+          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1723,177 +1723,185 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
+          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
+          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
+          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+          <t>https://www.diarioadn.co/seccion/cultura</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
+          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
+          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1903,57 +1911,57 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
+          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1963,7 +1971,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
+          <t>Adam Mosseri, director de Instagram, desmiente la existencia de “la adicción clínica” a las redes sociales</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1978,12 +1986,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1993,12 +2001,12 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
+          <t>https://www.infobae.com/tecno/2026/02/12/adam-mosseri-director-de-instagram-desmiente-la-existencia-de-la-adiccion-clinica-a-las-redes-sociales/</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
+          <t>El directivo admitió que ciertas funciones de la app como los filtros digitales generan riesgos sobre la imagen corporal y el bienestar de los usuarios jóvenes</t>
         </is>
       </c>
     </row>
@@ -2010,7 +2018,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
+          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2040,7 +2048,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/02/12/la-falta-de-sueno-deteriora-la-salud-cerebral-y-emocional-desde-la-infancia-60-de-los-ninos-y-adolescentes-no-duerme-las-horas-recomendadas/</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -2053,7 +2061,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Adam Mosseri, director de Instagram, desmiente la existencia de “la adicción clínica” a las redes sociales</t>
+          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2068,12 +2076,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2083,12 +2091,12 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/tecno/2026/02/12/adam-mosseri-director-de-instagram-desmiente-la-existencia-de-la-adiccion-clinica-a-las-redes-sociales/</t>
+          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>El directivo admitió que ciertas funciones de la app como los filtros digitales generan riesgos sobre la imagen corporal y el bienestar de los usuarios jóvenes</t>
+          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2108,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas</t>
+          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2130,7 +2138,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/12/la-falta-de-sueno-deteriora-la-salud-cerebral-y-emocional-desde-la-infancia-60-de-los-ninos-y-adolescentes-no-duerme-las-horas-recomendadas/</t>
+          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
@@ -2138,107 +2146,107 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
+          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2248,7 +2256,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2263,7 +2271,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
+          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
@@ -2271,27 +2279,27 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
+          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2306,20 +2314,24 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2334,22 +2346,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -2357,12 +2369,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2377,22 +2389,22 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -2400,22 +2412,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
+          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2435,29 +2447,25 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
+          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2472,7 +2480,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2482,7 +2490,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -2490,12 +2498,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
+          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2515,7 +2523,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2525,7 +2533,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -2538,59 +2546,59 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
+          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/inicio</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
+          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2600,12 +2608,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2615,7 +2623,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -2623,17 +2631,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
+          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2643,35 +2651,39 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/inicio</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
+          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2686,12 +2698,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2701,7 +2713,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -2709,12 +2721,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
+          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2729,22 +2741,22 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -2752,17 +2764,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2772,22 +2784,22 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -2795,12 +2807,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2820,7 +2832,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2830,7 +2842,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
+          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -2838,42 +2850,42 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Estados Unidos reclama a Colombia ante ONU el incremento de reclutamiento de menores de edad - El Espectador</t>
+          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxPVFRDQXk2WVcwQVhLTmljT1B4akFGM3ozQlBvc3QyOHJua1BfT1hxRnFJY212eFowWTVTdVBmTHN6d2REcXc5VGVuUmw1LWsxNWxOeW82UzBPaVQ3azZfQVNSb0pUTHFqTHdGVWJXS2Z5YmVSbXZJSXd4dzdTamNXdUtqMTRwVDV4MF9acHJFX1pTZ19NVVNvLWdNb1Y1d0FzZlN2dWVMamlvVlNCN01ZS2MxZDh1M250d2tsNEVpc2NYRUJXcE9KYk0yd1FHU3BiNUtFOENRdWZ4ZHdsR0l2cFRFMEpKTGYtaUk4dmhuRjhyaVU3RDYxbUpCUzjSAZACQVVfeXFMTmxJSVphakhMc1dSdUhqdDJFZW00OTIwT0NRNndiZGNtLWROVW1NZFFHWHhTMzVYb3N6aHRBV1NObF94cEVSeHZMOWpPTW1oVXdGeDloRU9uSWpIUXNldU1qY2lUM3dNWnhwMUNESWVTUy1SNGYzZkM0Nk1ORE9zQkNkdzc1MnJpUldVTnhKeUsycE1rcGdwMi1SN3F4bkZUdHZGNUJWT1RLeS1ZMFJUVkdmOXpHcnpId0N2QW9oOEVsbkYyVU9xbUtnTEVBdW1kNnlOY2wwVGVUY1dCc3N5WkQ5ZTBRUTFKSndYUU4zYVU2aUc1cUlsLUt4d3B6OTZ4Xzl0cC0tMFAwQ0hwM2JWUC0?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -2881,17 +2893,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2901,12 +2913,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2916,7 +2928,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -2924,12 +2936,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Estados Unidos hizo llamado de atención a Colombia ante la ONU por aumento de reclutamiento de menores de edad:“Dudas sobre impunidad al terrorismo” - Infobae</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2944,7 +2956,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2959,7 +2971,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgJBVV95cUxNNFJLRzNtTGZtU1ZCaVUxbGR1QUhBMzV5eFVUT2w4TWZVZnNfYmNMX1IydEVyYnhGT3ZJcDZMaG85R0RUUU9LaEsxT0hyYTFEcy1lNmVTMTA4TWlTbzJ2NmJNbTdxTXZQeUVsczJGMTdSZVlYVHlwblhqeG53UzZ5QkhsMVFyTWRORUQtOUNJMXFBSzJiNkZGQjJSZ1lvcWdfUHFTN1duQjJvcWVyMEZIZE01OGMyakhIQk5WbkROZlpIaDg5UHJRLWdEWVVSRlN4N21hNlhvemlncnlCZlNsM1BvYlJrX2hnUEpmREFCT1pzWS14YmtLMzNHWk1ndnN1NVE5YUdaajNmelBLZEViNEFHNHdjbFhqZEHSAbQCQVVfeXFMTXBsTHJ3d1N1RXh4WFdBdjAtMVFYcEJTV2xwd0xHZERGQVlHNXNvcW5hYmdpN09Wd1ljMjR4RjNSRWMxMl8xMmN5TzN2XzQzUDhCdlJ2WjdNSklzMG1yRzI5YnRnRDFhYWo3Wi1wOEdNbHE4UElzU2FGN3Z2b29XX0Z0bXBDczQzbE1oRE9zVjk1VG9OMzZSNlhsbjlFZUp4em84bGxJSTJyRG8yOWlvUkxPZkhVT0picHVCXzRRX2dhY1VTTWlJcUFYRnVBQzV0ck10YkktYXVpSE5uNm40U1lneGt5c0p5VUNzYnl0NEpqWmVLUE5UcWxOT1BJbnFDZmJRSG9XaTYyMXhqT3dhekhSUDBLSnh6dGxBNFNNYzktYTdZMmxmZm13bXhDd2x3Y0tvWkM?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -2967,12 +2979,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2987,7 +2999,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3002,7 +3014,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -3010,12 +3022,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>En el regreso a clases, el sueño insuficiente en adolescentes duplica el riesgo de problemas de atención y conducta - Infobae</t>
+          <t>Estados Unidos hizo llamado de atención a Colombia ante la ONU por aumento de reclutamiento de menores de edad:“Dudas sobre impunidad al terrorismo” - Infobae</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3030,12 +3042,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3045,7 +3057,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNTjNaNDNPUHFZYzdoUlNIaUJZbGlqb2JPZndHd3Rad0F4VGwtRHFFQXdzaEIzRWN3bndOTjhsa0JReEtYS1B3TWN5ZVhaRG1RZGtxTkVDVVI2TWV0aTFxTC1KZUJfT2NDZEpIc0tLckJjMmhEOHZvZjVHaEhGRDB2c2NxSmw5SUJpVi0tUlVaZDI1cDgyY1p5QzVRMTlMQ0NOMlkxNGlad243SzF0TFJXZ3RNRGtRY0xtSW5VSnNZaHZCYUJWWG83RzBEZEY4dUFZYUxtLTlqVGx0bWVjbk9vMzFBS0o2LUlyTXNLb3M3ZzbSAYsCQVVfeXFMTTZoYWJjUTZubmFSQjVXNzlCZkdxTkhLby1HTG1iUmdWVVNSMGZpM3EwNkd3U3NSaVhDZWJJeHpQcC1KbUlUWjhFMERwZVBmRXM5NnJVNFQ2RmFDZmNSaXlkOG5tYWhlZlFydUw5X0xVZGkxWmVIM0tuVmd4eHBOMF9SSExuc2tzQ2stNU9kdjlCemxvZTV4MUlVbElWT3dmYmVSYXE0c0VUQTRUTGtYVDZ1SmRKU0R6Z3ZlTEExQmVMa0RDRHl2ZVlvUmVTQWl3aVJJM3hrQU5rMlpLVUYzOUNjOVBDZmVzdWtoeFdqT3JLaUdGY2JOaUw0MnJyQXVNMTQ4Wl9JNHBaYjdv?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgJBVV95cUxNNFJLRzNtTGZtU1ZCaVUxbGR1QUhBMzV5eFVUT2w4TWZVZnNfYmNMX1IydEVyYnhGT3ZJcDZMaG85R0RUUU9LaEsxT0hyYTFEcy1lNmVTMTA4TWlTbzJ2NmJNbTdxTXZQeUVsczJGMTdSZVlYVHlwblhqeG53UzZ5QkhsMVFyTWRORUQtOUNJMXFBSzJiNkZGQjJSZ1lvcWdfUHFTN1duQjJvcWVyMEZIZE01OGMyakhIQk5WbkROZlpIaDg5UHJRLWdEWVVSRlN4N21hNlhvemlncnlCZlNsM1BvYlJrX2hnUEpmREFCT1pzWS14YmtLMzNHWk1ndnN1NVE5YUdaajNmelBLZEViNEFHNHdjbFhqZEHSAbQCQVVfeXFMTXBsTHJ3d1N1RXh4WFdBdjAtMVFYcEJTV2xwd0xHZERGQVlHNXNvcW5hYmdpN09Wd1ljMjR4RjNSRWMxMl8xMmN5TzN2XzQzUDhCdlJ2WjdNSklzMG1yRzI5YnRnRDFhYWo3Wi1wOEdNbHE4UElzU2FGN3Z2b29XX0Z0bXBDczQzbE1oRE9zVjk1VG9OMzZSNlhsbjlFZUp4em84bGxJSTJyRG8yOWlvUkxPZkhVT0picHVCXzRRX2dhY1VTTWlJcUFYRnVBQzV0ck10YkktYXVpSE5uNm40U1lneGt5c0p5VUNzYnl0NEpqWmVLUE5UcWxOT1BJbnFDZmJRSG9XaTYyMXhqT3dhekhSUDBLSnh6dGxBNFNNYzktYTdZMmxmZm13bXhDd2x3Y0tvWkM?oc=5</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -3053,27 +3065,27 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
+          <t>Estados Unidos reclama a Colombia ante ONU el incremento de reclutamiento de menores de edad - El Espectador</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3088,7 +3100,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxPVFRDQXk2WVcwQVhLTmljT1B4akFGM3ozQlBvc3QyOHJua1BfT1hxRnFJY212eFowWTVTdVBmTHN6d2REcXc5VGVuUmw1LWsxNWxOeW82UzBPaVQ3azZfQVNSb0pUTHFqTHdGVWJXS2Z5YmVSbXZJSXd4dzdTamNXdUtqMTRwVDV4MF9acHJFX1pTZ19NVVNvLWdNb1Y1d0FzZlN2dWVMamlvVlNCN01ZS2MxZDh1M250d2tsNEVpc2NYRUJXcE9KYk0yd1FHU3BiNUtFOENRdWZ4ZHdsR0l2cFRFMEpKTGYtaUk4dmhuRjhyaVU3RDYxbUpCUzjSAZACQVVfeXFMTmxJSVphakhMc1dSdUhqdDJFZW00OTIwT0NRNndiZGNtLWROVW1NZFFHWHhTMzVYb3N6aHRBV1NObF94cEVSeHZMOWpPTW1oVXdGeDloRU9uSWpIUXNldU1qY2lUM3dNWnhwMUNESWVTUy1SNGYzZkM0Nk1ORE9zQkNkdzc1MnJpUldVTnhKeUsycE1rcGdwMi1SN3F4bkZUdHZGNUJWT1RLeS1ZMFJUVkdmOXpHcnpId0N2QW9oOEVsbkYyVU9xbUtnTEVBdW1kNnlOY2wwVGVUY1dCc3N5WkQ5ZTBRUTFKSndYUU4zYVU2aUc1cUlsLUt4d3B6OTZ4Xzl0cC0tMFAwQ0hwM2JWUC0?oc=5</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -3096,12 +3108,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3121,7 +3133,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3131,7 +3143,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -3139,12 +3151,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3159,7 +3171,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3174,7 +3186,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -3182,12 +3194,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3207,17 +3219,17 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -3225,27 +3237,27 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
+          <t>En el regreso a clases, el sueño insuficiente en adolescentes duplica el riesgo de problemas de atención y conducta - Infobae</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3260,7 +3272,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNTjNaNDNPUHFZYzdoUlNIaUJZbGlqb2JPZndHd3Rad0F4VGwtRHFFQXdzaEIzRWN3bndOTjhsa0JReEtYS1B3TWN5ZVhaRG1RZGtxTkVDVVI2TWV0aTFxTC1KZUJfT2NDZEpIc0tLckJjMmhEOHZvZjVHaEhGRDB2c2NxSmw5SUJpVi0tUlVaZDI1cDgyY1p5QzVRMTlMQ0NOMlkxNGlad243SzF0TFJXZ3RNRGtRY0xtSW5VSnNZaHZCYUJWWG83RzBEZEY4dUFZYUxtLTlqVGx0bWVjbk9vMzFBS0o2LUlyTXNLb3M3ZzbSAYsCQVVfeXFMTTZoYWJjUTZubmFSQjVXNzlCZkdxTkhLby1HTG1iUmdWVVNSMGZpM3EwNkd3U3NSaVhDZWJJeHpQcC1KbUlUWjhFMERwZVBmRXM5NnJVNFQ2RmFDZmNSaXlkOG5tYWhlZlFydUw5X0xVZGkxWmVIM0tuVmd4eHBOMF9SSExuc2tzQ2stNU9kdjlCemxvZTV4MUlVbElWT3dmYmVSYXE0c0VUQTRUTGtYVDZ1SmRKU0R6Z3ZlTEExQmVMa0RDRHl2ZVlvUmVTQWl3aVJJM3hrQU5rMlpLVUYzOUNjOVBDZmVzdWtoeFdqT3JLaUdGY2JOaUw0MnJyQXVNMTQ4Wl9JNHBaYjdv?oc=5</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -3268,12 +3280,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Corte Constitucional fijó nuevos criterios para el manejo de conflictos escolares entre menores de edad - Infobae</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3288,7 +3300,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3303,7 +3315,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOOVhMdnBkeXFCaTNlNTNGX2ZaTGxqVnB0b2FIZ0owQTl3LXFiUldIQ2FhOFJZeGdEa3FJTjRoMkxuTHFYNFFBTTVMakFUY0tob051TWxCOVluajg1d24tdWRxM256TTFndk9FSUQ5b2FpNGY3U3ZxQ00za1JhYThoamVHUnBRVUdySkNHNzFhU1JFQ0JsLVJ1N0ZZLU1EdE5tcUViVXluc2hTWm0zblFKcWxXdW9mVDZic1FTWXpyS1NLTWNaZmlEMXZ1T0xoYVR4U2xwZjVycEtkOE1EQlBYLUtn0gH8AUFVX3lxTFB1aVQ2NGIzQ0hhVm54dGlrb0Q4WWtXUVFrdVA0N2dyVEMzWXN3T1p1QmlVZm4wQzdXZmJnZU5TcjlLSFFGTEZwODlYU0FmTU5ra0wtOEhuUWJVMWh5eXlqVEg2WGhHM2tMOVZwMkxTM25vZUFtRHA0S3JjQ1l3RElwVE8wWjRZSWhCcE5Ib1gwWXVpZ09TM2dvOVc5bzBFbFRWdmtYNUZSTzR3T1VrU1I1V25nLWlDSWsxRVJWUmczUFo2Z2lQNTBhOTR4MzhKZDc4YjJxSXJoaU5OU016NGdDX3JtTXp4dVNBTXozV09XSUhRaTJ0ckJvMS00Vw?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -3311,17 +3323,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3336,44 +3348,40 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
+          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3383,7 +3391,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3393,7 +3401,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -3406,44 +3414,40 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
+          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3495,17 +3499,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3520,30 +3524,34 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Corte Constitucional fijó nuevos criterios para el manejo de conflictos escolares entre menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3558,7 +3566,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3573,7 +3581,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOOVhMdnBkeXFCaTNlNTNGX2ZaTGxqVnB0b2FIZ0owQTl3LXFiUldIQ2FhOFJZeGdEa3FJTjRoMkxuTHFYNFFBTTVMakFUY0tob051TWxCOVluajg1d24tdWRxM256TTFndk9FSUQ5b2FpNGY3U3ZxQ00za1JhYThoamVHUnBRVUdySkNHNzFhU1JFQ0JsLVJ1N0ZZLU1EdE5tcUViVXluc2hTWm0zblFKcWxXdW9mVDZic1FTWXpyS1NLTWNaZmlEMXZ1T0xoYVR4U2xwZjVycEtkOE1EQlBYLUtn0gH8AUFVX3lxTFB1aVQ2NGIzQ0hhVm54dGlrb0Q4WWtXUVFrdVA0N2dyVEMzWXN3T1p1QmlVZm4wQzdXZmJnZU5TcjlLSFFGTEZwODlYU0FmTU5ra0wtOEhuUWJVMWh5eXlqVEg2WGhHM2tMOVZwMkxTM25vZUFtRHA0S3JjQ1l3RElwVE8wWjRZSWhCcE5Ib1gwWXVpZ09TM2dvOVc5bzBFbFRWdmtYNUZSTzR3T1VrU1I1V25nLWlDSWsxRVJWUmczUFo2Z2lQNTBhOTR4MzhKZDc4YjJxSXJoaU5OU016NGdDX3JtTXp4dVNBTXozV09XSUhRaTJ0ckJvMS00Vw?oc=5</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -3581,55 +3589,59 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3659,7 +3671,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -3667,12 +3679,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3702,7 +3714,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
@@ -3715,7 +3727,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
+          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3735,7 +3747,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3745,7 +3757,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -3758,7 +3770,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3778,7 +3790,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3788,7 +3800,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
         </is>
       </c>
       <c r="I75" t="inlineStr"/>
@@ -3796,17 +3808,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3821,17 +3833,17 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
         </is>
       </c>
       <c r="I76" t="inlineStr"/>
@@ -3839,17 +3851,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3859,12 +3871,12 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3874,24 +3886,20 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3911,17 +3919,17 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -3929,17 +3937,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -3949,22 +3957,22 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Barranquilla</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
+          <t>https://www.alertabogota.com/noticias/local</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -3972,27 +3980,27 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -4007,40 +4015,44 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4050,7 +4062,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -4058,12 +4070,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
+          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4078,12 +4090,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4093,7 +4105,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
       <c r="I82" t="inlineStr"/>
@@ -4101,27 +4113,27 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
+          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -4136,7 +4148,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
@@ -4144,32 +4156,32 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
+          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -4179,7 +4191,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
@@ -4187,32 +4199,32 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
+          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4222,7 +4234,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -4230,17 +4242,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
+          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Noticias Caracol</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -4250,7 +4262,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -4265,7 +4277,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
@@ -4273,12 +4285,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
+          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4308,7 +4320,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
         </is>
       </c>
       <c r="I87" t="inlineStr"/>
@@ -4316,42 +4328,42 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
+          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
         </is>
       </c>
       <c r="I88" t="inlineStr"/>
@@ -4359,17 +4371,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
+          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Noticias Caracol</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -4379,12 +4391,12 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4394,7 +4406,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
@@ -4402,74 +4414,70 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
+          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Política pública</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2025-11-13</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
+          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4484,71 +4492,63 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2025-11-07</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
+          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2025-10-16</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
+          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4563,7 +4563,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Política pública</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -4578,24 +4578,24 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
+          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2025-10-09</t>
+          <t>2025-11-13</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
+          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4625,24 +4625,24 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
+          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2025-09-23</t>
+          <t>2025-11-07</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
+          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4672,24 +4672,24 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
+          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2025-09-19</t>
+          <t>2025-10-16</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
+          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -4719,24 +4719,24 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2025-09-13</t>
+          <t>2025-10-09</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
+          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4766,24 +4766,24 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
+          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2025-09-23</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -4798,7 +4798,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4813,24 +4813,24 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2025-09-09</t>
+          <t>2025-09-19</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4860,57 +4860,198 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2025-09-09</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
           <t>2025-09-06</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
+      <c r="B103" t="inlineStr">
         <is>
           <t>El Frailejón abre sus puertas: Usme estrena nueva Casa de la Juventud</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
+      <c r="C103" t="inlineStr">
         <is>
           <t>SDIS - Juventud</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr">
+      <c r="D103" t="inlineStr">
         <is>
           <t>institucional</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
+      <c r="E103" t="inlineStr">
         <is>
           <t>Otra</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr">
+      <c r="F103" t="inlineStr">
         <is>
           <t>Bogotá</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr">
+      <c r="G103" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr">
+      <c r="H103" t="inlineStr">
         <is>
           <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c7eca5d4bd</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr">
+      <c r="I103" t="inlineStr">
         <is>
           <t>• Aunque ya existía una Casa de la Juventud en Usme, la sede se traslada y reinaugura para ofrecer mejores condiciones, ampliar servicios y fortalecer la atención a los jóvenes. • La reapertura se desarrolló con el acompañamiento de la Plataforma...</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-03-16
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I103"/>
+  <dimension ref="A1:I105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,32 +478,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Compensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo lograron?</t>
+          <t>Asesinan a joven de 15 años en Cartagena; su padre resultó herido al intentar defenderlo</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -513,34 +513,34 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/compensar-firmo-un-sorprendente-acuerdo-con-una-de-las-mejores-ligas-de-futbol-del-mundo-quienes-lo-lograron/</t>
+          <t>https://www.elespectador.com/colombia/asesinan-a-menor-de-15-anos-en-cartagena-su-padre-resulto-herido-al-intentar-defenderlo/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>La Liga española acepto hacer una alianza con la solida caja de copensacion familiar para fortalecer la formación de jóvenes talentosEl artículoCompensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo...</t>
+          <t>El presunto homicida ya fue localizado y detenido.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hallan el cuerpo de una adolescente en vivienda de Sahagún, Córdoba; autoridades investigan</t>
+          <t>Joven de 29 años ignoró síntomas creyendo que era TDAH, pero un accidente reveló un cáncer cerebral: 'Solo pedía llegar a los 30'</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -560,12 +560,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/hallan-el-cuerpo-de-una-menor-en-una-vivienda-de-sahagun-cordoba-autoridades-investigan/</t>
+          <t>https://www.diarioadn.co/seccion/vida</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>En lo que va de este año, este sería el tercer caso de una mujer asesinada en el municipio y el cuarto en el departamento.</t>
+          <t>Cuando los médicos le informaron del hallazgo en su cerebro, Lauren aseguró que muchas piezas encajaron de repente. "Fue casi un alivio", señaló.</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dos jóvenes fueron detenidos por presunta extorsión en Santo Tomás, Atlántico</t>
+          <t>Hallan el cuerpo de una adolescente en vivienda de Sahagún, Córdoba; autoridades investigan</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -607,24 +607,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/dos-jovenes-fueron-detenidos-por-presunta-extorsion-en-santo-tomas-atlantico/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/hallan-el-cuerpo-de-una-menor-en-una-vivienda-de-sahagun-cordoba-autoridades-investigan/</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>La investigación señala que los implicados habrían intimidado a un conductor de furgón.</t>
+          <t>En lo que va de este año, este sería el tercer caso de una mujer asesinada en el municipio y el cuarto en el departamento.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Con $86 mil millones de regalías, Bolívar construirá universidad en Montes de María y otros dos proyectos educativos</t>
+          <t>Compensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo lograron?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -654,44 +654,44 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/con-86-mil-millones-de-regalias-bolivar-construira-universidad-en-montes-de-maria-y-otros-dos-proyectos-educativos/</t>
+          <t>https://www.las2orillas.co/compensar-firmo-un-sorprendente-acuerdo-con-una-de-las-mejores-ligas-de-futbol-del-mundo-quienes-lo-lograron/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Los proyectos impulsados por Yamil Arana buscan, entre otras cosas, abrir más de 4 mil cupos para jóvenes de una región que durante años fue escenario de conflictoEl artículoCon $86 mil millones de regalías, Bolívar construirá universidad en Montes...</t>
+          <t>La Liga española acepto hacer una alianza con la solida caja de copensacion familiar para fortalecer la formación de jóvenes talentosEl artículoCompensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo...</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Los therian: un fenómeno que alarma</t>
+          <t>Dos jóvenes fueron detenidos por presunta extorsión en Santo Tomás, Atlántico</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -701,12 +701,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/los-therian-un-fenomeno-que-alarma/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/dos-jovenes-fueron-detenidos-por-presunta-extorsion-en-santo-tomas-atlantico/</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Cuando la identificación con un animal es persistente. se recomienda orientación psicológica para ayudar al joven en el desarrollo de una identidad saludableEl artículoLos therian: un fenómeno que alarmafue publicado originalmente enLas2orillas.co:...</t>
+          <t>La investigación señala que los implicados habrían intimidado a un conductor de furgón.</t>
         </is>
       </c>
     </row>
@@ -718,12 +718,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Pese a todo, la IA podría potenciar el criterio político de la juventud</t>
+          <t>Los therian: un fenómeno que alarma</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -733,12 +733,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -748,12 +748,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/red-de-expertos/red-de-democracia-y-tecnologia/pese-a-todo-la-ia-podria-potenciar-el-criterio-politico-de-la-juventud/</t>
+          <t>https://www.las2orillas.co/los-therian-un-fenomeno-que-alarma/</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Aunque la IA genera inquietudes en el ámbito educativo, también puede formar la conciencia política e histórica entre la juventud.The postPese a todo, la IA podría potenciar el criterio político de la juventudappeared first onLa Silla Vacía.</t>
+          <t>Cuando la identificación con un animal es persistente. se recomienda orientación psicológica para ayudar al joven en el desarrollo de una identidad saludableEl artículoLos therian: un fenómeno que alarmafue publicado originalmente enLas2orillas.co:...</t>
         </is>
       </c>
     </row>
@@ -765,12 +765,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Murió el influencer colombiano Alejo Little a los 33 años: estos fueron los quebrantos de salud que presentó en los últimos meses</t>
+          <t>Pese a todo, la IA podría potenciar el criterio político de la juventud</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -780,12 +780,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -795,34 +795,34 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/14/murio-el-influencer-colombiano-alejo-little-a-los-33-anos-estos-fueron-los-quebrantos-de-salud-que-presento-en-los-ultimos-meses/</t>
+          <t>https://www.lasillavacia.com/red-de-expertos/red-de-democracia-y-tecnologia/pese-a-todo-la-ia-podria-potenciar-el-criterio-politico-de-la-juventud/</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>El creador de contenido compartió experiencias sobre el acoso escolar y promovió la aceptación personal a través de sus redes sociales y charlas en instituciones educativas</t>
+          <t>Aunque la IA genera inquietudes en el ámbito educativo, también puede formar la conciencia política e histórica entre la juventud.The postPese a todo, la IA podría potenciar el criterio político de la juventudappeared first onLa Silla Vacía.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abren 200 becas para jóvenes del Pacífico que lideren proyectos en sus territorios</t>
+          <t>Con $86 mil millones de regalías, Bolívar construirá universidad en Montes de María y otros dos proyectos educativos</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -842,24 +842,24 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/abren-200-becas-para-jovenes-del-pacifico-que-lideren-proyectos-en-sus-territorios/</t>
+          <t>https://www.las2orillas.co/con-86-mil-millones-de-regalias-bolivar-construira-universidad-en-montes-de-maria-y-otros-dos-proyectos-educativos/</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>El programa DALE lidera Pacífico ofrecerá formación, mentorías y acompañamiento a jóvenes que impulsen iniciativas comunitarias en litoral.</t>
+          <t>Los proyectos impulsados por Yamil Arana buscan, entre otras cosas, abrir más de 4 mil cupos para jóvenes de una región que durante años fue escenario de conflictoEl artículoCon $86 mil millones de regalías, Bolívar construirá universidad en Montes...</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Figura de Independiente Medellín dedicó su gol en la clasificación del equipo en la Copa Libertadores a una persona que “está en tratamiento”</t>
+          <t>Murió el influencer colombiano Alejo Little a los 33 años: estos fueron los quebrantos de salud que presentó en los últimos meses</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -874,12 +874,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -889,24 +889,24 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/13/figura-de-independiente-medellin-dedico-su-gol-en-la-clasificacion-del-equipo-en-la-copa-libertadores-a-una-persona-que-esta-en-tratamiento/</t>
+          <t>https://www.infobae.com/colombia/2026/03/14/murio-el-influencer-colombiano-alejo-little-a-los-33-anos-estos-fueron-los-quebrantos-de-salud-que-presento-en-los-ultimos-meses/</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>El equipo dirigido por Alejandro Restrepo venció 2-1 a Juventud de Uruguay ante 12.000 hinchas y clasificó a la fase de grupos, donde acompañará a Deportes Tolima, Junior y Santa Fe en el torneo continental</t>
+          <t>El creador de contenido compartió experiencias sobre el acoso escolar y promovió la aceptación personal a través de sus redes sociales y charlas en instituciones educativas</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
+          <t>Figura de Independiente Medellín dedicó su gol en la clasificación del equipo en la Copa Libertadores a una persona que “está en tratamiento”</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -921,12 +921,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -936,34 +936,34 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/13/figura-de-independiente-medellin-dedico-su-gol-en-la-clasificacion-del-equipo-en-la-copa-libertadores-a-una-persona-que-esta-en-tratamiento/</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
+          <t>El equipo dirigido por Alejandro Restrepo venció 2-1 a Juventud de Uruguay ante 12.000 hinchas y clasificó a la fase de grupos, donde acompañará a Deportes Tolima, Junior y Santa Fe en el torneo continental</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Estudiantes de colegios públicos en Bogotá que tendrían que reponer clase el sábado</t>
+          <t>Abren 200 becas para jóvenes del Pacífico que lideren proyectos en sus territorios</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -973,20 +973,24 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/estudiantes-colegios-publicos-bogota-que-tendrian-que-reponer-clase-PP5091931A</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abren-200-becas-para-jovenes-del-pacifico-que-lideren-proyectos-en-sus-territorios/</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>El programa DALE lidera Pacífico ofrecerá formación, mentorías y acompañamiento a jóvenes que impulsen iniciativas comunitarias en litoral.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1043,7 +1047,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
+          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1058,12 +1062,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1073,7 +1077,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
+          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -1086,7 +1090,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
+          <t>Estudiantes de colegios públicos en Bogotá que tendrían que reponer clase el sábado</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1101,22 +1105,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
+          <t>https://www.pulzo.com/nacion/bogota/estudiantes-colegios-publicos-bogota-que-tendrian-que-reponer-clase-PP5091931A</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -1124,94 +1128,90 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
+          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
+          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
+          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
+          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Prosperidad Social inicia entrega de transferencia monetaria de Jóvenes en Paz</t>
+          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1253,12 +1253,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-inicia-entrega-de-transferencia-monetaria-de-jovenes-en-paz/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Esta transferencia corresponde al ciclo 1 de 2026. Más de 12.000 jóvenes en el país recibirán los recursos. Bogotá D. C., 24 de febrero de 2026. Prosperidad Social realizará este 27 de febrero la transferencia monetaria condicionada para los...</t>
+          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1270,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
+          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1300,12 +1300,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
+          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
+          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
+          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1332,27 +1332,27 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
+          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
         </is>
       </c>
     </row>
@@ -1364,17 +1364,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
+          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1384,22 +1384,22 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Valledupar</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
+          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
         </is>
       </c>
     </row>
@@ -1411,12 +1411,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
+          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1426,12 +1426,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Valledupar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1441,12 +1441,12 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
+          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
+          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
         </is>
       </c>
     </row>
@@ -1458,22 +1458,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
+          <t>Prosperidad Social inicia entrega de transferencia monetaria de Jóvenes en Paz</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1488,12 +1488,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-inicia-entrega-de-transferencia-monetaria-de-jovenes-en-paz/</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
+          <t>Esta transferencia corresponde al ciclo 1 de 2026. Más de 12.000 jóvenes en el país recibirán los recursos. Bogotá D. C., 24 de febrero de 2026. Prosperidad Social realizará este 27 de febrero la transferencia monetaria condicionada para los...</t>
         </is>
       </c>
     </row>
@@ -1505,59 +1505,59 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
+          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
+          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
+          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1582,71 +1582,71 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
+          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
+          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
+          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
+          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1676,24 +1676,24 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
+          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
+          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1723,34 +1723,34 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
+          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
+          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1770,59 +1770,59 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
+          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
+          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/cultura</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
+          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
         </is>
       </c>
     </row>
@@ -1834,17 +1834,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
+          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1864,34 +1864,34 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
+          <t>https://www.diarioadn.co/seccion/cultura</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
+          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
+          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1911,35 +1911,39 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
+          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1954,24 +1958,24 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Adam Mosseri, director de Instagram, desmiente la existencia de “la adicción clínica” a las redes sociales</t>
+          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1986,12 +1990,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2001,57 +2005,57 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/tecno/2026/02/12/adam-mosseri-director-de-instagram-desmiente-la-existencia-de-la-adiccion-clinica-a-las-redes-sociales/</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>El directivo admitió que ciertas funciones de la app como los filtros digitales generan riesgos sobre la imagen corporal y el bienestar de los usuarios jóvenes</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas</t>
+          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/12/la-falta-de-sueno-deteriora-la-salud-cerebral-y-emocional-desde-la-infancia-60-de-los-ninos-y-adolescentes-no-duerme-las-horas-recomendadas/</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2061,7 +2065,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
+          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2076,12 +2080,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2091,14 +2095,10 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/02/12/la-falta-de-sueno-deteriora-la-salud-cerebral-y-emocional-desde-la-infancia-60-de-los-ninos-y-adolescentes-no-duerme-las-horas-recomendadas/</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
+          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2123,12 +2123,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2138,10 +2138,14 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr"/>
+          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2151,22 +2155,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
+          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2181,7 +2185,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -2194,7 +2198,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
+          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2224,14 +2228,10 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2241,65 +2241,69 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
+          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
+          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2314,24 +2318,20 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>Adam Mosseri, director de Instagram, desmiente la existencia de “la adicción clínica” a las redes sociales</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2346,45 +2346,49 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr"/>
+          <t>https://www.infobae.com/tecno/2026/02/12/adam-mosseri-director-de-instagram-desmiente-la-existencia-de-la-adiccion-clinica-a-las-redes-sociales/</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>El directivo admitió que ciertas funciones de la app como los filtros digitales generan riesgos sobre la imagen corporal y el bienestar de los usuarios jóvenes</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2404,20 +2408,24 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2432,7 +2440,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2447,7 +2455,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -2455,12 +2463,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2475,22 +2483,22 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -2498,12 +2506,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
+          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2523,17 +2531,17 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -2541,22 +2549,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
+          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2566,39 +2574,35 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
+          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2613,7 +2617,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2623,7 +2627,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -2636,42 +2640,42 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
+          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/inicio</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
         </is>
       </c>
     </row>
@@ -2683,12 +2687,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
+          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2713,7 +2717,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -2721,17 +2725,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
+          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2741,7 +2745,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2756,20 +2760,24 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/inicio</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
+          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2784,22 +2792,22 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -2807,12 +2815,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
+          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2842,7 +2850,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -2850,12 +2858,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2870,7 +2878,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2885,7 +2893,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -2893,17 +2901,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2913,22 +2921,22 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -2936,12 +2944,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2961,7 +2969,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2971,7 +2979,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
+          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -2979,17 +2987,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2999,12 +3007,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3014,7 +3022,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -3022,12 +3030,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Estados Unidos hizo llamado de atención a Colombia ante la ONU por aumento de reclutamiento de menores de edad:“Dudas sobre impunidad al terrorismo” - Infobae</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3042,7 +3050,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -3057,7 +3065,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgJBVV95cUxNNFJLRzNtTGZtU1ZCaVUxbGR1QUhBMzV5eFVUT2w4TWZVZnNfYmNMX1IydEVyYnhGT3ZJcDZMaG85R0RUUU9LaEsxT0hyYTFEcy1lNmVTMTA4TWlTbzJ2NmJNbTdxTXZQeUVsczJGMTdSZVlYVHlwblhqeG53UzZ5QkhsMVFyTWRORUQtOUNJMXFBSzJiNkZGQjJSZ1lvcWdfUHFTN1duQjJvcWVyMEZIZE01OGMyakhIQk5WbkROZlpIaDg5UHJRLWdEWVVSRlN4N21hNlhvemlncnlCZlNsM1BvYlJrX2hnUEpmREFCT1pzWS14YmtLMzNHWk1ndnN1NVE5YUdaajNmelBLZEViNEFHNHdjbFhqZEHSAbQCQVVfeXFMTXBsTHJ3d1N1RXh4WFdBdjAtMVFYcEJTV2xwd0xHZERGQVlHNXNvcW5hYmdpN09Wd1ljMjR4RjNSRWMxMl8xMmN5TzN2XzQzUDhCdlJ2WjdNSklzMG1yRzI5YnRnRDFhYWo3Wi1wOEdNbHE4UElzU2FGN3Z2b29XX0Z0bXBDczQzbE1oRE9zVjk1VG9OMzZSNlhsbjlFZUp4em84bGxJSTJyRG8yOWlvUkxPZkhVT0picHVCXzRRX2dhY1VTTWlJcUFYRnVBQzV0ck10YkktYXVpSE5uNm40U1lneGt5c0p5VUNzYnl0NEpqWmVLUE5UcWxOT1BJbnFDZmJRSG9XaTYyMXhqT3dhekhSUDBLSnh6dGxBNFNNYzktYTdZMmxmZm13bXhDd2x3Y0tvWkM?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -3108,12 +3116,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3128,7 +3136,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3143,7 +3151,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -3151,12 +3159,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>Estados Unidos hizo llamado de atención a Colombia ante la ONU por aumento de reclutamiento de menores de edad:“Dudas sobre impunidad al terrorismo” - Infobae</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3171,12 +3179,12 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3186,7 +3194,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://news.google.com/rss/articles/CBMimgJBVV95cUxNNFJLRzNtTGZtU1ZCaVUxbGR1QUhBMzV5eFVUT2w4TWZVZnNfYmNMX1IydEVyYnhGT3ZJcDZMaG85R0RUUU9LaEsxT0hyYTFEcy1lNmVTMTA4TWlTbzJ2NmJNbTdxTXZQeUVsczJGMTdSZVlYVHlwblhqeG53UzZ5QkhsMVFyTWRORUQtOUNJMXFBSzJiNkZGQjJSZ1lvcWdfUHFTN1duQjJvcWVyMEZIZE01OGMyakhIQk5WbkROZlpIaDg5UHJRLWdEWVVSRlN4N21hNlhvemlncnlCZlNsM1BvYlJrX2hnUEpmREFCT1pzWS14YmtLMzNHWk1ndnN1NVE5YUdaajNmelBLZEViNEFHNHdjbFhqZEHSAbQCQVVfeXFMTXBsTHJ3d1N1RXh4WFdBdjAtMVFYcEJTV2xwd0xHZERGQVlHNXNvcW5hYmdpN09Wd1ljMjR4RjNSRWMxMl8xMmN5TzN2XzQzUDhCdlJ2WjdNSklzMG1yRzI5YnRnRDFhYWo3Wi1wOEdNbHE4UElzU2FGN3Z2b29XX0Z0bXBDczQzbE1oRE9zVjk1VG9OMzZSNlhsbjlFZUp4em84bGxJSTJyRG8yOWlvUkxPZkhVT0picHVCXzRRX2dhY1VTTWlJcUFYRnVBQzV0ck10YkktYXVpSE5uNm40U1lneGt5c0p5VUNzYnl0NEpqWmVLUE5UcWxOT1BJbnFDZmJRSG9XaTYyMXhqT3dhekhSUDBLSnh6dGxBNFNNYzktYTdZMmxmZm13bXhDd2x3Y0tvWkM?oc=5</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -3194,12 +3202,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3229,7 +3237,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -3280,12 +3288,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3300,12 +3308,12 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3315,7 +3323,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -3323,12 +3331,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3348,17 +3356,17 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -3366,27 +3374,27 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3401,7 +3409,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -3409,12 +3417,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3429,22 +3437,22 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -3452,49 +3460,45 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Casas de Juventud lanzan nuevos Semilleros Distritales para potenciar el talento juvenil en Bogotá</t>
+          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#f8686f5026</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>•Bogotá abre la convocatoria a semilleros gratuitos en artes, deporte y cultura urbana, dirigidos a jóvenes entre 14 y 28 años de todas las localidades, como una estrategia distrital para fortalecer la expresión, la participación y el desarrollo de...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3504,42 +3508,42 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
         </is>
       </c>
     </row>
@@ -3594,69 +3598,69 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Casas de Juventud lanzan nuevos Semilleros Distritales para potenciar el talento juvenil en Bogotá</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3671,20 +3675,24 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#f8686f5026</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>•Bogotá abre la convocatoria a semilleros gratuitos en artes, deporte y cultura urbana, dirigidos a jóvenes entre 14 y 28 años de todas las localidades, como una estrategia distrital para fortalecer la expresión, la participación y el desarrollo de...</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3699,12 +3707,12 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3714,7 +3722,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
@@ -3722,12 +3730,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3747,7 +3755,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3757,7 +3765,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -3765,12 +3773,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3785,22 +3793,22 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="I75" t="inlineStr"/>
@@ -3813,7 +3821,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3833,7 +3841,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3843,7 +3851,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
         </is>
       </c>
       <c r="I76" t="inlineStr"/>
@@ -3856,7 +3864,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3871,12 +3879,12 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3886,7 +3894,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
@@ -3899,7 +3907,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3914,22 +3922,22 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -3937,17 +3945,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -3957,22 +3965,22 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -3980,17 +3988,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -4000,29 +4008,25 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4070,17 +4074,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4090,12 +4094,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Barranquilla</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4105,50 +4109,54 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
+          <t>https://www.alertabogota.com/noticias/local</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
@@ -4156,32 +4164,32 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
+          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -4191,7 +4199,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
@@ -4199,32 +4207,32 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
+          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4234,7 +4242,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -4242,32 +4250,32 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
+          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4277,7 +4285,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
@@ -4285,12 +4293,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
+          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4310,7 +4318,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -4320,7 +4328,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
         </is>
       </c>
       <c r="I87" t="inlineStr"/>
@@ -4328,27 +4336,27 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
+          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -4363,7 +4371,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
         </is>
       </c>
       <c r="I88" t="inlineStr"/>
@@ -4371,17 +4379,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
+          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Noticias Caracol</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -4391,7 +4399,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -4406,7 +4414,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
@@ -4414,27 +4422,27 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
+          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -4449,7 +4457,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -4457,17 +4465,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
+          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Noticias Caracol</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -4477,22 +4485,22 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
         </is>
       </c>
       <c r="I91" t="inlineStr"/>
@@ -4500,12 +4508,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
+          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4525,7 +4533,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -4535,7 +4543,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
@@ -4543,27 +4551,27 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
+          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Política pública</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -4578,71 +4586,63 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2025-11-13</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
+          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2025-11-07</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
+          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Política pública</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4672,24 +4672,24 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
+          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2025-10-16</t>
+          <t>2025-11-13</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
+          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -4704,7 +4704,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -4719,24 +4719,24 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
+          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2025-10-09</t>
+          <t>2025-11-07</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
+          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -4766,24 +4766,24 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
+          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2025-09-23</t>
+          <t>2025-10-16</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
+          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -4813,24 +4813,24 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2025-09-19</t>
+          <t>2025-10-09</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
+          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4860,24 +4860,24 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
+          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2025-09-13</t>
+          <t>2025-09-23</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
+          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4907,24 +4907,24 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2025-09-19</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4939,7 +4939,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -4954,24 +4954,24 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2025-09-09</t>
+          <t>2025-09-13</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -5001,57 +5001,151 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2025-09-09</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
           <t>2025-09-06</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B105" t="inlineStr">
         <is>
           <t>El Frailejón abre sus puertas: Usme estrena nueva Casa de la Juventud</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
+      <c r="C105" t="inlineStr">
         <is>
           <t>SDIS - Juventud</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr">
+      <c r="D105" t="inlineStr">
         <is>
           <t>institucional</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
+      <c r="E105" t="inlineStr">
         <is>
           <t>Otra</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr">
+      <c r="F105" t="inlineStr">
         <is>
           <t>Bogotá</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr">
+      <c r="G105" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr">
+      <c r="H105" t="inlineStr">
         <is>
           <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c7eca5d4bd</t>
         </is>
       </c>
-      <c r="I103" t="inlineStr">
+      <c r="I105" t="inlineStr">
         <is>
           <t>• Aunque ya existía una Casa de la Juventud en Usme, la sede se traslada y reinaugura para ofrecer mejores condiciones, ampliar servicios y fortalecer la atención a los jóvenes. • La reapertura se desarrolló con el acompañamiento de la Plataforma...</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-03-17
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,32 +478,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Asesinan a joven de 15 años en Cartagena; su padre resultó herido al intentar defenderlo</t>
+          <t>Estudiantes de un colegio en La Ceja, Antioquia, impidieron la construcción de un hospital sobre un humedal</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -513,29 +513,29 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/asesinan-a-menor-de-15-anos-en-cartagena-su-padre-resulto-herido-al-intentar-defenderlo/</t>
+          <t>https://www.las2orillas.co/estudiantes-de-un-colegio-en-la-ceja-antioquia-impidieron-la-construccion-de-un-hospital-sobre-un-humedal/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>El presunto homicida ya fue localizado y detenido.</t>
+          <t>Estudiantes y docentes del Bernardo Uribe Londoño marchan en defensa de su humedal. Un conflicto entre la salud y el equilibrio ambiental sacude a La CejaEl artículoEstudiantes de un colegio en La Ceja, Antioquia, impidieron la construcción de un...</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Joven de 29 años ignoró síntomas creyendo que era TDAH, pero un accidente reveló un cáncer cerebral: 'Solo pedía llegar a los 30'</t>
+          <t>Mafe Carrascal explicó por qué la bancada del Pacto Histórico por Bogotá no asistió a encuentro con el alcalde Carlos Fernando Galán</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -545,49 +545,49 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
+          <t>https://www.infobae.com/colombia/2026/03/17/mafe-carrascal-explico-por-que-la-bancada-del-pacto-historico-por-bogota-no-asistio-a-encuentro-con-el-alcalde-carlos-fernando-galan/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Cuando los médicos le informaron del hallazgo en su cerebro, Lauren aseguró que muchas piezas encajaron de repente. "Fue casi un alivio", señaló.</t>
+          <t>La representante indicó que la reunión se realizaría a puerta cerrada y que esta decisión contradice los intereses de su partido. Además, afirmó que al gobierno local le falta implementar políticas dirigidas a los jóvenes y a la prevención de...</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hallan el cuerpo de una adolescente en vivienda de Sahagún, Córdoba; autoridades investigan</t>
+          <t>Joven de 29 años ignoró síntomas creyendo que era TDAH, pero un accidente reveló un cáncer cerebral: 'Solo pedía llegar a los 30'</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -607,44 +607,44 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/hallan-el-cuerpo-de-una-menor-en-una-vivienda-de-sahagun-cordoba-autoridades-investigan/</t>
+          <t>https://www.diarioadn.co/seccion/vida</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>En lo que va de este año, este sería el tercer caso de una mujer asesinada en el municipio y el cuarto en el departamento.</t>
+          <t>Cuando los médicos le informaron del hallazgo en su cerebro, Lauren aseguró que muchas piezas encajaron de repente. "Fue casi un alivio", señaló.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Compensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo lograron?</t>
+          <t>Asesinan a joven de 15 años en Cartagena; su padre resultó herido al intentar defenderlo</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -654,12 +654,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/compensar-firmo-un-sorprendente-acuerdo-con-una-de-las-mejores-ligas-de-futbol-del-mundo-quienes-lo-lograron/</t>
+          <t>https://www.elespectador.com/colombia/asesinan-a-menor-de-15-anos-en-cartagena-su-padre-resulto-herido-al-intentar-defenderlo/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>La Liga española acepto hacer una alianza con la solida caja de copensacion familiar para fortalecer la formación de jóvenes talentosEl artículoCompensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo...</t>
+          <t>El presunto homicida ya fue localizado y detenido.</t>
         </is>
       </c>
     </row>
@@ -713,12 +713,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Los therian: un fenómeno que alarma</t>
+          <t>Compensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo lograron?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -748,34 +748,34 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/los-therian-un-fenomeno-que-alarma/</t>
+          <t>https://www.las2orillas.co/compensar-firmo-un-sorprendente-acuerdo-con-una-de-las-mejores-ligas-de-futbol-del-mundo-quienes-lo-lograron/</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Cuando la identificación con un animal es persistente. se recomienda orientación psicológica para ayudar al joven en el desarrollo de una identidad saludableEl artículoLos therian: un fenómeno que alarmafue publicado originalmente enLas2orillas.co:...</t>
+          <t>La Liga española acepto hacer una alianza con la solida caja de copensacion familiar para fortalecer la formación de jóvenes talentosEl artículoCompensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo...</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Pese a todo, la IA podría potenciar el criterio político de la juventud</t>
+          <t>Hallan el cuerpo de una adolescente en vivienda de Sahagún, Córdoba; autoridades investigan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -795,12 +795,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/red-de-expertos/red-de-democracia-y-tecnologia/pese-a-todo-la-ia-podria-potenciar-el-criterio-politico-de-la-juventud/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/hallan-el-cuerpo-de-una-menor-en-una-vivienda-de-sahagun-cordoba-autoridades-investigan/</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Aunque la IA genera inquietudes en el ámbito educativo, también puede formar la conciencia política e histórica entre la juventud.The postPese a todo, la IA podría potenciar el criterio político de la juventudappeared first onLa Silla Vacía.</t>
+          <t>En lo que va de este año, este sería el tercer caso de una mujer asesinada en el municipio y el cuarto en el departamento.</t>
         </is>
       </c>
     </row>
@@ -901,17 +901,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Figura de Independiente Medellín dedicó su gol en la clasificación del equipo en la Copa Libertadores a una persona que “está en tratamiento”</t>
+          <t>Los therian: un fenómeno que alarma</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -921,12 +921,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -936,39 +936,39 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/13/figura-de-independiente-medellin-dedico-su-gol-en-la-clasificacion-del-equipo-en-la-copa-libertadores-a-una-persona-que-esta-en-tratamiento/</t>
+          <t>https://www.las2orillas.co/los-therian-un-fenomeno-que-alarma/</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>El equipo dirigido por Alejandro Restrepo venció 2-1 a Juventud de Uruguay ante 12.000 hinchas y clasificó a la fase de grupos, donde acompañará a Deportes Tolima, Junior y Santa Fe en el torneo continental</t>
+          <t>Cuando la identificación con un animal es persistente. se recomienda orientación psicológica para ayudar al joven en el desarrollo de una identidad saludableEl artículoLos therian: un fenómeno que alarmafue publicado originalmente enLas2orillas.co:...</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Abren 200 becas para jóvenes del Pacífico que lideren proyectos en sus territorios</t>
+          <t>Pese a todo, la IA podría potenciar el criterio político de la juventud</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -983,29 +983,29 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/abren-200-becas-para-jovenes-del-pacifico-que-lideren-proyectos-en-sus-territorios/</t>
+          <t>https://www.lasillavacia.com/red-de-expertos/red-de-democracia-y-tecnologia/pese-a-todo-la-ia-podria-potenciar-el-criterio-politico-de-la-juventud/</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>El programa DALE lidera Pacífico ofrecerá formación, mentorías y acompañamiento a jóvenes que impulsen iniciativas comunitarias en litoral.</t>
+          <t>Aunque la IA genera inquietudes en el ámbito educativo, también puede formar la conciencia política e histórica entre la juventud.The postPese a todo, la IA podría potenciar el criterio político de la juventudappeared first onLa Silla Vacía.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>La travesía del gigante telescopio que Rodolfo Llinás le regaló al histórico Observatorio de la Universidad Nacional</t>
+          <t>Figura de Independiente Medellín dedicó su gol en la clasificación del equipo en la Copa Libertadores a una persona que “está en tratamiento”</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1015,12 +1015,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1030,44 +1030,44 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-travesia-del-gigante-telescopio-que-rodolfo-llinas-le-regalo-al-historico-observatorio-de-la-universidad-nacional/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/13/figura-de-independiente-medellin-dedico-su-gol-en-la-clasificacion-del-equipo-en-la-copa-libertadores-a-una-persona-que-esta-en-tratamiento/</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>En medio del paro de la Nacional, el cientifico donó su telescopio personal, el más grande instalado en Colombia, ahora al servicio de estudiantes e investigadoresEl artículoLa travesía del gigante telescopio que Rodolfo Llinás le regaló al...</t>
+          <t>El equipo dirigido por Alejandro Restrepo venció 2-1 a Juventud de Uruguay ante 12.000 hinchas y clasificó a la fase de grupos, donde acompañará a Deportes Tolima, Junior y Santa Fe en el torneo continental</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
+          <t>Abren 200 becas para jóvenes del Pacífico que lideren proyectos en sus territorios</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1077,10 +1077,14 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abren-200-becas-para-jovenes-del-pacifico-que-lideren-proyectos-en-sus-territorios/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>El programa DALE lidera Pacífico ofrecerá formación, mentorías y acompañamiento a jóvenes que impulsen iniciativas comunitarias en litoral.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1090,12 +1094,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Estudiantes de colegios públicos en Bogotá que tendrían que reponer clase el sábado</t>
+          <t>La travesía del gigante telescopio que Rodolfo Llinás le regaló al histórico Observatorio de la Universidad Nacional</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1110,20 +1114,24 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/estudiantes-colegios-publicos-bogota-que-tendrian-que-reponer-clase-PP5091931A</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
+          <t>https://www.las2orillas.co/la-travesia-del-gigante-telescopio-que-rodolfo-llinas-le-regalo-al-historico-observatorio-de-la-universidad-nacional/</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>En medio del paro de la Nacional, el cientifico donó su telescopio personal, el más grande instalado en Colombia, ahora al servicio de estudiantes e investigadoresEl artículoLa travesía del gigante telescopio que Rodolfo Llinás le regaló al...</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1133,7 +1141,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
+          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1148,12 +1156,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1163,7 +1171,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
+          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -1176,12 +1184,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
+          <t>Estudiantes de colegios públicos en Bogotá que tendrían que reponer clase el sábado</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1196,86 +1204,78 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/bogota/estudiantes-colegios-publicos-bogota-que-tendrian-que-reponer-clase-PP5091931A</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
+          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
+          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1300,12 +1300,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
+          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
+          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
+          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1332,27 +1332,27 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
+          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
         </is>
       </c>
     </row>
@@ -1364,42 +1364,42 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
+          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Valledupar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
+          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
         </is>
       </c>
     </row>
@@ -1411,42 +1411,42 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
+          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
+          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
         </is>
       </c>
     </row>
@@ -1505,42 +1505,42 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
+          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
+          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
+          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
         </is>
       </c>
     </row>
@@ -1552,22 +1552,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
+          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1582,12 +1582,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
+          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
         </is>
       </c>
     </row>
@@ -1599,12 +1599,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
+          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1614,12 +1614,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1629,29 +1629,29 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
+          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
+          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
+          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1676,71 +1676,71 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
+          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
+          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Valledupar</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
+          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
+          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1770,24 +1770,24 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
+          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
+          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1817,106 +1817,106 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
+          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
+          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/cultura</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
+          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
+          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
+          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
         </is>
       </c>
     </row>
@@ -1970,17 +1970,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
+          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2005,67 +2005,71 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/cultura</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
+          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas</t>
+          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2080,12 +2084,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2095,7 +2099,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/12/la-falta-de-sueno-deteriora-la-salud-cerebral-y-emocional-desde-la-infancia-60-de-los-ninos-y-adolescentes-no-duerme-las-horas-recomendadas/</t>
+          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
@@ -2103,47 +2107,47 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
+          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
+          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
         </is>
       </c>
     </row>
@@ -2155,7 +2159,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
+          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2170,12 +2174,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2185,10 +2189,14 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr"/>
+          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2198,22 +2206,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
+          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2228,7 +2236,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -2241,7 +2249,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
+          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2271,14 +2279,10 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2288,40 +2292,44 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
+          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2331,12 +2339,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Adam Mosseri, director de Instagram, desmiente la existencia de “la adicción clínica” a las redes sociales</t>
+          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2346,86 +2354,82 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/tecno/2026/02/12/adam-mosseri-director-de-instagram-desmiente-la-existencia-de-la-adiccion-clinica-a-las-redes-sociales/</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>El directivo admitió que ciertas funciones de la app como los filtros digitales generan riesgos sobre la imagen corporal y el bienestar de los usuarios jóvenes</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
+          <t>Adam Mosseri, director de Instagram, desmiente la existencia de “la adicción clínica” a las redes sociales</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
+          <t>https://www.infobae.com/tecno/2026/02/12/adam-mosseri-director-de-instagram-desmiente-la-existencia-de-la-adiccion-clinica-a-las-redes-sociales/</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
+          <t>El directivo admitió que ciertas funciones de la app como los filtros digitales generan riesgos sobre la imagen corporal y el bienestar de los usuarios jóvenes</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2440,22 +2444,22 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/02/12/la-falta-de-sueno-deteriora-la-salud-cerebral-y-emocional-desde-la-infancia-60-de-los-ninos-y-adolescentes-no-duerme-las-horas-recomendadas/</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -2463,22 +2467,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2498,20 +2502,24 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2526,7 +2534,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2541,7 +2549,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -2549,12 +2557,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2569,22 +2577,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -2592,12 +2600,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
+          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2617,17 +2625,17 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -2635,22 +2643,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
+          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2660,39 +2668,35 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
+          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2707,7 +2711,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2717,7 +2721,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -2730,42 +2734,42 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
+          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/inicio</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
         </is>
       </c>
     </row>
@@ -2777,12 +2781,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
+          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2807,7 +2811,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -2815,17 +2819,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
+          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2835,7 +2839,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2850,20 +2854,24 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/inicio</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
+          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2878,22 +2886,22 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -2901,12 +2909,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
+          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2921,22 +2929,22 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -2944,12 +2952,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2964,22 +2972,22 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -2987,17 +2995,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3007,22 +3015,22 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -3030,12 +3038,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3055,7 +3063,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3065,7 +3073,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
+          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -3073,32 +3081,32 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Estados Unidos reclama a Colombia ante ONU el incremento de reclutamiento de menores de edad - El Espectador</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3108,7 +3116,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxPVFRDQXk2WVcwQVhLTmljT1B4akFGM3ozQlBvc3QyOHJua1BfT1hxRnFJY212eFowWTVTdVBmTHN6d2REcXc5VGVuUmw1LWsxNWxOeW82UzBPaVQ3azZfQVNSb0pUTHFqTHdGVWJXS2Z5YmVSbXZJSXd4dzdTamNXdUtqMTRwVDV4MF9acHJFX1pTZ19NVVNvLWdNb1Y1d0FzZlN2dWVMamlvVlNCN01ZS2MxZDh1M250d2tsNEVpc2NYRUJXcE9KYk0yd1FHU3BiNUtFOENRdWZ4ZHdsR0l2cFRFMEpKTGYtaUk4dmhuRjhyaVU3RDYxbUpCUzjSAZACQVVfeXFMTmxJSVphakhMc1dSdUhqdDJFZW00OTIwT0NRNndiZGNtLWROVW1NZFFHWHhTMzVYb3N6aHRBV1NObF94cEVSeHZMOWpPTW1oVXdGeDloRU9uSWpIUXNldU1qY2lUM3dNWnhwMUNESWVTUy1SNGYzZkM0Nk1ORE9zQkNkdzc1MnJpUldVTnhKeUsycE1rcGdwMi1SN3F4bkZUdHZGNUJWT1RLeS1ZMFJUVkdmOXpHcnpId0N2QW9oOEVsbkYyVU9xbUtnTEVBdW1kNnlOY2wwVGVUY1dCc3N5WkQ5ZTBRUTFKSndYUU4zYVU2aUc1cUlsLUt4d3B6OTZ4Xzl0cC0tMFAwQ0hwM2JWUC0?oc=5</t>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -3116,12 +3124,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3151,7 +3159,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -3202,27 +3210,27 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Estados Unidos reclama a Colombia ante ONU el incremento de reclutamiento de menores de edad - El Espectador</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3237,7 +3245,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxPVFRDQXk2WVcwQVhLTmljT1B4akFGM3ozQlBvc3QyOHJua1BfT1hxRnFJY212eFowWTVTdVBmTHN6d2REcXc5VGVuUmw1LWsxNWxOeW82UzBPaVQ3azZfQVNSb0pUTHFqTHdGVWJXS2Z5YmVSbXZJSXd4dzdTamNXdUtqMTRwVDV4MF9acHJFX1pTZ19NVVNvLWdNb1Y1d0FzZlN2dWVMamlvVlNCN01ZS2MxZDh1M250d2tsNEVpc2NYRUJXcE9KYk0yd1FHU3BiNUtFOENRdWZ4ZHdsR0l2cFRFMEpKTGYtaUk4dmhuRjhyaVU3RDYxbUpCUzjSAZACQVVfeXFMTmxJSVphakhMc1dSdUhqdDJFZW00OTIwT0NRNndiZGNtLWROVW1NZFFHWHhTMzVYb3N6aHRBV1NObF94cEVSeHZMOWpPTW1oVXdGeDloRU9uSWpIUXNldU1qY2lUM3dNWnhwMUNESWVTUy1SNGYzZkM0Nk1ORE9zQkNkdzc1MnJpUldVTnhKeUsycE1rcGdwMi1SN3F4bkZUdHZGNUJWT1RLeS1ZMFJUVkdmOXpHcnpId0N2QW9oOEVsbkYyVU9xbUtnTEVBdW1kNnlOY2wwVGVUY1dCc3N5WkQ5ZTBRUTFKSndYUU4zYVU2aUc1cUlsLUt4d3B6OTZ4Xzl0cC0tMFAwQ0hwM2JWUC0?oc=5</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -3245,12 +3253,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>En el regreso a clases, el sueño insuficiente en adolescentes duplica el riesgo de problemas de atención y conducta - Infobae</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3265,12 +3273,12 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3280,7 +3288,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNTjNaNDNPUHFZYzdoUlNIaUJZbGlqb2JPZndHd3Rad0F4VGwtRHFFQXdzaEIzRWN3bndOTjhsa0JReEtYS1B3TWN5ZVhaRG1RZGtxTkVDVVI2TWV0aTFxTC1KZUJfT2NDZEpIc0tLckJjMmhEOHZvZjVHaEhGRDB2c2NxSmw5SUJpVi0tUlVaZDI1cDgyY1p5QzVRMTlMQ0NOMlkxNGlad243SzF0TFJXZ3RNRGtRY0xtSW5VSnNZaHZCYUJWWG83RzBEZEY4dUFZYUxtLTlqVGx0bWVjbk9vMzFBS0o2LUlyTXNLb3M3ZzbSAYsCQVVfeXFMTTZoYWJjUTZubmFSQjVXNzlCZkdxTkhLby1HTG1iUmdWVVNSMGZpM3EwNkd3U3NSaVhDZWJJeHpQcC1KbUlUWjhFMERwZVBmRXM5NnJVNFQ2RmFDZmNSaXlkOG5tYWhlZlFydUw5X0xVZGkxWmVIM0tuVmd4eHBOMF9SSExuc2tzQ2stNU9kdjlCemxvZTV4MUlVbElWT3dmYmVSYXE0c0VUQTRUTGtYVDZ1SmRKU0R6Z3ZlTEExQmVMa0RDRHl2ZVlvUmVTQWl3aVJJM3hrQU5rMlpLVUYzOUNjOVBDZmVzdWtoeFdqT3JLaUdGY2JOaUw0MnJyQXVNMTQ4Wl9JNHBaYjdv?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -3288,12 +3296,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3323,7 +3331,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -3374,12 +3382,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3394,12 +3402,12 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3409,7 +3417,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -3417,12 +3425,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>En el regreso a clases, el sueño insuficiente en adolescentes duplica el riesgo de problemas de atención y conducta - Infobae</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3442,17 +3450,17 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNTjNaNDNPUHFZYzdoUlNIaUJZbGlqb2JPZndHd3Rad0F4VGwtRHFFQXdzaEIzRWN3bndOTjhsa0JReEtYS1B3TWN5ZVhaRG1RZGtxTkVDVVI2TWV0aTFxTC1KZUJfT2NDZEpIc0tLckJjMmhEOHZvZjVHaEhGRDB2c2NxSmw5SUJpVi0tUlVaZDI1cDgyY1p5QzVRMTlMQ0NOMlkxNGlad243SzF0TFJXZ3RNRGtRY0xtSW5VSnNZaHZCYUJWWG83RzBEZEY4dUFZYUxtLTlqVGx0bWVjbk9vMzFBS0o2LUlyTXNLb3M3ZzbSAYsCQVVfeXFMTTZoYWJjUTZubmFSQjVXNzlCZkdxTkhLby1HTG1iUmdWVVNSMGZpM3EwNkd3U3NSaVhDZWJJeHpQcC1KbUlUWjhFMERwZVBmRXM5NnJVNFQ2RmFDZmNSaXlkOG5tYWhlZlFydUw5X0xVZGkxWmVIM0tuVmd4eHBOMF9SSExuc2tzQ2stNU9kdjlCemxvZTV4MUlVbElWT3dmYmVSYXE0c0VUQTRUTGtYVDZ1SmRKU0R6Z3ZlTEExQmVMa0RDRHl2ZVlvUmVTQWl3aVJJM3hrQU5rMlpLVUYzOUNjOVBDZmVzdWtoeFdqT3JLaUdGY2JOaUw0MnJyQXVNMTQ4Wl9JNHBaYjdv?oc=5</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -3460,27 +3468,27 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3495,7 +3503,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -3503,27 +3511,27 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3538,39 +3546,35 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Corte Constitucional fijó nuevos criterios para el manejo de conflictos escolares entre menores de edad - Infobae</t>
+          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3585,7 +3589,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOOVhMdnBkeXFCaTNlNTNGX2ZaTGxqVnB0b2FIZ0owQTl3LXFiUldIQ2FhOFJZeGdEa3FJTjRoMkxuTHFYNFFBTTVMakFUY0tob051TWxCOVluajg1d24tdWRxM256TTFndk9FSUQ5b2FpNGY3U3ZxQ00za1JhYThoamVHUnBRVUdySkNHNzFhU1JFQ0JsLVJ1N0ZZLU1EdE5tcUViVXluc2hTWm0zblFKcWxXdW9mVDZic1FTWXpyS1NLTWNaZmlEMXZ1T0xoYVR4U2xwZjVycEtkOE1EQlBYLUtn0gH8AUFVX3lxTFB1aVQ2NGIzQ0hhVm54dGlrb0Q4WWtXUVFrdVA0N2dyVEMzWXN3T1p1QmlVZm4wQzdXZmJnZU5TcjlLSFFGTEZwODlYU0FmTU5ra0wtOEhuUWJVMWh5eXlqVEg2WGhHM2tMOVZwMkxTM25vZUFtRHA0S3JjQ1l3RElwVE8wWjRZSWhCcE5Ib1gwWXVpZ09TM2dvOVc5bzBFbFRWdmtYNUZSTzR3T1VrU1I1V25nLWlDSWsxRVJWUmczUFo2Z2lQNTBhOTR4MzhKZDc4YjJxSXJoaU5OU016NGdDX3JtTXp4dVNBTXozV09XSUhRaTJ0ckJvMS00Vw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -3598,12 +3602,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3613,12 +3617,12 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3628,14 +3632,10 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3692,12 +3692,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3707,12 +3707,12 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3722,20 +3722,24 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Corte Constitucional fijó nuevos criterios para el manejo de conflictos escolares entre menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3750,7 +3754,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3765,7 +3769,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOOVhMdnBkeXFCaTNlNTNGX2ZaTGxqVnB0b2FIZ0owQTl3LXFiUldIQ2FhOFJZeGdEa3FJTjRoMkxuTHFYNFFBTTVMakFUY0tob051TWxCOVluajg1d24tdWRxM256TTFndk9FSUQ5b2FpNGY3U3ZxQ00za1JhYThoamVHUnBRVUdySkNHNzFhU1JFQ0JsLVJ1N0ZZLU1EdE5tcUViVXluc2hTWm0zblFKcWxXdW9mVDZic1FTWXpyS1NLTWNaZmlEMXZ1T0xoYVR4U2xwZjVycEtkOE1EQlBYLUtn0gH8AUFVX3lxTFB1aVQ2NGIzQ0hhVm54dGlrb0Q4WWtXUVFrdVA0N2dyVEMzWXN3T1p1QmlVZm4wQzdXZmJnZU5TcjlLSFFGTEZwODlYU0FmTU5ra0wtOEhuUWJVMWh5eXlqVEg2WGhHM2tMOVZwMkxTM25vZUFtRHA0S3JjQ1l3RElwVE8wWjRZSWhCcE5Ib1gwWXVpZ09TM2dvOVc5bzBFbFRWdmtYNUZSTzR3T1VrU1I1V25nLWlDSWsxRVJWUmczUFo2Z2lQNTBhOTR4MzhKZDc4YjJxSXJoaU5OU016NGdDX3JtTXp4dVNBTXozV09XSUhRaTJ0ckJvMS00Vw?oc=5</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -3773,27 +3777,27 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3808,20 +3812,24 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3836,22 +3844,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="I76" t="inlineStr"/>
@@ -3859,12 +3867,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3894,7 +3902,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
@@ -3907,7 +3915,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3927,7 +3935,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3937,7 +3945,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -3950,7 +3958,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3965,12 +3973,12 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3980,7 +3988,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -3993,7 +4001,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4008,22 +4016,22 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -4031,12 +4039,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4056,7 +4064,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4066,7 +4074,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -4074,17 +4082,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4094,29 +4102,25 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4164,17 +4168,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4184,12 +4188,12 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Barranquilla</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -4199,30 +4203,34 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4242,7 +4250,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -4250,32 +4258,32 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
+          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4285,7 +4293,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
@@ -4293,32 +4301,32 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
+          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -4328,7 +4336,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
         </is>
       </c>
       <c r="I87" t="inlineStr"/>
@@ -4336,32 +4344,32 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
+          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -4371,7 +4379,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
         </is>
       </c>
       <c r="I88" t="inlineStr"/>
@@ -4379,12 +4387,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
+          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -4404,7 +4412,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4414,7 +4422,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
@@ -4422,27 +4430,27 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
+          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -4457,7 +4465,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -4465,17 +4473,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
+          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Noticias Caracol</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -4485,7 +4493,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4500,7 +4508,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
         </is>
       </c>
       <c r="I91" t="inlineStr"/>
@@ -4508,27 +4516,27 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
+          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -4543,7 +4551,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
@@ -4551,17 +4559,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
+          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Noticias Caracol</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -4571,22 +4579,22 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
         </is>
       </c>
       <c r="I93" t="inlineStr"/>
@@ -4594,12 +4602,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
+          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4619,7 +4627,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -4629,7 +4637,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
         </is>
       </c>
       <c r="I94" t="inlineStr"/>
@@ -4637,27 +4645,27 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
+          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Política pública</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4672,71 +4680,63 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
-        </is>
-      </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2025-11-13</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
+          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2025-11-07</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
+          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Política pública</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -4766,24 +4766,24 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
+          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2025-10-16</t>
+          <t>2025-11-13</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
+          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -4798,7 +4798,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4813,24 +4813,24 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
+          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2025-10-09</t>
+          <t>2025-11-07</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
+          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4845,7 +4845,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -4860,24 +4860,24 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
+          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2025-09-23</t>
+          <t>2025-10-16</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
+          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4907,24 +4907,24 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2025-09-19</t>
+          <t>2025-10-09</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
+          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4954,24 +4954,24 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
+          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2025-09-13</t>
+          <t>2025-09-23</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
+          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -5001,24 +5001,24 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2025-09-19</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -5048,24 +5048,24 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2025-09-09</t>
+          <t>2025-09-13</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -5095,57 +5095,151 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2025-09-09</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
           <t>2025-09-06</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="B107" t="inlineStr">
         <is>
           <t>El Frailejón abre sus puertas: Usme estrena nueva Casa de la Juventud</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
+      <c r="C107" t="inlineStr">
         <is>
           <t>SDIS - Juventud</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr">
+      <c r="D107" t="inlineStr">
         <is>
           <t>institucional</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
+      <c r="E107" t="inlineStr">
         <is>
           <t>Otra</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr">
+      <c r="F107" t="inlineStr">
         <is>
           <t>Bogotá</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr">
+      <c r="G107" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr">
+      <c r="H107" t="inlineStr">
         <is>
           <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c7eca5d4bd</t>
         </is>
       </c>
-      <c r="I105" t="inlineStr">
+      <c r="I107" t="inlineStr">
         <is>
           <t>• Aunque ya existía una Casa de la Juventud en Usme, la sede se traslada y reinaugura para ofrecer mejores condiciones, ampliar servicios y fortalecer la atención a los jóvenes. • La reapertura se desarrolló con el acompañamiento de la Plataforma...</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-03-18
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I107"/>
+  <dimension ref="A1:I110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,32 +478,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Estudiantes de un colegio en La Ceja, Antioquia, impidieron la construcción de un hospital sobre un humedal</t>
+          <t>Por explotación sexual, capturaron a estadounidense en hotel del norte de Barranquilla</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -513,34 +513,34 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/estudiantes-de-un-colegio-en-la-ceja-antioquia-impidieron-la-construccion-de-un-hospital-sobre-un-humedal/</t>
+          <t>https://www.elespectador.com/colombia/barranquilla/por-explotacion-sexual-capturaron-a-estadounidense-en-hotel-del-norte-de-barranquilla/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Estudiantes y docentes del Bernardo Uribe Londoño marchan en defensa de su humedal. Un conflicto entre la salud y el equilibrio ambiental sacude a La CejaEl artículoEstudiantes de un colegio en La Ceja, Antioquia, impidieron la construcción de un...</t>
+          <t>Las autoridades capturaron a un extranjero y a una joven de 19 años por explotación sexual de menor de edad y proxenetismo.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Mafe Carrascal explicó por qué la bancada del Pacto Histórico por Bogotá no asistió a encuentro con el alcalde Carlos Fernando Galán</t>
+          <t>Adolescente de 14 años murió en riña entre menores de edad fuera de un colegio en Cali</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -550,39 +550,39 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/17/mafe-carrascal-explico-por-que-la-bancada-del-pacto-historico-por-bogota-no-asistio-a-encuentro-con-el-alcalde-carlos-fernando-galan/</t>
+          <t>https://www.elespectador.com/colombia/cali/adolescente-de-14-anos-murio-en-rina-entre-menores-de-edad-fuera-de-un-colegio-en-cali/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>La representante indicó que la reunión se realizaría a puerta cerrada y que esta decisión contradice los intereses de su partido. Además, afirmó que al gobierno local le falta implementar políticas dirigidas a los jóvenes y a la prevención de...</t>
+          <t>Adolescente de 14 años murió en riña entre menores afuera de un colegio en Cali. ¿Qué dicen las autoridades?</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Joven de 29 años ignoró síntomas creyendo que era TDAH, pero un accidente reveló un cáncer cerebral: 'Solo pedía llegar a los 30'</t>
+          <t>Colombia tendrá más viejos que jóvenes a partir de esta fecha; hay alerta por las pensiones</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -607,91 +607,87 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Cuando los médicos le informaron del hallazgo en su cerebro, Lauren aseguró que muchas piezas encajaron de repente. "Fue casi un alivio", señaló.</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/economia/colombia-tendra-mas-viejos-que-jovenes-partir-esta-fecha-hay-alerta-PP5100998A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Asesinan a joven de 15 años en Cartagena; su padre resultó herido al intentar defenderlo</t>
+          <t>Mafe Carrascal explicó por qué la bancada del Pacto Histórico por Bogotá no asistió a encuentro con el alcalde Carlos Fernando Galán</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/asesinan-a-menor-de-15-anos-en-cartagena-su-padre-resulto-herido-al-intentar-defenderlo/</t>
+          <t>https://www.infobae.com/colombia/2026/03/17/mafe-carrascal-explico-por-que-la-bancada-del-pacto-historico-por-bogota-no-asistio-a-encuentro-con-el-alcalde-carlos-fernando-galan/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>El presunto homicida ya fue localizado y detenido.</t>
+          <t>La representante indicó que la reunión se realizaría a puerta cerrada y que esta decisión contradice los intereses de su partido. Además, afirmó que al gobierno local le falta implementar políticas dirigidas a los jóvenes y a la prevención de...</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dos jóvenes fueron detenidos por presunta extorsión en Santo Tomás, Atlántico</t>
+          <t>Estudiantes de un colegio en La Ceja, Antioquia, impidieron la construcción de un hospital sobre un humedal</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -701,44 +697,44 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/dos-jovenes-fueron-detenidos-por-presunta-extorsion-en-santo-tomas-atlantico/</t>
+          <t>https://www.las2orillas.co/estudiantes-de-un-colegio-en-la-ceja-antioquia-impidieron-la-construccion-de-un-hospital-sobre-un-humedal/</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>La investigación señala que los implicados habrían intimidado a un conductor de furgón.</t>
+          <t>Estudiantes y docentes del Bernardo Uribe Londoño marchan en defensa de su humedal. Un conflicto entre la salud y el equilibrio ambiental sacude a La CejaEl artículoEstudiantes de un colegio en La Ceja, Antioquia, impidieron la construcción de un...</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Compensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo lograron?</t>
+          <t>Asesinan a joven de 15 años en Cartagena; su padre resultó herido al intentar defenderlo</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -748,34 +744,34 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/compensar-firmo-un-sorprendente-acuerdo-con-una-de-las-mejores-ligas-de-futbol-del-mundo-quienes-lo-lograron/</t>
+          <t>https://www.elespectador.com/colombia/asesinan-a-menor-de-15-anos-en-cartagena-su-padre-resulto-herido-al-intentar-defenderlo/</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>La Liga española acepto hacer una alianza con la solida caja de copensacion familiar para fortalecer la formación de jóvenes talentosEl artículoCompensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo...</t>
+          <t>El presunto homicida ya fue localizado y detenido.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hallan el cuerpo de una adolescente en vivienda de Sahagún, Córdoba; autoridades investigan</t>
+          <t>Joven de 29 años ignoró síntomas creyendo que era TDAH, pero un accidente reveló un cáncer cerebral: 'Solo pedía llegar a los 30'</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -795,44 +791,44 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/hallan-el-cuerpo-de-una-menor-en-una-vivienda-de-sahagun-cordoba-autoridades-investigan/</t>
+          <t>https://www.diarioadn.co/seccion/vida</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>En lo que va de este año, este sería el tercer caso de una mujer asesinada en el municipio y el cuarto en el departamento.</t>
+          <t>Cuando los médicos le informaron del hallazgo en su cerebro, Lauren aseguró que muchas piezas encajaron de repente. "Fue casi un alivio", señaló.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Con $86 mil millones de regalías, Bolívar construirá universidad en Montes de María y otros dos proyectos educativos</t>
+          <t>Hallan el cuerpo de una adolescente en vivienda de Sahagún, Córdoba; autoridades investigan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -842,44 +838,44 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/con-86-mil-millones-de-regalias-bolivar-construira-universidad-en-montes-de-maria-y-otros-dos-proyectos-educativos/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/hallan-el-cuerpo-de-una-menor-en-una-vivienda-de-sahagun-cordoba-autoridades-investigan/</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Los proyectos impulsados por Yamil Arana buscan, entre otras cosas, abrir más de 4 mil cupos para jóvenes de una región que durante años fue escenario de conflictoEl artículoCon $86 mil millones de regalías, Bolívar construirá universidad en Montes...</t>
+          <t>En lo que va de este año, este sería el tercer caso de una mujer asesinada en el municipio y el cuarto en el departamento.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Murió el influencer colombiano Alejo Little a los 33 años: estos fueron los quebrantos de salud que presentó en los últimos meses</t>
+          <t>Dos jóvenes fueron detenidos por presunta extorsión en Santo Tomás, Atlántico</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -889,24 +885,24 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/14/murio-el-influencer-colombiano-alejo-little-a-los-33-anos-estos-fueron-los-quebrantos-de-salud-que-presento-en-los-ultimos-meses/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/dos-jovenes-fueron-detenidos-por-presunta-extorsion-en-santo-tomas-atlantico/</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>El creador de contenido compartió experiencias sobre el acoso escolar y promovió la aceptación personal a través de sus redes sociales y charlas en instituciones educativas</t>
+          <t>La investigación señala que los implicados habrían intimidado a un conductor de furgón.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Los therian: un fenómeno que alarma</t>
+          <t>Compensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo lograron?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -921,7 +917,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -936,12 +932,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/los-therian-un-fenomeno-que-alarma/</t>
+          <t>https://www.las2orillas.co/compensar-firmo-un-sorprendente-acuerdo-con-una-de-las-mejores-ligas-de-futbol-del-mundo-quienes-lo-lograron/</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Cuando la identificación con un animal es persistente. se recomienda orientación psicológica para ayudar al joven en el desarrollo de una identidad saludableEl artículoLos therian: un fenómeno que alarmafue publicado originalmente enLas2orillas.co:...</t>
+          <t>La Liga española acepto hacer una alianza con la solida caja de copensacion familiar para fortalecer la formación de jóvenes talentosEl artículoCompensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo...</t>
         </is>
       </c>
     </row>
@@ -995,12 +991,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Figura de Independiente Medellín dedicó su gol en la clasificación del equipo en la Copa Libertadores a una persona que “está en tratamiento”</t>
+          <t>Murió el influencer colombiano Alejo Little a los 33 años: estos fueron los quebrantos de salud que presentó en los últimos meses</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1015,12 +1011,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1030,34 +1026,34 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/13/figura-de-independiente-medellin-dedico-su-gol-en-la-clasificacion-del-equipo-en-la-copa-libertadores-a-una-persona-que-esta-en-tratamiento/</t>
+          <t>https://www.infobae.com/colombia/2026/03/14/murio-el-influencer-colombiano-alejo-little-a-los-33-anos-estos-fueron-los-quebrantos-de-salud-que-presento-en-los-ultimos-meses/</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>El equipo dirigido por Alejandro Restrepo venció 2-1 a Juventud de Uruguay ante 12.000 hinchas y clasificó a la fase de grupos, donde acompañará a Deportes Tolima, Junior y Santa Fe en el torneo continental</t>
+          <t>El creador de contenido compartió experiencias sobre el acoso escolar y promovió la aceptación personal a través de sus redes sociales y charlas en instituciones educativas</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abren 200 becas para jóvenes del Pacífico que lideren proyectos en sus territorios</t>
+          <t>Con $86 mil millones de regalías, Bolívar construirá universidad en Montes de María y otros dos proyectos educativos</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1067,7 +1063,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1077,24 +1073,24 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/abren-200-becas-para-jovenes-del-pacifico-que-lideren-proyectos-en-sus-territorios/</t>
+          <t>https://www.las2orillas.co/con-86-mil-millones-de-regalias-bolivar-construira-universidad-en-montes-de-maria-y-otros-dos-proyectos-educativos/</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>El programa DALE lidera Pacífico ofrecerá formación, mentorías y acompañamiento a jóvenes que impulsen iniciativas comunitarias en litoral.</t>
+          <t>Los proyectos impulsados por Yamil Arana buscan, entre otras cosas, abrir más de 4 mil cupos para jóvenes de una región que durante años fue escenario de conflictoEl artículoCon $86 mil millones de regalías, Bolívar construirá universidad en Montes...</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>La travesía del gigante telescopio que Rodolfo Llinás le regaló al histórico Observatorio de la Universidad Nacional</t>
+          <t>Los therian: un fenómeno que alarma</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1109,7 +1105,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1124,29 +1120,29 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-travesia-del-gigante-telescopio-que-rodolfo-llinas-le-regalo-al-historico-observatorio-de-la-universidad-nacional/</t>
+          <t>https://www.las2orillas.co/los-therian-un-fenomeno-que-alarma/</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>En medio del paro de la Nacional, el cientifico donó su telescopio personal, el más grande instalado en Colombia, ahora al servicio de estudiantes e investigadoresEl artículoLa travesía del gigante telescopio que Rodolfo Llinás le regaló al...</t>
+          <t>Cuando la identificación con un animal es persistente. se recomienda orientación psicológica para ayudar al joven en el desarrollo de una identidad saludableEl artículoLos therian: un fenómeno que alarmafue publicado originalmente enLas2orillas.co:...</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
+          <t>Figura de Independiente Medellín dedicó su gol en la clasificación del equipo en la Copa Libertadores a una persona que “está en tratamiento”</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1161,7 +1157,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1171,30 +1167,34 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/13/figura-de-independiente-medellin-dedico-su-gol-en-la-clasificacion-del-equipo-en-la-copa-libertadores-a-una-persona-que-esta-en-tratamiento/</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>El equipo dirigido por Alejandro Restrepo venció 2-1 a Juventud de Uruguay ante 12.000 hinchas y clasificó a la fase de grupos, donde acompañará a Deportes Tolima, Junior y Santa Fe en el torneo continental</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Estudiantes de colegios públicos en Bogotá que tendrían que reponer clase el sábado</t>
+          <t>Abren 200 becas para jóvenes del Pacífico que lideren proyectos en sus territorios</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1204,20 +1204,24 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/estudiantes-colegios-publicos-bogota-que-tendrian-que-reponer-clase-PP5091931A</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abren-200-becas-para-jovenes-del-pacifico-que-lideren-proyectos-en-sus-territorios/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>El programa DALE lidera Pacífico ofrecerá formación, mentorías y acompañamiento a jóvenes que impulsen iniciativas comunitarias en litoral.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1227,7 +1231,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
+          <t>Estudiantes de colegios públicos en Bogotá que tendrían que reponer clase el sábado</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1247,17 +1251,17 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
+          <t>https://www.pulzo.com/nacion/bogota/estudiantes-colegios-publicos-bogota-que-tendrian-que-reponer-clase-PP5091931A</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -1270,12 +1274,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
+          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1290,7 +1294,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1300,24 +1304,20 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
+          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1332,12 +1332,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1347,108 +1347,104 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
+          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
+          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
+          <t>La travesía del gigante telescopio que Rodolfo Llinás le regaló al histórico Observatorio de la Universidad Nacional</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
+          <t>https://www.las2orillas.co/la-travesia-del-gigante-telescopio-que-rodolfo-llinas-le-regalo-al-historico-observatorio-de-la-universidad-nacional/</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
+          <t>En medio del paro de la Nacional, el cientifico donó su telescopio personal, el más grande instalado en Colombia, ahora al servicio de estudiantes e investigadoresEl artículoLa travesía del gigante telescopio que Rodolfo Llinás le regaló al...</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
+          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1458,17 +1454,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Prosperidad Social inicia entrega de transferencia monetaria de Jóvenes en Paz</t>
+          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1478,22 +1474,22 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Valledupar</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-inicia-entrega-de-transferencia-monetaria-de-jovenes-en-paz/</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Esta transferencia corresponde al ciclo 1 de 2026. Más de 12.000 jóvenes en el país recibirán los recursos. Bogotá D. C., 24 de febrero de 2026. Prosperidad Social realizará este 27 de febrero la transferencia monetaria condicionada para los...</t>
+          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
         </is>
       </c>
     </row>
@@ -1505,42 +1501,42 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
+          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
+          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
         </is>
       </c>
     </row>
@@ -1552,12 +1548,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
+          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1572,22 +1568,22 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
+          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
+          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
         </is>
       </c>
     </row>
@@ -1599,12 +1595,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
+          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1619,22 +1615,22 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
+          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1642,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
+          <t>Prosperidad Social inicia entrega de transferencia monetaria de Jóvenes en Paz</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1676,12 +1672,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-inicia-entrega-de-transferencia-monetaria-de-jovenes-en-paz/</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
+          <t>Esta transferencia corresponde al ciclo 1 de 2026. Más de 12.000 jóvenes en el país recibirán los recursos. Bogotá D. C., 24 de febrero de 2026. Prosperidad Social realizará este 27 de febrero la transferencia monetaria condicionada para los...</t>
         </is>
       </c>
     </row>
@@ -1693,17 +1689,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
+          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1713,39 +1709,39 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Valledupar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
+          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
+          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1755,7 +1751,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1770,118 +1766,118 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
+          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
+          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
+          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
+          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
+          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
+          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
+          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1896,7 +1892,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1911,34 +1907,34 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
+          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
+          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1958,128 +1954,128 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
+          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
+          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/cultura</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
+          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
+          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
+          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
+          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2089,7 +2085,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2099,35 +2095,39 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
+          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2142,29 +2142,29 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
+          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2174,12 +2174,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2189,24 +2189,24 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
+          <t>https://www.diarioadn.co/seccion/cultura</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
+          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
+          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2221,12 +2221,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -2244,45 +2244,49 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
+          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2339,37 +2343,37 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
+          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -2467,59 +2471,59 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
+          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
+          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
+          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2534,22 +2538,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -2557,17 +2561,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2577,7 +2581,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2592,7 +2596,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
+          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -2600,27 +2604,27 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
+          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2635,20 +2639,24 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2663,22 +2671,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -2686,12 +2694,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2706,22 +2714,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -2729,22 +2737,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
+          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2764,29 +2772,25 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
+          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2801,7 +2805,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2811,7 +2815,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -2819,17 +2823,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
+          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2839,12 +2843,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2854,14 +2858,10 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/inicio</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2871,12 +2871,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
+          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -2909,17 +2909,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
+          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2944,20 +2944,24 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/inicio</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
+          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2972,22 +2976,22 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -2995,22 +2999,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
+          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3030,20 +3034,24 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
+          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3073,7 +3081,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -3081,17 +3089,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3101,22 +3109,22 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -3124,12 +3132,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3149,7 +3157,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3159,7 +3167,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
+          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -3167,12 +3175,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Estados Unidos hizo llamado de atención a Colombia ante la ONU por aumento de reclutamiento de menores de edad:“Dudas sobre impunidad al terrorismo” - Infobae</t>
+          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3187,22 +3195,22 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgJBVV95cUxNNFJLRzNtTGZtU1ZCaVUxbGR1QUhBMzV5eFVUT2w4TWZVZnNfYmNMX1IydEVyYnhGT3ZJcDZMaG85R0RUUU9LaEsxT0hyYTFEcy1lNmVTMTA4TWlTbzJ2NmJNbTdxTXZQeUVsczJGMTdSZVlYVHlwblhqeG53UzZ5QkhsMVFyTWRORUQtOUNJMXFBSzJiNkZGQjJSZ1lvcWdfUHFTN1duQjJvcWVyMEZIZE01OGMyakhIQk5WbkROZlpIaDg5UHJRLWdEWVVSRlN4N21hNlhvemlncnlCZlNsM1BvYlJrX2hnUEpmREFCT1pzWS14YmtLMzNHWk1ndnN1NVE5YUdaajNmelBLZEViNEFHNHdjbFhqZEHSAbQCQVVfeXFMTXBsTHJ3d1N1RXh4WFdBdjAtMVFYcEJTV2xwd0xHZERGQVlHNXNvcW5hYmdpN09Wd1ljMjR4RjNSRWMxMl8xMmN5TzN2XzQzUDhCdlJ2WjdNSklzMG1yRzI5YnRnRDFhYWo3Wi1wOEdNbHE4UElzU2FGN3Z2b29XX0Z0bXBDczQzbE1oRE9zVjk1VG9OMzZSNlhsbjlFZUp4em84bGxJSTJyRG8yOWlvUkxPZkhVT0picHVCXzRRX2dhY1VTTWlJcUFYRnVBQzV0ck10YkktYXVpSE5uNm40U1lneGt5c0p5VUNzYnl0NEpqWmVLUE5UcWxOT1BJbnFDZmJRSG9XaTYyMXhqT3dhekhSUDBLSnh6dGxBNFNNYzktYTdZMmxmZm13bXhDd2x3Y0tvWkM?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -3210,32 +3218,32 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Estados Unidos reclama a Colombia ante ONU el incremento de reclutamiento de menores de edad - El Espectador</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3245,7 +3253,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxPVFRDQXk2WVcwQVhLTmljT1B4akFGM3ozQlBvc3QyOHJua1BfT1hxRnFJY212eFowWTVTdVBmTHN6d2REcXc5VGVuUmw1LWsxNWxOeW82UzBPaVQ3azZfQVNSb0pUTHFqTHdGVWJXS2Z5YmVSbXZJSXd4dzdTamNXdUtqMTRwVDV4MF9acHJFX1pTZ19NVVNvLWdNb1Y1d0FzZlN2dWVMamlvVlNCN01ZS2MxZDh1M250d2tsNEVpc2NYRUJXcE9KYk0yd1FHU3BiNUtFOENRdWZ4ZHdsR0l2cFRFMEpKTGYtaUk4dmhuRjhyaVU3RDYxbUpCUzjSAZACQVVfeXFMTmxJSVphakhMc1dSdUhqdDJFZW00OTIwT0NRNndiZGNtLWROVW1NZFFHWHhTMzVYb3N6aHRBV1NObF94cEVSeHZMOWpPTW1oVXdGeDloRU9uSWpIUXNldU1qY2lUM3dNWnhwMUNESWVTUy1SNGYzZkM0Nk1ORE9zQkNkdzc1MnJpUldVTnhKeUsycE1rcGdwMi1SN3F4bkZUdHZGNUJWT1RLeS1ZMFJUVkdmOXpHcnpId0N2QW9oOEVsbkYyVU9xbUtnTEVBdW1kNnlOY2wwVGVUY1dCc3N5WkQ5ZTBRUTFKSndYUU4zYVU2aUc1cUlsLUt4d3B6OTZ4Xzl0cC0tMFAwQ0hwM2JWUC0?oc=5</t>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -3253,12 +3261,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3288,7 +3296,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -3296,12 +3304,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Estados Unidos hizo llamado de atención a Colombia ante la ONU por aumento de reclutamiento de menores de edad:“Dudas sobre impunidad al terrorismo” - Infobae</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3316,7 +3324,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3331,7 +3339,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://news.google.com/rss/articles/CBMimgJBVV95cUxNNFJLRzNtTGZtU1ZCaVUxbGR1QUhBMzV5eFVUT2w4TWZVZnNfYmNMX1IydEVyYnhGT3ZJcDZMaG85R0RUUU9LaEsxT0hyYTFEcy1lNmVTMTA4TWlTbzJ2NmJNbTdxTXZQeUVsczJGMTdSZVlYVHlwblhqeG53UzZ5QkhsMVFyTWRORUQtOUNJMXFBSzJiNkZGQjJSZ1lvcWdfUHFTN1duQjJvcWVyMEZIZE01OGMyakhIQk5WbkROZlpIaDg5UHJRLWdEWVVSRlN4N21hNlhvemlncnlCZlNsM1BvYlJrX2hnUEpmREFCT1pzWS14YmtLMzNHWk1ndnN1NVE5YUdaajNmelBLZEViNEFHNHdjbFhqZEHSAbQCQVVfeXFMTXBsTHJ3d1N1RXh4WFdBdjAtMVFYcEJTV2xwd0xHZERGQVlHNXNvcW5hYmdpN09Wd1ljMjR4RjNSRWMxMl8xMmN5TzN2XzQzUDhCdlJ2WjdNSklzMG1yRzI5YnRnRDFhYWo3Wi1wOEdNbHE4UElzU2FGN3Z2b29XX0Z0bXBDczQzbE1oRE9zVjk1VG9OMzZSNlhsbjlFZUp4em84bGxJSTJyRG8yOWlvUkxPZkhVT0picHVCXzRRX2dhY1VTTWlJcUFYRnVBQzV0ck10YkktYXVpSE5uNm40U1lneGt5c0p5VUNzYnl0NEpqWmVLUE5UcWxOT1BJbnFDZmJRSG9XaTYyMXhqT3dhekhSUDBLSnh6dGxBNFNNYzktYTdZMmxmZm13bXhDd2x3Y0tvWkM?oc=5</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -3339,32 +3347,32 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>Estados Unidos reclama a Colombia ante ONU el incremento de reclutamiento de menores de edad - El Espectador</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3374,7 +3382,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxPVFRDQXk2WVcwQVhLTmljT1B4akFGM3ozQlBvc3QyOHJua1BfT1hxRnFJY212eFowWTVTdVBmTHN6d2REcXc5VGVuUmw1LWsxNWxOeW82UzBPaVQ3azZfQVNSb0pUTHFqTHdGVWJXS2Z5YmVSbXZJSXd4dzdTamNXdUtqMTRwVDV4MF9acHJFX1pTZ19NVVNvLWdNb1Y1d0FzZlN2dWVMamlvVlNCN01ZS2MxZDh1M250d2tsNEVpc2NYRUJXcE9KYk0yd1FHU3BiNUtFOENRdWZ4ZHdsR0l2cFRFMEpKTGYtaUk4dmhuRjhyaVU3RDYxbUpCUzjSAZACQVVfeXFMTmxJSVphakhMc1dSdUhqdDJFZW00OTIwT0NRNndiZGNtLWROVW1NZFFHWHhTMzVYb3N6aHRBV1NObF94cEVSeHZMOWpPTW1oVXdGeDloRU9uSWpIUXNldU1qY2lUM3dNWnhwMUNESWVTUy1SNGYzZkM0Nk1ORE9zQkNkdzc1MnJpUldVTnhKeUsycE1rcGdwMi1SN3F4bkZUdHZGNUJWT1RLeS1ZMFJUVkdmOXpHcnpId0N2QW9oOEVsbkYyVU9xbUtnTEVBdW1kNnlOY2wwVGVUY1dCc3N5WkQ5ZTBRUTFKSndYUU4zYVU2aUc1cUlsLUt4d3B6OTZ4Xzl0cC0tMFAwQ0hwM2JWUC0?oc=5</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -3382,12 +3390,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3402,7 +3410,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3417,7 +3425,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -3425,12 +3433,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>En el regreso a clases, el sueño insuficiente en adolescentes duplica el riesgo de problemas de atención y conducta - Infobae</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3450,7 +3458,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3460,7 +3468,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNTjNaNDNPUHFZYzdoUlNIaUJZbGlqb2JPZndHd3Rad0F4VGwtRHFFQXdzaEIzRWN3bndOTjhsa0JReEtYS1B3TWN5ZVhaRG1RZGtxTkVDVVI2TWV0aTFxTC1KZUJfT2NDZEpIc0tLckJjMmhEOHZvZjVHaEhGRDB2c2NxSmw5SUJpVi0tUlVaZDI1cDgyY1p5QzVRMTlMQ0NOMlkxNGlad243SzF0TFJXZ3RNRGtRY0xtSW5VSnNZaHZCYUJWWG83RzBEZEY4dUFZYUxtLTlqVGx0bWVjbk9vMzFBS0o2LUlyTXNLb3M3ZzbSAYsCQVVfeXFMTTZoYWJjUTZubmFSQjVXNzlCZkdxTkhLby1HTG1iUmdWVVNSMGZpM3EwNkd3U3NSaVhDZWJJeHpQcC1KbUlUWjhFMERwZVBmRXM5NnJVNFQ2RmFDZmNSaXlkOG5tYWhlZlFydUw5X0xVZGkxWmVIM0tuVmd4eHBOMF9SSExuc2tzQ2stNU9kdjlCemxvZTV4MUlVbElWT3dmYmVSYXE0c0VUQTRUTGtYVDZ1SmRKU0R6Z3ZlTEExQmVMa0RDRHl2ZVlvUmVTQWl3aVJJM3hrQU5rMlpLVUYzOUNjOVBDZmVzdWtoeFdqT3JLaUdGY2JOaUw0MnJyQXVNMTQ4Wl9JNHBaYjdv?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -3468,12 +3476,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3488,7 +3496,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3503,7 +3511,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -3511,12 +3519,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3536,17 +3544,17 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -3554,27 +3562,27 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
+          <t>En el regreso a clases, el sueño insuficiente en adolescentes duplica el riesgo de problemas de atención y conducta - Infobae</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3589,7 +3597,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNTjNaNDNPUHFZYzdoUlNIaUJZbGlqb2JPZndHd3Rad0F4VGwtRHFFQXdzaEIzRWN3bndOTjhsa0JReEtYS1B3TWN5ZVhaRG1RZGtxTkVDVVI2TWV0aTFxTC1KZUJfT2NDZEpIc0tLckJjMmhEOHZvZjVHaEhGRDB2c2NxSmw5SUJpVi0tUlVaZDI1cDgyY1p5QzVRMTlMQ0NOMlkxNGlad243SzF0TFJXZ3RNRGtRY0xtSW5VSnNZaHZCYUJWWG83RzBEZEY4dUFZYUxtLTlqVGx0bWVjbk9vMzFBS0o2LUlyTXNLb3M3ZzbSAYsCQVVfeXFMTTZoYWJjUTZubmFSQjVXNzlCZkdxTkhLby1HTG1iUmdWVVNSMGZpM3EwNkd3U3NSaVhDZWJJeHpQcC1KbUlUWjhFMERwZVBmRXM5NnJVNFQ2RmFDZmNSaXlkOG5tYWhlZlFydUw5X0xVZGkxWmVIM0tuVmd4eHBOMF9SSExuc2tzQ2stNU9kdjlCemxvZTV4MUlVbElWT3dmYmVSYXE0c0VUQTRUTGtYVDZ1SmRKU0R6Z3ZlTEExQmVMa0RDRHl2ZVlvUmVTQWl3aVJJM3hrQU5rMlpLVUYzOUNjOVBDZmVzdWtoeFdqT3JLaUdGY2JOaUw0MnJyQXVNMTQ4Wl9JNHBaYjdv?oc=5</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -3597,12 +3605,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3617,12 +3625,12 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3632,7 +3640,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
@@ -3640,27 +3648,27 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Casas de Juventud lanzan nuevos Semilleros Distritales para potenciar el talento juvenil en Bogotá</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3675,39 +3683,35 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#f8686f5026</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>•Bogotá abre la convocatoria a semilleros gratuitos en artes, deporte y cultura urbana, dirigidos a jóvenes entre 14 y 28 años de todas las localidades, como una estrategia distrital para fortalecer la expresión, la participación y el desarrollo de...</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
+          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3722,14 +3726,10 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/regiones</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3739,40 +3739,44 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Corte Constitucional fijó nuevos criterios para el manejo de conflictos escolares entre menores de edad - Infobae</t>
+          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOOVhMdnBkeXFCaTNlNTNGX2ZaTGxqVnB0b2FIZ0owQTl3LXFiUldIQ2FhOFJZeGdEa3FJTjRoMkxuTHFYNFFBTTVMakFUY0tob051TWxCOVluajg1d24tdWRxM256TTFndk9FSUQ5b2FpNGY3U3ZxQ00za1JhYThoamVHUnBRVUdySkNHNzFhU1JFQ0JsLVJ1N0ZZLU1EdE5tcUViVXluc2hTWm0zblFKcWxXdW9mVDZic1FTWXpyS1NLTWNaZmlEMXZ1T0xoYVR4U2xwZjVycEtkOE1EQlBYLUtn0gH8AUFVX3lxTFB1aVQ2NGIzQ0hhVm54dGlrb0Q4WWtXUVFrdVA0N2dyVEMzWXN3T1p1QmlVZm4wQzdXZmJnZU5TcjlLSFFGTEZwODlYU0FmTU5ra0wtOEhuUWJVMWh5eXlqVEg2WGhHM2tMOVZwMkxTM25vZUFtRHA0S3JjQ1l3RElwVE8wWjRZSWhCcE5Ib1gwWXVpZ09TM2dvOVc5bzBFbFRWdmtYNUZSTzR3T1VrU1I1V25nLWlDSWsxRVJWUmczUFo2Z2lQNTBhOTR4MzhKZDc4YjJxSXJoaU5OU016NGdDX3JtTXp4dVNBTXozV09XSUhRaTJ0ckJvMS00Vw?oc=5</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3782,59 +3786,55 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
+          <t>Corte Constitucional fijó nuevos criterios para el manejo de conflictos escolares entre menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOOVhMdnBkeXFCaTNlNTNGX2ZaTGxqVnB0b2FIZ0owQTl3LXFiUldIQ2FhOFJZeGdEa3FJTjRoMkxuTHFYNFFBTTVMakFUY0tob051TWxCOVluajg1d24tdWRxM256TTFndk9FSUQ5b2FpNGY3U3ZxQ00za1JhYThoamVHUnBRVUdySkNHNzFhU1JFQ0JsLVJ1N0ZZLU1EdE5tcUViVXluc2hTWm0zblFKcWxXdW9mVDZic1FTWXpyS1NLTWNaZmlEMXZ1T0xoYVR4U2xwZjVycEtkOE1EQlBYLUtn0gH8AUFVX3lxTFB1aVQ2NGIzQ0hhVm54dGlrb0Q4WWtXUVFrdVA0N2dyVEMzWXN3T1p1QmlVZm4wQzdXZmJnZU5TcjlLSFFGTEZwODlYU0FmTU5ra0wtOEhuUWJVMWh5eXlqVEg2WGhHM2tMOVZwMkxTM25vZUFtRHA0S3JjQ1l3RElwVE8wWjRZSWhCcE5Ib1gwWXVpZ09TM2dvOVc5bzBFbFRWdmtYNUZSTzR3T1VrU1I1V25nLWlDSWsxRVJWUmczUFo2Z2lQNTBhOTR4MzhKZDc4YjJxSXJoaU5OU016NGdDX3JtTXp4dVNBTXozV09XSUhRaTJ0ckJvMS00Vw?oc=5</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Yumbo se pone la camiseta del futuro: lanza Aulas STEAM con inversión histórica de $ 9.500 millones</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3849,73 +3849,81 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/regiones</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Iniciativa busca impactar a más de 10.400 estudiantes</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Casas de Juventud lanzan nuevos Semilleros Distritales para potenciar el talento juvenil en Bogotá</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#f8686f5026</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>•Bogotá abre la convocatoria a semilleros gratuitos en artes, deporte y cultura urbana, dirigidos a jóvenes entre 14 y 28 años de todas las localidades, como una estrategia distrital para fortalecer la expresión, la participación y el desarrollo de...</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
+          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3930,7 +3938,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3945,7 +3953,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -3953,12 +3961,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3973,22 +3981,22 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -3996,12 +4004,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4031,7 +4039,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -4044,7 +4052,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4059,7 +4067,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -4074,7 +4082,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -4087,7 +4095,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4102,22 +4110,22 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
         </is>
       </c>
       <c r="I82" t="inlineStr"/>
@@ -4125,17 +4133,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -4150,17 +4158,17 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
@@ -4168,17 +4176,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4188,12 +4196,12 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -4203,24 +4211,20 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4240,17 +4244,17 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -4258,12 +4262,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4278,12 +4282,12 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Barranquilla</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4293,7 +4297,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
@@ -4301,27 +4305,27 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -4336,50 +4340,54 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
+          <t>https://www.alertabogota.com/noticias/local</t>
         </is>
       </c>
       <c r="I88" t="inlineStr"/>
@@ -4387,12 +4395,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
+          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -4407,12 +4415,12 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4422,7 +4430,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
@@ -4430,27 +4438,27 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
+          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -4465,7 +4473,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -4473,32 +4481,32 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
+          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -4508,7 +4516,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
         </is>
       </c>
       <c r="I91" t="inlineStr"/>
@@ -4516,32 +4524,32 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
+          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -4551,7 +4559,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
@@ -4559,17 +4567,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
+          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Noticias Caracol</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -4579,7 +4587,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -4594,7 +4602,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
         </is>
       </c>
       <c r="I93" t="inlineStr"/>
@@ -4602,12 +4610,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
+          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4637,7 +4645,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
         </is>
       </c>
       <c r="I94" t="inlineStr"/>
@@ -4645,42 +4653,42 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
+          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
         </is>
       </c>
       <c r="I95" t="inlineStr"/>
@@ -4688,17 +4696,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
+          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Noticias Caracol</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -4708,12 +4716,12 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -4723,7 +4731,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
         </is>
       </c>
       <c r="I96" t="inlineStr"/>
@@ -4731,74 +4739,70 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
+          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Política pública</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
-        </is>
-      </c>
-      <c r="I97" t="inlineStr">
-        <is>
-          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2025-11-13</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
+          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4813,71 +4817,63 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
-        </is>
-      </c>
-      <c r="I98" t="inlineStr">
-        <is>
-          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2025-11-07</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
+          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2025-10-16</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
+          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4892,7 +4888,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Política pública</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -4907,24 +4903,24 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
+          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2025-10-09</t>
+          <t>2025-11-13</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
+          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4939,7 +4935,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -4954,24 +4950,24 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
+          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2025-09-23</t>
+          <t>2025-11-07</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
+          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4986,7 +4982,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -5001,24 +4997,24 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
+          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2025-09-19</t>
+          <t>2025-10-16</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
+          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -5048,24 +5044,24 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2025-09-13</t>
+          <t>2025-10-09</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
+          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -5095,24 +5091,24 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
+          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2025-09-23</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -5127,7 +5123,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -5142,24 +5138,24 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2025-09-09</t>
+          <t>2025-09-19</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -5189,57 +5185,198 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2025-09-09</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
           <t>2025-09-06</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
+      <c r="B110" t="inlineStr">
         <is>
           <t>El Frailejón abre sus puertas: Usme estrena nueva Casa de la Juventud</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
+      <c r="C110" t="inlineStr">
         <is>
           <t>SDIS - Juventud</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr">
+      <c r="D110" t="inlineStr">
         <is>
           <t>institucional</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
+      <c r="E110" t="inlineStr">
         <is>
           <t>Otra</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr">
+      <c r="F110" t="inlineStr">
         <is>
           <t>Bogotá</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr">
+      <c r="G110" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr">
+      <c r="H110" t="inlineStr">
         <is>
           <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c7eca5d4bd</t>
         </is>
       </c>
-      <c r="I107" t="inlineStr">
+      <c r="I110" t="inlineStr">
         <is>
           <t>• Aunque ya existía una Casa de la Juventud en Usme, la sede se traslada y reinaugura para ofrecer mejores condiciones, ampliar servicios y fortalecer la atención a los jóvenes. • La reapertura se desarrolló con el acompañamiento de la Plataforma...</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-03-19
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I110"/>
+  <dimension ref="A1:I112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,12 +478,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Por explotación sexual, capturaron a estadounidense en hotel del norte de Barranquilla</t>
+          <t>Condenaron en Miami a hombre que viajó a Medellín a abusar sexualmente de una menor de edad</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -498,12 +498,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Barranquilla</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -513,61 +513,57 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/barranquilla/por-explotacion-sexual-capturaron-a-estadounidense-en-hotel-del-norte-de-barranquilla/</t>
+          <t>https://www.elespectador.com/colombia/medellin/condenaron-en-miami-a-hombre-que-viajo-a-medellin-a-abusar-sexualmente-de-una-menor-de-edad/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Las autoridades capturaron a un extranjero y a una joven de 19 años por explotación sexual de menor de edad y proxenetismo.</t>
+          <t>Declarado culpable en Miami hombre que viajó a Medellín a abusar sexualmente de una menor.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Adolescente de 14 años murió en riña entre menores de edad fuera de un colegio en Cali</t>
+          <t>Insólito pedido de familia de David Acosta luego de que el joven apareciera con vida en Bogotá</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/adolescente-de-14-anos-murio-en-rina-entre-menores-de-edad-fuera-de-un-colegio-en-cali/</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Adolescente de 14 años murió en riña entre menores afuera de un colegio en Cali. ¿Qué dicen las autoridades?</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/bogota/caso-david-acosta-familia-pide-cerrar-investigacion-falsa-desaparicion-PP5103111</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -577,27 +573,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Colombia tendrá más viejos que jóvenes a partir de esta fecha; hay alerta por las pensiones</t>
+          <t>Adolescente de 14 años murió en riña entre menores de edad fuera de un colegio en Cali</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -607,72 +603,76 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/economia/colombia-tendra-mas-viejos-que-jovenes-partir-esta-fecha-hay-alerta-PP5100998A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/cali/adolescente-de-14-anos-murio-en-rina-entre-menores-de-edad-fuera-de-un-colegio-en-cali/</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Adolescente de 14 años murió en riña entre menores afuera de un colegio en Cali. ¿Qué dicen las autoridades?</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mafe Carrascal explicó por qué la bancada del Pacto Histórico por Bogotá no asistió a encuentro con el alcalde Carlos Fernando Galán</t>
+          <t>Por explotación sexual, capturaron a estadounidense en hotel del norte de Barranquilla</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/17/mafe-carrascal-explico-por-que-la-bancada-del-pacto-historico-por-bogota-no-asistio-a-encuentro-con-el-alcalde-carlos-fernando-galan/</t>
+          <t>https://www.elespectador.com/colombia/barranquilla/por-explotacion-sexual-capturaron-a-estadounidense-en-hotel-del-norte-de-barranquilla/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>La representante indicó que la reunión se realizaría a puerta cerrada y que esta decisión contradice los intereses de su partido. Además, afirmó que al gobierno local le falta implementar políticas dirigidas a los jóvenes y a la prevención de...</t>
+          <t>Las autoridades capturaron a un extranjero y a una joven de 19 años por explotación sexual de menor de edad y proxenetismo.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Estudiantes de un colegio en La Ceja, Antioquia, impidieron la construcción de un hospital sobre un humedal</t>
+          <t>Colombia tendrá más viejos que jóvenes a partir de esta fecha; hay alerta por las pensiones</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -697,44 +697,40 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/estudiantes-de-un-colegio-en-la-ceja-antioquia-impidieron-la-construccion-de-un-hospital-sobre-un-humedal/</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Estudiantes y docentes del Bernardo Uribe Londoño marchan en defensa de su humedal. Un conflicto entre la salud y el equilibrio ambiental sacude a La CejaEl artículoEstudiantes de un colegio en La Ceja, Antioquia, impidieron la construcción de un...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/economia/colombia-tendra-mas-viejos-que-jovenes-partir-esta-fecha-hay-alerta-PP5100998A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Asesinan a joven de 15 años en Cartagena; su padre resultó herido al intentar defenderlo</t>
+          <t>Estudiantes de un colegio en La Ceja, Antioquia, impidieron la construcción de un hospital sobre un humedal</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -744,29 +740,29 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/asesinan-a-menor-de-15-anos-en-cartagena-su-padre-resulto-herido-al-intentar-defenderlo/</t>
+          <t>https://www.las2orillas.co/estudiantes-de-un-colegio-en-la-ceja-antioquia-impidieron-la-construccion-de-un-hospital-sobre-un-humedal/</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>El presunto homicida ya fue localizado y detenido.</t>
+          <t>Estudiantes y docentes del Bernardo Uribe Londoño marchan en defensa de su humedal. Un conflicto entre la salud y el equilibrio ambiental sacude a La CejaEl artículoEstudiantes de un colegio en La Ceja, Antioquia, impidieron la construcción de un...</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Joven de 29 años ignoró síntomas creyendo que era TDAH, pero un accidente reveló un cáncer cerebral: 'Solo pedía llegar a los 30'</t>
+          <t>Mafe Carrascal explicó por qué la bancada del Pacto Histórico por Bogotá no asistió a encuentro con el alcalde Carlos Fernando Galán</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -776,39 +772,39 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
+          <t>https://www.infobae.com/colombia/2026/03/17/mafe-carrascal-explico-por-que-la-bancada-del-pacto-historico-por-bogota-no-asistio-a-encuentro-con-el-alcalde-carlos-fernando-galan/</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Cuando los médicos le informaron del hallazgo en su cerebro, Lauren aseguró que muchas piezas encajaron de repente. "Fue casi un alivio", señaló.</t>
+          <t>La representante indicó que la reunión se realizaría a puerta cerrada y que esta decisión contradice los intereses de su partido. Además, afirmó que al gobierno local le falta implementar políticas dirigidas a los jóvenes y a la prevención de...</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Hallan el cuerpo de una adolescente en vivienda de Sahagún, Córdoba; autoridades investigan</t>
+          <t>Asesinan a joven de 15 años en Cartagena; su padre resultó herido al intentar defenderlo</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -823,12 +819,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -838,39 +834,39 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/hallan-el-cuerpo-de-una-menor-en-una-vivienda-de-sahagun-cordoba-autoridades-investigan/</t>
+          <t>https://www.elespectador.com/colombia/asesinan-a-menor-de-15-anos-en-cartagena-su-padre-resulto-herido-al-intentar-defenderlo/</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>En lo que va de este año, este sería el tercer caso de una mujer asesinada en el municipio y el cuarto en el departamento.</t>
+          <t>El presunto homicida ya fue localizado y detenido.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dos jóvenes fueron detenidos por presunta extorsión en Santo Tomás, Atlántico</t>
+          <t>Joven de 29 años ignoró síntomas creyendo que era TDAH, pero un accidente reveló un cáncer cerebral: 'Solo pedía llegar a los 30'</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -885,12 +881,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/dos-jovenes-fueron-detenidos-por-presunta-extorsion-en-santo-tomas-atlantico/</t>
+          <t>https://www.diarioadn.co/seccion/vida</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>La investigación señala que los implicados habrían intimidado a un conductor de furgón.</t>
+          <t>Cuando los médicos le informaron del hallazgo en su cerebro, Lauren aseguró que muchas piezas encajaron de repente. "Fue casi un alivio", señaló.</t>
         </is>
       </c>
     </row>
@@ -902,27 +898,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Compensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo lograron?</t>
+          <t>Dos jóvenes fueron detenidos por presunta extorsión en Santo Tomás, Atlántico</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -932,34 +928,34 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/compensar-firmo-un-sorprendente-acuerdo-con-una-de-las-mejores-ligas-de-futbol-del-mundo-quienes-lo-lograron/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/dos-jovenes-fueron-detenidos-por-presunta-extorsion-en-santo-tomas-atlantico/</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>La Liga española acepto hacer una alianza con la solida caja de copensacion familiar para fortalecer la formación de jóvenes talentosEl artículoCompensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo...</t>
+          <t>La investigación señala que los implicados habrían intimidado a un conductor de furgón.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pese a todo, la IA podría potenciar el criterio político de la juventud</t>
+          <t>Hallan el cuerpo de una adolescente en vivienda de Sahagún, Córdoba; autoridades investigan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -979,29 +975,29 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/red-de-expertos/red-de-democracia-y-tecnologia/pese-a-todo-la-ia-podria-potenciar-el-criterio-politico-de-la-juventud/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/hallan-el-cuerpo-de-una-menor-en-una-vivienda-de-sahagun-cordoba-autoridades-investigan/</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Aunque la IA genera inquietudes en el ámbito educativo, también puede formar la conciencia política e histórica entre la juventud.The postPese a todo, la IA podría potenciar el criterio político de la juventudappeared first onLa Silla Vacía.</t>
+          <t>En lo que va de este año, este sería el tercer caso de una mujer asesinada en el municipio y el cuarto en el departamento.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Murió el influencer colombiano Alejo Little a los 33 años: estos fueron los quebrantos de salud que presentó en los últimos meses</t>
+          <t>Compensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo lograron?</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1011,7 +1007,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1026,12 +1022,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/14/murio-el-influencer-colombiano-alejo-little-a-los-33-anos-estos-fueron-los-quebrantos-de-salud-que-presento-en-los-ultimos-meses/</t>
+          <t>https://www.las2orillas.co/compensar-firmo-un-sorprendente-acuerdo-con-una-de-las-mejores-ligas-de-futbol-del-mundo-quienes-lo-lograron/</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>El creador de contenido compartió experiencias sobre el acoso escolar y promovió la aceptación personal a través de sus redes sociales y charlas en instituciones educativas</t>
+          <t>La Liga española acepto hacer una alianza con la solida caja de copensacion familiar para fortalecer la formación de jóvenes talentosEl artículoCompensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo...</t>
         </is>
       </c>
     </row>
@@ -1043,12 +1039,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Con $86 mil millones de regalías, Bolívar construirá universidad en Montes de María y otros dos proyectos educativos</t>
+          <t>Pese a todo, la IA podría potenciar el criterio político de la juventud</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1058,12 +1054,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1073,12 +1069,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/con-86-mil-millones-de-regalias-bolivar-construira-universidad-en-montes-de-maria-y-otros-dos-proyectos-educativos/</t>
+          <t>https://www.lasillavacia.com/red-de-expertos/red-de-democracia-y-tecnologia/pese-a-todo-la-ia-podria-potenciar-el-criterio-politico-de-la-juventud/</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Los proyectos impulsados por Yamil Arana buscan, entre otras cosas, abrir más de 4 mil cupos para jóvenes de una región que durante años fue escenario de conflictoEl artículoCon $86 mil millones de regalías, Bolívar construirá universidad en Montes...</t>
+          <t>Aunque la IA genera inquietudes en el ámbito educativo, también puede formar la conciencia política e histórica entre la juventud.The postPese a todo, la IA podría potenciar el criterio político de la juventudappeared first onLa Silla Vacía.</t>
         </is>
       </c>
     </row>
@@ -1090,12 +1086,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Los therian: un fenómeno que alarma</t>
+          <t>Murió el influencer colombiano Alejo Little a los 33 años: estos fueron los quebrantos de salud que presentó en los últimos meses</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1120,29 +1116,29 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/los-therian-un-fenomeno-que-alarma/</t>
+          <t>https://www.infobae.com/colombia/2026/03/14/murio-el-influencer-colombiano-alejo-little-a-los-33-anos-estos-fueron-los-quebrantos-de-salud-que-presento-en-los-ultimos-meses/</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Cuando la identificación con un animal es persistente. se recomienda orientación psicológica para ayudar al joven en el desarrollo de una identidad saludableEl artículoLos therian: un fenómeno que alarmafue publicado originalmente enLas2orillas.co:...</t>
+          <t>El creador de contenido compartió experiencias sobre el acoso escolar y promovió la aceptación personal a través de sus redes sociales y charlas en instituciones educativas</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Figura de Independiente Medellín dedicó su gol en la clasificación del equipo en la Copa Libertadores a una persona que “está en tratamiento”</t>
+          <t>Con $86 mil millones de regalías, Bolívar construirá universidad en Montes de María y otros dos proyectos educativos</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1152,12 +1148,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1167,44 +1163,44 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/13/figura-de-independiente-medellin-dedico-su-gol-en-la-clasificacion-del-equipo-en-la-copa-libertadores-a-una-persona-que-esta-en-tratamiento/</t>
+          <t>https://www.las2orillas.co/con-86-mil-millones-de-regalias-bolivar-construira-universidad-en-montes-de-maria-y-otros-dos-proyectos-educativos/</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>El equipo dirigido por Alejandro Restrepo venció 2-1 a Juventud de Uruguay ante 12.000 hinchas y clasificó a la fase de grupos, donde acompañará a Deportes Tolima, Junior y Santa Fe en el torneo continental</t>
+          <t>Los proyectos impulsados por Yamil Arana buscan, entre otras cosas, abrir más de 4 mil cupos para jóvenes de una región que durante años fue escenario de conflictoEl artículoCon $86 mil millones de regalías, Bolívar construirá universidad en Montes...</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Abren 200 becas para jóvenes del Pacífico que lideren proyectos en sus territorios</t>
+          <t>Los therian: un fenómeno que alarma</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1214,29 +1210,29 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/abren-200-becas-para-jovenes-del-pacifico-que-lideren-proyectos-en-sus-territorios/</t>
+          <t>https://www.las2orillas.co/los-therian-un-fenomeno-que-alarma/</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>El programa DALE lidera Pacífico ofrecerá formación, mentorías y acompañamiento a jóvenes que impulsen iniciativas comunitarias en litoral.</t>
+          <t>Cuando la identificación con un animal es persistente. se recomienda orientación psicológica para ayudar al joven en el desarrollo de una identidad saludableEl artículoLos therian: un fenómeno que alarmafue publicado originalmente enLas2orillas.co:...</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Estudiantes de colegios públicos en Bogotá que tendrían que reponer clase el sábado</t>
+          <t>Figura de Independiente Medellín dedicó su gol en la clasificación del equipo en la Copa Libertadores a una persona que “está en tratamiento”</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1246,45 +1242,49 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/estudiantes-colegios-publicos-bogota-que-tendrian-que-reponer-clase-PP5091931A</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/13/figura-de-independiente-medellin-dedico-su-gol-en-la-clasificacion-del-equipo-en-la-copa-libertadores-a-una-persona-que-esta-en-tratamiento/</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>El equipo dirigido por Alejandro Restrepo venció 2-1 a Juventud de Uruguay ante 12.000 hinchas y clasificó a la fase de grupos, donde acompañará a Deportes Tolima, Junior y Santa Fe en el torneo continental</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
+          <t>Abren 200 becas para jóvenes del Pacífico que lideren proyectos en sus territorios</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1304,10 +1304,14 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abren-200-becas-para-jovenes-del-pacifico-que-lideren-proyectos-en-sus-territorios/</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>El programa DALE lidera Pacífico ofrecerá formación, mentorías y acompañamiento a jóvenes que impulsen iniciativas comunitarias en litoral.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1317,12 +1321,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
+          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1332,12 +1336,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1347,14 +1351,10 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1364,12 +1364,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>La travesía del gigante telescopio que Rodolfo Llinás le regaló al histórico Observatorio de la Universidad Nacional</t>
+          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1394,14 +1394,10 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-travesia-del-gigante-telescopio-que-rodolfo-llinas-le-regalo-al-historico-observatorio-de-la-universidad-nacional/</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>En medio del paro de la Nacional, el cientifico donó su telescopio personal, el más grande instalado en Colombia, ahora al servicio de estudiantes e investigadoresEl artículoLa travesía del gigante telescopio que Rodolfo Llinás le regaló al...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1411,12 +1407,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
+          <t>La travesía del gigante telescopio que Rodolfo Llinás le regaló al histórico Observatorio de la Universidad Nacional</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1426,12 +1422,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1441,20 +1437,24 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr"/>
+          <t>https://www.las2orillas.co/la-travesia-del-gigante-telescopio-que-rodolfo-llinas-le-regalo-al-historico-observatorio-de-la-universidad-nacional/</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>En medio del paro de la Nacional, el cientifico donó su telescopio personal, el más grande instalado en Colombia, ahora al servicio de estudiantes e investigadoresEl artículoLa travesía del gigante telescopio que Rodolfo Llinás le regaló al...</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
+          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1469,12 +1469,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Valledupar</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1484,39 +1484,39 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
+          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
+          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
+          <t>Estudiantes de colegios públicos en Bogotá que tendrían que reponer clase el sábado</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1531,14 +1531,10 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/bogota/estudiantes-colegios-publicos-bogota-que-tendrian-que-reponer-clase-PP5091931A</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1548,42 +1544,42 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
+          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
+          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1591,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
+          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1610,27 +1606,27 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
+          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1638,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Prosperidad Social inicia entrega de transferencia monetaria de Jóvenes en Paz</t>
+          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1657,7 +1653,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1672,12 +1668,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-inicia-entrega-de-transferencia-monetaria-de-jovenes-en-paz/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Esta transferencia corresponde al ciclo 1 de 2026. Más de 12.000 jóvenes en el país recibirán los recursos. Bogotá D. C., 24 de febrero de 2026. Prosperidad Social realizará este 27 de febrero la transferencia monetaria condicionada para los...</t>
+          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
         </is>
       </c>
     </row>
@@ -1689,42 +1685,42 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
+          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
+          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
+          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1732,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
+          <t>Prosperidad Social inicia entrega de transferencia monetaria de Jóvenes en Paz</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1751,7 +1747,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1766,12 +1762,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-inicia-entrega-de-transferencia-monetaria-de-jovenes-en-paz/</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
+          <t>Esta transferencia corresponde al ciclo 1 de 2026. Más de 12.000 jóvenes en el país recibirán los recursos. Bogotá D. C., 24 de febrero de 2026. Prosperidad Social realizará este 27 de febrero la transferencia monetaria condicionada para los...</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1779,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
+          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1798,27 +1794,27 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
+          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
         </is>
       </c>
     </row>
@@ -1830,7 +1826,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
+          <t>La crisis de natalidad acaba el negocio de los colegios privados, pero abre una oportunidad para mejorar la educación</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1845,7 +1841,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1860,29 +1856,29 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
+          <t>https://www.las2orillas.co/la-crisis-de-natalidad-acaba-el-negocio-de-los-colegios-privados-pero-abre-una-oportunidad-para-mejorar-la-educacion/</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
+          <t>Colombia tiene 33 alumnos por docente, el triple que los países líderes. La crisis de natalidad permite reducir esta brecha y apostar por la equidad socialEl artículoLa crisis de natalidad acaba el negocio de los colegios privados, pero abre una...</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
+          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1892,7 +1888,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1907,71 +1903,71 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
+          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
+          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Valledupar</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
+          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
+          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2001,24 +1997,24 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
+          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
+          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2033,7 +2029,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2048,86 +2044,86 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
+          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
+          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
+          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
+          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2142,12 +2138,12 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
+          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
         </is>
       </c>
     </row>
@@ -2159,17 +2155,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
+          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2179,7 +2175,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2189,29 +2185,29 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/cultura</t>
+          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
+          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
+          <t>Persecución del ICE en Georgia termina con la muerte de una profesora: 'Dedicó su carrera a que cada niño se sintiera valorado'</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2226,7 +2222,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2236,35 +2232,39 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/cultura</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Una de sus compañeras afirmó que Linda Davis hacía sentir importantes a todos a su alrededor, desde estudiantes hasta personal administrativo.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
+          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2279,44 +2279,44 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
+          <t>Gustavo Petro aseguró que ha salvado a “miles de niños” en Colombia y en redes le recordaron la muerte de Kevin Acosta - Infobae</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2326,57 +2326,57 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxNRE1yOXc4NEJZaU8wdFVIY0tmUFdnMTNKOTE3X2ZubVNNOWxfZzdjSWNNbXQxNDRlbE1UenN5OFI0VE5WYzdZTXNIVXkzVFdpT3Z1cnRQRU5Qc0poSno1R29fU0tPTV9PRFJPZWVYcTdqVDY3Nl94R0ZITUNQSllRZUNzTl9LNXpURlBweEdiS0pPaHdHajhkNkJtQUFHbVJrRTViek9NWWtuQThXVTktV3BZWmR3VTJMREdlakJJMzd2YlRFdFB3X0h2MmQ2QnFTMnNiZTZ0dFFUTFVzemFlVUNyMjRmd0pxNzVVN2NfTVF1eHhsMVBQUXAzMF9yUXF3ZlZQNzRiTFJJZ9IBpAJBVV95cUxPRFZUS283NTMwczZpenJCYnotZXBpd1BPTWJ0NWxsTGVVNGdzZkcxR2R1TjFpaTR3ZlNaZ2dHNklweDZtbE9mbERfNVpUMm1yTFNEMER1UF90RnlZb21fZ21FX3dGRngyaE1RaFpjWmVuSWtfU1EtYUtWWjhKUzB5VEhWTEdhdzRYTGIxNGJROGhBUC1JdTFQUWVPanJkWWJTQVBzMmVBVjBwZkhsRTZZcTFlM3VyTm1aaWRQa0JNdy1kUGRqV1ZOendLbW1IRnZVRWMxUVlPWU04VWxuUDFhUHBvVWZtb2ZPS1B4UlhuVWJHQko3V3VXM0JKZFhYOEJJMWlwQllzYkRjdmxQbzB1ZHZDUlZBTVpDN0JLVC1qYmVPTE9X?oc=5</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
+          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Adam Mosseri, director de Instagram, desmiente la existencia de “la adicción clínica” a las redes sociales</t>
+          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2401,12 +2401,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2416,12 +2416,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/tecno/2026/02/12/adam-mosseri-director-de-instagram-desmiente-la-existencia-de-la-adiccion-clinica-a-las-redes-sociales/</t>
+          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>El directivo admitió que ciertas funciones de la app como los filtros digitales generan riesgos sobre la imagen corporal y el bienestar de los usuarios jóvenes</t>
+          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
         </is>
       </c>
     </row>
@@ -2433,12 +2433,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas</t>
+          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2448,22 +2448,22 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/12/la-falta-de-sueno-deteriora-la-salud-cerebral-y-emocional-desde-la-infancia-60-de-los-ninos-y-adolescentes-no-duerme-las-horas-recomendadas/</t>
+          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>La Defensoría alerta sobre retrocesos en el sistema educativo por recortes fiscales en Costa Rica</t>
+          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2491,12 +2491,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2506,14 +2506,10 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/costa-rica/2026/02/12/la-defensoria-alerta-sobre-retrocesos-en-el-sistema-educativo-por-recortes-fiscales-en-costa-rica/</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>La institución destaca que los menores recursos afectan gravemente a quienes estudian en comunidades rurales o con discapacidad, evidenciando riesgos persistentes para la equidad, la calidad y la inclusión escolar</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2523,7 +2519,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas - Infobae</t>
+          <t>La falta de sueño deteriora la salud cerebral y emocional desde la infancia: 60% de los niños y adolescentes no duerme las horas recomendadas</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2553,7 +2549,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPYUdxTE4wbVhKbEgzN1NYZm0xcmNxQjNJbllOYmhWTWY0UGJJS3VRMnhRZW1tblhtNEVlQjQ0NHIxSWdLejJrbHIyV2NqSWQ2MU1HS2RCYkJlRDM1cms0QW1wb2ZTX3VmdFNsc3JobDFGcGVRdGxTU1o1dEZOZnFtTUVURmJLR1p1WFJqVnlaRUNvdVI2VWdsb3phbjQwd2ZqeUtWeGpnak13cGhEMHgzUTNrZi1ORWZLdGxuT3ptc00xdjI1MWJVY3RnV21pMWktT0djZnhtd1pLX3VhRDUyZjZGZXd1NkNWS1F4WHZTMkt6QzNWV1VkVDVhV1Z4b0FjQjJXamdiT1lFUkV1ZDhNMVBB0gGsAkFVX3lxTFBJbVlTbjYxN0p5SmttZkFLVHByV0c5NmdkR0FUemxMWk5mcUtuaUV6SWc2RlVxa1FtQ2kzZXpMZHRvYU4tNmhLT2pCaEhGM2xKcG9icFRTUnZUVHZtTnUxamRHbXQyZWdaYll0Y3FTYXdnUWNMUXZIS3hwR2pYUW9vdnUwVm15ZExiRWNuR2RabjVLOG5tcjA0YTB1Tl9vRlc4WjBlSENPbXpvV1BmUGt1ckRuR0tXSHFoWWJmOVR0a2VFUDFWVkhRZ2ZiSzJTYjBvZVh3RjgxTS0tdGRlaW0zaXlBb05UWUlEY0MzdjE3M1BHbjRpdUFfN3VqWlhtTGNlaVRKdjVYSEtlX3BUUE0wSFlCd2JpaVdzNnMwQWdqRDNIdHVwS28tUDl1VA?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/02/12/la-falta-de-sueno-deteriora-la-salud-cerebral-y-emocional-desde-la-infancia-60-de-los-ninos-y-adolescentes-no-duerme-las-horas-recomendadas/</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -2566,12 +2562,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Cómo están perros que sobrevivieron a presunto envenenamiento en colegio de Bogotá; niños los cuidaban</t>
+          <t>Adam Mosseri, director de Instagram, desmiente la existencia de “la adicción clínica” a las redes sociales</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2581,112 +2577,116 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/como-estan-perros-sobrevivientes-presunto-envenenamiento-colegio-bogota-PP5043509</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr"/>
+          <t>https://www.infobae.com/tecno/2026/02/12/adam-mosseri-director-de-instagram-desmiente-la-existencia-de-la-adiccion-clinica-a-las-redes-sociales/</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>El directivo admitió que ciertas funciones de la app como los filtros digitales generan riesgos sobre la imagen corporal y el bienestar de los usuarios jóvenes</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
+          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
+          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>Los niños tienen un precio en la guerra: así crece el drama del reclutamiento infantil - El Espectador</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPV1dwRWQwYkh3X0U2a29wSGF2emFEU2ZiRzgyREhoUFJPUHdjTVc2dl9NQU5rYkhaWDl5c0k3SGpsQy1nNC0xdkZtRGxIZ25iMWdkWHFRbkdjMnN5MWhZM2lqZVN1eVVCc1IyelBlc001bDVYeC1MRENOZXRuSUtUVWdZX3BRT1JENkJjaEdyLWdPcUE2ckFxRHl6aW9yclRRUEs1a3dTVkJMb2dOeWdxY2ZaRkV6dHpHMzRaeVZ5bkMtYU1fWXEyaUtzeVE1RzBSSGVpVXVvZTRpOWlmZGcybXl0a1Z4RXZVYi1JaTFHUUYtelZ4WDRjTjlETdIBjwJBVV95cUxObmdzakVTVkJwZUpvRkREbllOQ3YzZXVSN1BTTzNhbjJvVnlCYmdkbi1qV2lPQm1VMkZ2TG9YVlhvbkU5dHdUNXM1dnpLbzJ2T1dsZDRPSGNfbGZvUTZTNjZVZjQ3WnJiM0V4aVRqNm9Sb3UxUnNkZDNKcDZtX1ZxSTFpRm5uSjhicElWaDFZNUZoRzBfTldEZktXcGpDamNFN1dLbFBjenpSUl85YVNEajNYVGJHaDRxTUtrRHZnY0RJRENrNjZUMTZzM095Skt0THAxaHdQa2hORjl3X095b0l3MEZTR1F0M2RFR3JRajBnQmF3STBaZ2NzWlotQTB3TjgzWjRUV0prb2VtYkV3?oc=5</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -2694,22 +2694,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2729,20 +2729,24 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2757,7 +2761,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2772,7 +2776,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -2780,12 +2784,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2800,22 +2804,22 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -2823,12 +2827,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
+          <t>Crisis en los colegios privados en Colombia: el Marymount y el Gimnasio Campestre de Bogotá anunciaron trascendental decisión - Infobae</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2848,17 +2852,17 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNT3E4SHRFSW0tVUVna2NoQzlDQmFUSmxweXVUVzE5ZXA3Um5KdzV5MVFfcl90aExyLUJfUzJxY1ozd1RfdndQNjNmX3d2b2laN1FyLXZiNWtBbEw1OEVZMUNLZDFCZnBjOWlSQkJNUGRMUUFsdTdBdGRGSUtya09tTHBQUEdTcVl6d3J2WFhGUkNPUjhSX2RlRDFwLTV0ZE1EdThDaEVsMzF5UUxQZzd0T1diYm9jR3RNNFppLXlNZlNVMVdaU3VPZlBYbllqckRsV09GNURkXzJ2TFMtejBpeFFjc2s4dmlKRXBPR1hUT1lveTZLV2Y5UVVDbVlhZ9IBmAJBVV95cUxOenZORjNhQTY4T18xRXVmbGpyMjd2cE1MaUVjVmp4c3hEZGtVSmJMUDZlSDZTaEdoaU9IYmMyYkVFRVU1bUdvUEVmckZmTlJiLVRqR2FOVFdSakNpa2FTemdReUxlZ0xXOExEdUliVFNHYkxzTl92bEZKOWhxVDJKNVhpNTZiN3NfTHBoZWlpRGJWLWJia25aRG9kQU5ucHZuMUZlZld5c01Qc2RXX200NEUycUhxU2M0bmVWYmpONWJlREN5eDFZNG5seE5NSTMtRVpoTTNYcm9KcVY5V0xwMDFtRzFnUm5TZ28ta1huSlpIbHNRLWpqZE9LUXk4bWt4OVpUS1paaEkwRDlycUxnbXotQ1pyeFYy?oc=5</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -2866,17 +2870,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
+          <t>Ropa interior menstrual: en qué consiste esta prenda que colegio en Cundinamarca incorporó al uniforme de las adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2891,7 +2895,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2901,7 +2905,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPUnIyNTdTak1qbjFfN3YxZ0V4SHJ3ajZ1LUZBSlVTd2R6djlJNVgySzJpU0VDWllTUDhHZHJVTXFSZE1tYVJ2dnZiU0diZDFjVjNxY1c4cUFfalBFUFJ4ZGZ6WHB5bUcwb2ZyQVo3VmxJaGIzd2RDdTJfWVhCOXhVUGJqNzVOVmU0LXdsNTdYMllTYlNyQ2tzVnJaU09NSFhoTXRHX0tsZ2FvemliREhOanAtWWp2N2hBdlI5NXdtdjJEZVdpd2U5SXZHX1dNOUt6QmV0NXRjckt2d3lQbWNHa2ZSNzBoZ2pHN1BiS2tGaUhfX2pya0pyVS0zSdIBlgJBVV95cUxQQUJFQ0w5TUgyZ2Z5QjZ0TWJ4dERKMjB2OWpzSVdMS3BwaG5NM094alJ2UzFFTHFnMEc5RnA1LVptNFVQSnhmRS1XSksxRXZNTlBZczRMdVpoZmxENGhmQTI5NnRKX2FsemlSWVVBUjBWNHFXeGdyUEMyODUwbkRpVm5xYWwyQTNxUkFrUGVidU5WM0g0ZmgzMWJ4SDl4U3pERE9fdGRqNFJjWGRBSzd3bjRrQnlFT19xNlRqeXNObU5mMW90TXR4dm1wdHJaUjU0eERCT2diRFd5eXdfTDRDa2JVeFEwQ1JmeEFESnl1ZU1wOHFMbVUzRkRPOVkzaE00aDlZMTZTVHRncEkwSElwZ1Q1Wk52QQ?oc=5</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -2909,17 +2913,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
+          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2929,12 +2933,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2944,14 +2948,10 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/inicio</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2961,17 +2961,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
+          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2981,20 +2981,24 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3004,17 +3008,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
+          <t>Estas son las universidades de Colombiamás han ganado y mas han perdido estudiantes en los últimos años - Infobae</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3024,39 +3028,35 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOT2ZVRVpaR0pGYnpicTBVZEc2a0tRa2txaXRtUGdMb01zZzZFSmp4TXVFbk9WalhsU3g3NURNNkU2N1ROWU9tZFJQZEctVi1vZlVzMm05Q3Q5UFdZVzFhNXAtWmtOV1dRUkYzTHBUdFZJZUt2ZEVpcElENU5lYXR2REdnY1VMTktyZmpFaHIzb1dYVFc0bGRMa1cxT1BQZ2pYOUFCSjlYcnh3d0JyeVJNRm5FRDkydW53dkJIUExzVWdGdHlDX2E0SFJFdWJsUVItekJFVUt1bzhIaGl3TWVKUlRQNV9LUV9YQWlUUHRYQk9hZHB10gGPAkFVX3lxTFBuSEp2R1NQSm1qeS1sUE9ld0dPNEJEZFpLSFYxX0pGRW0tQmZHZVdPMWowZXVvMDg4Slo0bk1JcmVncDF1Q1htTFB0MExXYlVwQnowak1yRjFLT3ZwNDN5NnJ1ZUxicm1RWWdFaWZnVi12Q1Z2X21INWFWSE95ME05bjg3a1ZsaHBkaTAySHVNZ3RQSDFMbEh1T3MwdVNrejNnN1lWd19TNmttWmVHc0FKN05fMnhVTEVEcFhPdU05eFoxN3F2bXh5bmw5Z2czRzN2S21mbmNYZ1BEX1JUOG12NmxneTlRRTlsbHpJa1dLZXlpZzBUR29sZldJa1pBWkRiRzdWcFVHVzNWZTRLT1E?oc=5</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
+          <t>CNSC abre convocatoria con más de 1.100 vacantes en la Dian y salarios de hasta $17 millones</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3066,7 +3066,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -3081,25 +3081,29 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/inicio</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Las inscripciones estarán abiertas del 28 de enero al 6 de febrero, con oportunidades para jóvenes sin experiencia y personas con discapacidad.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
+          <t>Universidades en que más se matriculan estudiantes en Colombia: U. San José le gana a los Andes - Pulzo</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3109,22 +3113,22 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWDZMaWZRYlpZb2pqZDdYaUJtdXlfU1VKTHJPRWg0ZmVlZnV5dC1KRTM1YVVaamZVVzV6djZXU1d2MGp2bVZXcW5vSllmcnVGQ3o4aFlYOGhMbzNMY1dVOC01Q3p4VkRFbm5iSWpYZjI5a3JhRnZEa1AtRnBNQU9BeUE2VVc0cTZqYzc3V09XZFBrS2tUMmYyNThyUlJtRHZFUW1B0gGoAUFVX3lxTFA4MDVZYUt4bXV5WTlKX3hVOHZaRmgxQzhtX292OEVSWC1EQ0FONlI3MEd5S0RObDAzWnM3b3c2XzhVaFF6VnJSQVdtTGh0V29OMW9FQkppblNnZHZwbm8tdGItLXBMX2t3ZWFfLWtWTElDRVdVblRIUW0tWHowZE54c0ZrMVY5d2xRWmZFbkx3WkJXT1FBVi1vMEQ0dDVsaDlOMGUyTGU2UQ?oc=5</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -3132,12 +3136,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
+          <t>Especialistas alertan por nuevas señales poco visibles de ansiedad y depresión en niños y adolescentes - Infobae</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3167,7 +3171,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPcVZ0TmNveF9iVzl2RXFxWjhYdW9Xb3lCQkdmX2I5ZlpDSndwc3Npby02Z0NnZ0lQVXh3QlZWRjVzT1VEdWFyQnJUd0xaeXYxcWpFUWxYWjJXMG85RzNNd1EzcGRkSkEzV2QtLWotbXFTTm9EcHhiSU9WTFhyT0lTd1NkXzl5d3pScmhRTjBrZ2taYVlQR083dWZ1d3piandoUzhpSlRwT2lmSzhXd2JNNllCTU5DZXVGVWZ5OTB0Slo4V1Q0dGpJOVdNM0NPVHRkVlRQakpUbWdhQzNJU1VGR9IB-wFBVV95cUxNYW5KQWtqQ2tUbDVLdmdoWGc1RTY5bmFpcVdCR09CY210eUFENjR2UDc0NWRiWnJWRFNRUGFVUTZnLUlsa2JPX0JzcThNWGNaclBlckRQU0tIVTNLSUFqZWF0SmdLY0R6UWs3SkdUMkl5Zml3eFlHOW1xNXFpbXF2dU1DRDJNeC0wMFF0cGRoU3FfMzlzbzFYRlRKS2tPWjNILUdUYmhudHJBQVJVVjBTZWV2bFlKa3RRUktjQTJLcThxOGVZdVRSeTQxVnFUZFcyWFZGQ09UOTJhOXdyMXJ3SjVkOVR5QTdWSHlNNGdRbUpLcjBIQmNMSDQtZw?oc=5</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -3175,12 +3179,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3195,7 +3199,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3210,7 +3214,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -3218,17 +3222,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Programa de Movilidad Escolar 2026 en Bogotá: Aún hay plazo para acceder a transporte y subsidios para estudiantes</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3238,22 +3242,22 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://www.infobae.com/colombia/2026/01/25/programa-de-movilidad-escolar-2026-en-bogota-aun-hay-plazo-para-acceder-a-transporte-y-subsidios-para-estudiantes/</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -3261,12 +3265,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
+          <t>Globo de mecha cayó en una cancha llena de niños y desató pánico en el Valle de Aburrá</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3286,7 +3290,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3296,7 +3300,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
+          <t>https://www.infobae.com/colombia/2026/01/26/globo-de-mecha-cayo-en-una-cancha-llena-de-ninos-y-desato-panico-en-el-valle-de-aburra/</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -3304,17 +3308,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Estados Unidos hizo llamado de atención a Colombia ante la ONU por aumento de reclutamiento de menores de edad:“Dudas sobre impunidad al terrorismo” - Infobae</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3324,12 +3328,12 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3339,7 +3343,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgJBVV95cUxNNFJLRzNtTGZtU1ZCaVUxbGR1QUhBMzV5eFVUT2w4TWZVZnNfYmNMX1IydEVyYnhGT3ZJcDZMaG85R0RUUU9LaEsxT0hyYTFEcy1lNmVTMTA4TWlTbzJ2NmJNbTdxTXZQeUVsczJGMTdSZVlYVHlwblhqeG53UzZ5QkhsMVFyTWRORUQtOUNJMXFBSzJiNkZGQjJSZ1lvcWdfUHFTN1duQjJvcWVyMEZIZE01OGMyakhIQk5WbkROZlpIaDg5UHJRLWdEWVVSRlN4N21hNlhvemlncnlCZlNsM1BvYlJrX2hnUEpmREFCT1pzWS14YmtLMzNHWk1ndnN1NVE5YUdaajNmelBLZEViNEFHNHdjbFhqZEHSAbQCQVVfeXFMTXBsTHJ3d1N1RXh4WFdBdjAtMVFYcEJTV2xwd0xHZERGQVlHNXNvcW5hYmdpN09Wd1ljMjR4RjNSRWMxMl8xMmN5TzN2XzQzUDhCdlJ2WjdNSklzMG1yRzI5YnRnRDFhYWo3Wi1wOEdNbHE4UElzU2FGN3Z2b29XX0Z0bXBDczQzbE1oRE9zVjk1VG9OMzZSNlhsbjlFZUp4em84bGxJSTJyRG8yOWlvUkxPZkhVT0picHVCXzRRX2dhY1VTTWlJcUFYRnVBQzV0ck10YkktYXVpSE5uNm40U1lneGt5c0p5VUNzYnl0NEpqWmVLUE5UcWxOT1BJbnFDZmJRSG9XaTYyMXhqT3dhekhSUDBLSnh6dGxBNFNNYzktYTdZMmxmZm13bXhDd2x3Y0tvWkM?oc=5</t>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -3347,27 +3351,27 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Estados Unidos reclama a Colombia ante ONU el incremento de reclutamiento de menores de edad - El Espectador</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3382,7 +3386,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxPVFRDQXk2WVcwQVhLTmljT1B4akFGM3ozQlBvc3QyOHJua1BfT1hxRnFJY212eFowWTVTdVBmTHN6d2REcXc5VGVuUmw1LWsxNWxOeW82UzBPaVQ3azZfQVNSb0pUTHFqTHdGVWJXS2Z5YmVSbXZJSXd4dzdTamNXdUtqMTRwVDV4MF9acHJFX1pTZ19NVVNvLWdNb1Y1d0FzZlN2dWVMamlvVlNCN01ZS2MxZDh1M250d2tsNEVpc2NYRUJXcE9KYk0yd1FHU3BiNUtFOENRdWZ4ZHdsR0l2cFRFMEpKTGYtaUk4dmhuRjhyaVU3RDYxbUpCUzjSAZACQVVfeXFMTmxJSVphakhMc1dSdUhqdDJFZW00OTIwT0NRNndiZGNtLWROVW1NZFFHWHhTMzVYb3N6aHRBV1NObF94cEVSeHZMOWpPTW1oVXdGeDloRU9uSWpIUXNldU1qY2lUM3dNWnhwMUNESWVTUy1SNGYzZkM0Nk1ORE9zQkNkdzc1MnJpUldVTnhKeUsycE1rcGdwMi1SN3F4bkZUdHZGNUJWT1RLeS1ZMFJUVkdmOXpHcnpId0N2QW9oOEVsbkYyVU9xbUtnTEVBdW1kNnlOY2wwVGVUY1dCc3N5WkQ5ZTBRUTFKSndYUU4zYVU2aUc1cUlsLUt4d3B6OTZ4Xzl0cC0tMFAwQ0hwM2JWUC0?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/24/estados-unidos-condeno-a-cadena-perpetua-a-manuel-poceiro-turista-que-llego-a-colombia-a-explotar-sexualmente-a-menores-de-edad/</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -3395,22 +3399,22 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
+          <t>Estados Unidos reclama a Colombia ante ONU el incremento de reclutamiento de menores de edad - El Espectador</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3425,7 +3429,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxPVFRDQXk2WVcwQVhLTmljT1B4akFGM3ozQlBvc3QyOHJua1BfT1hxRnFJY212eFowWTVTdVBmTHN6d2REcXc5VGVuUmw1LWsxNWxOeW82UzBPaVQ3azZfQVNSb0pUTHFqTHdGVWJXS2Z5YmVSbXZJSXd4dzdTamNXdUtqMTRwVDV4MF9acHJFX1pTZ19NVVNvLWdNb1Y1d0FzZlN2dWVMamlvVlNCN01ZS2MxZDh1M250d2tsNEVpc2NYRUJXcE9KYk0yd1FHU3BiNUtFOENRdWZ4ZHdsR0l2cFRFMEpKTGYtaUk4dmhuRjhyaVU3RDYxbUpCUzjSAZACQVVfeXFMTmxJSVphakhMc1dSdUhqdDJFZW00OTIwT0NRNndiZGNtLWROVW1NZFFHWHhTMzVYb3N6aHRBV1NObF94cEVSeHZMOWpPTW1oVXdGeDloRU9uSWpIUXNldU1qY2lUM3dNWnhwMUNESWVTUy1SNGYzZkM0Nk1ORE9zQkNkdzc1MnJpUldVTnhKeUsycE1rcGdwMi1SN3F4bkZUdHZGNUJWT1RLeS1ZMFJUVkdmOXpHcnpId0N2QW9oOEVsbkYyVU9xbUtnTEVBdW1kNnlOY2wwVGVUY1dCc3N5WkQ5ZTBRUTFKSndYUU4zYVU2aUc1cUlsLUt4d3B6OTZ4Xzl0cC0tMFAwQ0hwM2JWUC0?oc=5</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -3433,12 +3437,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
+          <t>Estados Unidos hizo llamado de atención a Colombia ante la ONU por aumento de reclutamiento de menores de edad:“Dudas sobre impunidad al terrorismo” - Infobae</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3453,7 +3457,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3468,7 +3472,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
+          <t>https://news.google.com/rss/articles/CBMimgJBVV95cUxNNFJLRzNtTGZtU1ZCaVUxbGR1QUhBMzV5eFVUT2w4TWZVZnNfYmNMX1IydEVyYnhGT3ZJcDZMaG85R0RUUU9LaEsxT0hyYTFEcy1lNmVTMTA4TWlTbzJ2NmJNbTdxTXZQeUVsczJGMTdSZVlYVHlwblhqeG53UzZ5QkhsMVFyTWRORUQtOUNJMXFBSzJiNkZGQjJSZ1lvcWdfUHFTN1duQjJvcWVyMEZIZE01OGMyakhIQk5WbkROZlpIaDg5UHJRLWdEWVVSRlN4N21hNlhvemlncnlCZlNsM1BvYlJrX2hnUEpmREFCT1pzWS14YmtLMzNHWk1ndnN1NVE5YUdaajNmelBLZEViNEFHNHdjbFhqZEHSAbQCQVVfeXFMTXBsTHJ3d1N1RXh4WFdBdjAtMVFYcEJTV2xwd0xHZERGQVlHNXNvcW5hYmdpN09Wd1ljMjR4RjNSRWMxMl8xMmN5TzN2XzQzUDhCdlJ2WjdNSklzMG1yRzI5YnRnRDFhYWo3Wi1wOEdNbHE4UElzU2FGN3Z2b29XX0Z0bXBDczQzbE1oRE9zVjk1VG9OMzZSNlhsbjlFZUp4em84bGxJSTJyRG8yOWlvUkxPZkhVT0picHVCXzRRX2dhY1VTTWlJcUFYRnVBQzV0ck10YkktYXVpSE5uNm40U1lneGt5c0p5VUNzYnl0NEpqWmVLUE5UcWxOT1BJbnFDZmJRSG9XaTYyMXhqT3dhekhSUDBLSnh6dGxBNFNNYzktYTdZMmxmZm13bXhDd2x3Y0tvWkM?oc=5</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -3476,12 +3480,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
+          <t>Estados Unidos condenó a cadena perpetua a Manuel Poceiro, turista que llegó a Colombia a explotar sexualmente a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3496,12 +3500,12 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3511,7 +3515,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQSmlvdlUzeHJlOVhEOTBjQVN5TlhCWkNmaUNEQnczelA1YWVHXzJ1ZHZkM2JKcWdCNzdKYkViRnQyaFpldFB5MGQ4SU54WDVoVGNlbWdRQzJhM0hvRGFaaF9MR3lxUWhSbGJUTFNKcHVmQjJ4MjlibnNuaGNVcXVaVE1aa0stdmFzYmxvTnlmc1hwMFdQUDJGVkVuS2Y4NTgydk9zQlZsU2l0OXA2NjUzZnk3SnpDOUx6RjItNE9EYWlscDBlR19XV1pIdEgxVF9XT2RWMHItMmdEeHlqdmdfYzh1X0dIT2lLNjlvR2RsRWhDZ25iMWVGbTNzaUtQZy1STHfSAZwCQVVfeXFMTXRiNGt6QnJSZDJ3NXItNWZ1enZWUkZmMEhPSm5pNWpLT2hSLXdLWnBzOTFLcVdzM3Q2SWZ1UWpzdU13NjVDNUR6S2o5N1BhOWdlYWEyVDh2bGVqTE1LR19KUnFaUFJEVWZhTlZ4Z3RwV3J2U1I3VmtReVVaTGxMTldfeEZmclhOby1iaFpVU2ZjOUJqRERwNFlMNVdzbDVFX3BQWmg1YjNhY0hrQWJ4UW53Z0lRTWlLWFEyWm5Jck5qX3ROSXVqZUxtTHM3WDk2TDJzUDJUN21VTjkxamZMRUd2Unl3emJEaGJxejJPdFViSkNWbTRudzNRUmE4bFg4a1JaLURLa0lQakk0U0kyRFFwV0ZlRHBtZ3VNc1Q?oc=5</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -3519,12 +3523,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3554,7 +3558,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/el-club-mas-exclusivo-de-la-educacion-colombiana-solo-cinco-colegios-en-la-categoria-mas-alta-de-importante-ranking/</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -3567,7 +3571,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>En el regreso a clases, el sueño insuficiente en adolescentes duplica el riesgo de problemas de atención y conducta - Infobae</t>
+          <t>Docente indígena en Risaralda enfrenta cargos por presunto abuso sexual a estudiantes de una institución educativa</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3597,7 +3601,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNTjNaNDNPUHFZYzdoUlNIaUJZbGlqb2JPZndHd3Rad0F4VGwtRHFFQXdzaEIzRWN3bndOTjhsa0JReEtYS1B3TWN5ZVhaRG1RZGtxTkVDVVI2TWV0aTFxTC1KZUJfT2NDZEpIc0tLckJjMmhEOHZvZjVHaEhGRDB2c2NxSmw5SUJpVi0tUlVaZDI1cDgyY1p5QzVRMTlMQ0NOMlkxNGlad243SzF0TFJXZ3RNRGtRY0xtSW5VSnNZaHZCYUJWWG83RzBEZEY4dUFZYUxtLTlqVGx0bWVjbk9vMzFBS0o2LUlyTXNLb3M3ZzbSAYsCQVVfeXFMTTZoYWJjUTZubmFSQjVXNzlCZkdxTkhLby1HTG1iUmdWVVNSMGZpM3EwNkd3U3NSaVhDZWJJeHpQcC1KbUlUWjhFMERwZVBmRXM5NnJVNFQ2RmFDZmNSaXlkOG5tYWhlZlFydUw5X0xVZGkxWmVIM0tuVmd4eHBOMF9SSExuc2tzQ2stNU9kdjlCemxvZTV4MUlVbElWT3dmYmVSYXE0c0VUQTRUTGtYVDZ1SmRKU0R6Z3ZlTEExQmVMa0RDRHl2ZVlvUmVTQWl3aVJJM3hrQU5rMlpLVUYzOUNjOVBDZmVzdWtoeFdqT3JLaUdGY2JOaUw0MnJyQXVNMTQ4Wl9JNHBaYjdv?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/21/docente-indigena-en-risaralda-enfrenta-cargos-por-presunto-abuso-sexual-a-estudiantes-de-una-institucion-educativa/</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -3605,12 +3609,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
+          <t>El club más exclusivo de la educación colombiana: solo cinco colegios en la categoría más alta de importante ranking - Infobae</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3625,12 +3629,12 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3640,7 +3644,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQdlZHUENSeWozNzYtd3djZFRrTmxGeE9sXzlpNDFXYXVyYUlLWWQza0V0MlZBTVRxWmI2Zm9GNk1zMVBlWFI0NDY2Yy1kYjdmOUh4VGg1VnpxZERDWFFMM2tGZ1VVMVBDMFFUWE10SFkxLUJ6am1zYm4zYTVSUEc0Zmx1eXdHUEw2STFiNVRINUs4alBQV28xZGpTYV9RX3NaMFhsN3BMVWU3N2JtZ3UyNjdrYl9DMmJVTC01blVkblh6Q09PRzJuTVZyMFdSYnhOM1M0cFZvNXRlSGhOSzdfMDJzTHNqNndIVEIzOHEybWVDd9IBjAJBVV95cUxPQkpOR214eE1HM3l2WTFaQ01jNmRIa25id0psWW5TVmFibHFrNGxnYkxSTDNzajlYcWg4UjBMelQ5WXVaX3RjaEI5cnRqNDlVdGpyenJvTVFPMEZLeExwMUNFUWlWM2d3NTRlOWJHb0tuck5wVnlkNGZ3MkJsUXhCQTZFX3N4MV82V1B2V0pMWmdWZE43UmlHLXQxOEV1bndwdy01YWVhRmJVd2xVcC1XaDJDVWxvNFVNcEJMSHMtMHRiUENjUTBIRURsZXU2ejZuLVR2UDI2ZzJaTFk3QW1ZWGNQYVlWZ0MwNlVXaUF0SEo4Uy1pdzFKSkFFWjN3WkpLTXBKdEo3MUVZZnk2?oc=5</t>
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
@@ -3648,12 +3652,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
+          <t>En el regreso a clases, el sueño insuficiente en adolescentes duplica el riesgo de problemas de atención y conducta - Infobae</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3673,17 +3677,17 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNTjNaNDNPUHFZYzdoUlNIaUJZbGlqb2JPZndHd3Rad0F4VGwtRHFFQXdzaEIzRWN3bndOTjhsa0JReEtYS1B3TWN5ZVhaRG1RZGtxTkVDVVI2TWV0aTFxTC1KZUJfT2NDZEpIc0tLckJjMmhEOHZvZjVHaEhGRDB2c2NxSmw5SUJpVi0tUlVaZDI1cDgyY1p5QzVRMTlMQ0NOMlkxNGlad243SzF0TFJXZ3RNRGtRY0xtSW5VSnNZaHZCYUJWWG83RzBEZEY4dUFZYUxtLTlqVGx0bWVjbk9vMzFBS0o2LUlyTXNLb3M3ZzbSAYsCQVVfeXFMTTZoYWJjUTZubmFSQjVXNzlCZkdxTkhLby1HTG1iUmdWVVNSMGZpM3EwNkd3U3NSaVhDZWJJeHpQcC1KbUlUWjhFMERwZVBmRXM5NnJVNFQ2RmFDZmNSaXlkOG5tYWhlZlFydUw5X0xVZGkxWmVIM0tuVmd4eHBOMF9SSExuc2tzQ2stNU9kdjlCemxvZTV4MUlVbElWT3dmYmVSYXE0c0VUQTRUTGtYVDZ1SmRKU0R6Z3ZlTEExQmVMa0RDRHl2ZVlvUmVTQWl3aVJJM3hrQU5rMlpLVUYzOUNjOVBDZmVzdWtoeFdqT3JLaUdGY2JOaUw0MnJyQXVNMTQ4Wl9JNHBaYjdv?oc=5</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -3691,27 +3695,27 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
+          <t>Así fue la reacción de jóvenes españoles al descubrir los múltiples significados de la palabra ‘cachucha’</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3726,7 +3730,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/19/asi-fue-la-reaccion-de-jovenes-espanoles-al-descubrir-los-multiples-significados-de-la-palabra-cachucha/</t>
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
@@ -3734,27 +3738,27 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
+          <t>Este es el calendario de vacaciones y recesos en colegios públicos de Bogotá en 2026, prográmese</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3769,39 +3773,35 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/17/este-es-el-calendario-de-vacaciones-y-recesos-en-colegios-publicos-de-bogota-en-2026-programese/</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Corte Constitucional fijó nuevos criterios para el manejo de conflictos escolares entre menores de edad - Infobae</t>
+          <t>Mejoró la ocupación laboral de la juventud: ¿cuáles son los puntos ciegos? - El Espectador</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOOVhMdnBkeXFCaTNlNTNGX2ZaTGxqVnB0b2FIZ0owQTl3LXFiUldIQ2FhOFJZeGdEa3FJTjRoMkxuTHFYNFFBTTVMakFUY0tob051TWxCOVluajg1d24tdWRxM256TTFndk9FSUQ5b2FpNGY3U3ZxQ00za1JhYThoamVHUnBRVUdySkNHNzFhU1JFQ0JsLVJ1N0ZZLU1EdE5tcUViVXluc2hTWm0zblFKcWxXdW9mVDZic1FTWXpyS1NLTWNaZmlEMXZ1T0xoYVR4U2xwZjVycEtkOE1EQlBYLUtn0gH8AUFVX3lxTFB1aVQ2NGIzQ0hhVm54dGlrb0Q4WWtXUVFrdVA0N2dyVEMzWXN3T1p1QmlVZm4wQzdXZmJnZU5TcjlLSFFGTEZwODlYU0FmTU5ra0wtOEhuUWJVMWh5eXlqVEg2WGhHM2tMOVZwMkxTM25vZUFtRHA0S3JjQ1l3RElwVE8wWjRZSWhCcE5Ib1gwWXVpZ09TM2dvOVc5bzBFbFRWdmtYNUZSTzR3T1VrU1I1V25nLWlDSWsxRVJWUmczUFo2Z2lQNTBhOTR4MzhKZDc4YjJxSXJoaU5OU016NGdDX3JtTXp4dVNBTXozV09XSUhRaTJ0ckJvMS00Vw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOaUM2MXFDODhjdXVZLS1BUG9oUm52dEExRVFkb3hiZ2RCR3oyM1AwUEV2SEhIZTVjRlhWdnJ2dUdkRjE3bVhtc2hUcFpSODVCWkgyZG83T3ZPQ2ctY0l6ZXV3UVBxYmxxRzhEcDdQYlVkT3Rvdk83eWRGZkpNVEpfSEs2Y3A0V3BGcnhiQ3hwVENoZjZQS0J5SGp2VDhFVS1rM3JKcnhxdnpIR3BjWDdObkpkSE0tdw?oc=5</t>
         </is>
       </c>
       <c r="I75" t="inlineStr"/>
@@ -3961,12 +3961,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
+          <t>Corte Constitucional fijó nuevos criterios para el manejo de conflictos escolares entre menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3986,17 +3986,17 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOOVhMdnBkeXFCaTNlNTNGX2ZaTGxqVnB0b2FIZ0owQTl3LXFiUldIQ2FhOFJZeGdEa3FJTjRoMkxuTHFYNFFBTTVMakFUY0tob051TWxCOVluajg1d24tdWRxM256TTFndk9FSUQ5b2FpNGY3U3ZxQ00za1JhYThoamVHUnBRVUdySkNHNzFhU1JFQ0JsLVJ1N0ZZLU1EdE5tcUViVXluc2hTWm0zblFKcWxXdW9mVDZic1FTWXpyS1NLTWNaZmlEMXZ1T0xoYVR4U2xwZjVycEtkOE1EQlBYLUtn0gH8AUFVX3lxTFB1aVQ2NGIzQ0hhVm54dGlrb0Q4WWtXUVFrdVA0N2dyVEMzWXN3T1p1QmlVZm4wQzdXZmJnZU5TcjlLSFFGTEZwODlYU0FmTU5ra0wtOEhuUWJVMWh5eXlqVEg2WGhHM2tMOVZwMkxTM25vZUFtRHA0S3JjQ1l3RElwVE8wWjRZSWhCcE5Ib1gwWXVpZ09TM2dvOVc5bzBFbFRWdmtYNUZSTzR3T1VrU1I1V25nLWlDSWsxRVJWUmczUFo2Z2lQNTBhOTR4MzhKZDc4YjJxSXJoaU5OU016NGdDX3JtTXp4dVNBTXozV09XSUhRaTJ0ckJvMS00Vw?oc=5</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -4004,22 +4004,22 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
+          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -4029,30 +4029,34 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4067,22 +4071,22 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/el-desplome-de-los-colegios-privados-en-bogota-no-se-detiene-35-cierran-sus-puertas-para-2026/</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -4090,12 +4094,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
+          <t>La caída del “capo dei capi” de la Cosa Nostra: de una infancia dura al líder más temido de la mafia siciliana</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4125,7 +4129,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
+          <t>https://www.infobae.com/historias/2026/01/15/la-caida-del-capo-dei-capi-de-la-cosa-nostra-de-una-infancia-dura-al-lider-mas-temido-de-la-mafia-siciliana/</t>
         </is>
       </c>
       <c r="I82" t="inlineStr"/>
@@ -4138,7 +4142,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -4153,12 +4157,12 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -4168,7 +4172,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
@@ -4181,7 +4185,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4201,17 +4205,17 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
@@ -4224,7 +4228,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>El desplome de los colegios privados en Bogotá no se detiene: 35 cierran sus puertas para 2026 - Infobae</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a enviar mensaje de terror a otros niños</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4239,22 +4243,22 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPa1M0STVRWFpyLVgzeEMwUW9fTDdXVWs5RzdvbWt0WE9ZcHFZZVQ3dnhQMjh2TnJqaUV0eFFESUk2YzV3MkxVMTNNLTI4VUxrdnhUcy1Zck5WMHZVQVVYY0hEZFdwTUF1RUNJcmRQMWYwR1JfaWNvR0JQYlNDZ01BUi1lQzBJWTcweFBFMm13aVA0ajdqbTFncDJ2VTd1VjFkUUViNU1HWjgzb2ZvWWJqZjg0bWdFMjVTN1BlOEJBUUdGSnFjNUFfNDdRakZFcjA2ZDUyQ9IB7wFBVV95cUxOT05HTjcwSXlhWFBKN3dPUXd1enFRVE5UenJpZENPOTB1U1RuZTRKODN0aVc1MVpuaS1wY1pTZ1laemFkeE5zWHAzWF9aZXlYOFE0cUk2M0dRY3g1amRMUXBRNEd1VzNVdVljWHlMeVAxRWliWExhQWZFQkFvdVhXaVk2dnd2eFowVXVoN2hoc1FhNHNtdVBaQng2Y0pjTTJzR08xRktlenRmQnBnWExqSExKU3FBeEljT2c0MGxXLVo1VWFFQWlpNFUtbmx3Z2RZLWtqV0JwNlhLMWZWNFRUb3MyTXp1VHdMdllnTFI4SQ?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-que-fue-secuestrada-en-el-catatumbo-denuncio-que-las-disidencias-la-obligaron-a-enviar-mensaje-de-terror-a-otros-ninos/</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -4262,12 +4266,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
+          <t>Menor que fue secuestrada en el Catatumbo denunció que las disidencias la obligaron a grabar mensaje de terror a otros niños - Infobae</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4282,7 +4286,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -4297,7 +4301,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxObmZIdEpqTkVXcjc4UjRzR0hob1dZYk1GUUljTXNIc2psanNtWU9YZjJRaU41NWNsR3FaUUpmR0JhQTVxdEpvUXBCbjZFcWFtWXBwTFYyak9tc3Nldng1d041LVlkWGZLRm5ULW5OU2x5b1NIbHJTUTBJY3ZDbHB4ZThnUS1JV09DUm0xVEVSMV9TZ1BpdktCRzFTNnA2LUwxQnpBLTZxWHJoOXhXZTV4ZkNrRlFFSHNjNjBqOUF4bW8yNUY2el9DUDdlbU1iNXRHTGZ3eEV3d1JBNGRuUFhzM0hXd1RmdDhoYS1tM2otLVZmLUFROE9iSHYwZlRfQdIBmAJBVV95cUxQeGhobjhnanVFNTItaDNFczFzbWZBeExqSEo0bXo0LVZGYVFHcEtTTW1Seks2T21Ya19QcVVIdzJsbjgxVUJVWHE4MXZyMmVTYXBkeGdvXzAzSGljU0YtcERJdDcweFgwcVdvOFRWX0d4cEFKcG10dGc5UkVOeVZRN1BOcEREWUJwa2Q4Y1VXU0ZJR242QWtIdlFHWkQ3LXR0cnlDVE1WYU90SV9HUmdqdVI0T0FIbkwzbXI1TXZpbTNvWnNwWl9iOWF1dXZ1eGh0Zk4xSmpTUmhMdEZVTy1CeVBtS3VaZHJwY3BrS3FuZmszQTZxOWh1TkdzclZOVFU4cElBY3JRMUtDYm81djJ6XzR0YTVRRW5J?oc=5</t>
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
@@ -4305,17 +4309,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
+          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -4325,12 +4329,12 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -4340,14 +4344,10 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/actualidad</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4357,12 +4357,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
+          <t>Treinta niños quedaron sin aulas en zona rural de Nechí, Antioquia: incendio incineró la única escuela de un caserío</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Alerta Bogotá</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -4372,22 +4372,22 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://www.alertabogota.com/noticias/local</t>
+          <t>https://www.infobae.com/colombia/2026/01/13/treinta-ninos-quedaron-sin-aulas-en-zona-rural-de-nechi-antioquia-incendio-incinero-la-unica-escuela-de-un-caserio/</t>
         </is>
       </c>
       <c r="I88" t="inlineStr"/>
@@ -4395,17 +4395,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
+          <t>Tres estudiantes resultan heridos tras caer desde un bus de dos niveles; autoridades investigan</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -4415,12 +4415,12 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Barranquilla</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4430,50 +4430,54 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr"/>
+          <t>https://www.diarioadn.co/seccion/actualidad</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Los menores, de 13 y 14 años, tuvieron que ser hospitalizados.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
+          <t>Estudiantes respiran con el aumento del pasaje de TransMilenio: no tendrán que gastarse lo del almuerzo</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Alerta Bogotá</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
+          <t>https://www.alertabogota.com/noticias/local</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -4481,32 +4485,32 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
+          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -4516,7 +4520,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
       <c r="I91" t="inlineStr"/>
@@ -4524,32 +4528,32 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
+          <t>¿Cuándo entran a clases los colegios públicos y distritales en enero de 2026? - El Espectador</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -4559,7 +4563,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQVGV3a0tQeW5uLVpJdlBBT3Rrc0NrUm9Va3pHY3NYMko1d1N4bjUzdjVYZ3ZjZWZpQ0xYak0yQVNLdFRsVXJxbnJMSVJVT3ZyaEZ4ZEZIU01RWVoyUHd6Q0hiNFdCMElNeXExYXVrQVJaQU8tN0RUMC0xZERQdFZ2aWo0UXQtZTZ5VmN6NE9YSjlhYUVGd01ycDBCaC1RMEhUcmk5TTdEekozS3g5Ry02SEVTOWprUdIBygFBVV95cUxQMlJDNFNLREl3U2ZaeXVGYy1GS2NmWlVydW1DX24wRE9NOVhBbzhqNWNzMmhTNEdTa0JFa281R1FVRUFfdjlUXzd2Nl8xTGxMb3JIaUVxOG1DTTBwRlluV1B3QVF6QTI1cEd1TTlVQlJiVWJkLWFFRFo1RlVsQjRMS2ZmTDhpUTY3bGdfRzlXWmliT2NybEFPcnRfaWJpX3UtazA0ekRpOFpOeU93TGNsOTV6Ynp3VkhKRnVPcmswemZHYnZNQUxrWHNn?oc=5</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
@@ -4567,32 +4571,32 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
+          <t>Niños colombianos pasan 8.9 horas diarias frente a pantallas: qué efectos hay en su salud - El Espectador</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -4602,7 +4606,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPZkRQZ0I3REZBYkZoNlVha2RNQ3F6dmlSYU5hTTBBOGkzMlBSM2xXV0RsMFRKcy1XRG1xWWNmQk5mUWE3ci1BMGZpNGZHeHFjcDBmdGQxb1cwNG95V0R0RVNodGlYcXFFcHRLdWU3bWgtSC1vV2YwTE5wVVpBejlZd2ZmRENoVTl4cDNnNWQwUDBxRFlIak83MjRYelRLRVdodS1wNnRLeC1wS1ViT2Y2SDhOSmdYZ0taY3BDNmxYMUpuUdIB1gFBVV95cUxOTUtIYTlOYUdmTHVzRmZWQVNGRkVsdDk3cEg4bDlRaXhVRUZyd2tBOHFXUWplMUtQYUpRX29LbDZNOHhDcXc4OHQ0OTVNS1I3cElDR1RRNFliRXA0UjV0Y1kzbmdzRzFVSnNYUlZUeEN4OEt1SnZDbXRzQ1hycHoxRTE1RlZzNk5BR1o2LTBTTWZka01pR2oycmV1MWlZY2ZoSjVvRlBvMWVLODJMbnFaZ251aU0zWGZqWHkwX1lMTEZCaC04ZEQwZTNTaU1ycktSUDhuRVRR?oc=5</t>
         </is>
       </c>
       <c r="I93" t="inlineStr"/>
@@ -4610,12 +4614,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
+          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4635,7 +4639,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -4645,7 +4649,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
         </is>
       </c>
       <c r="I94" t="inlineStr"/>
@@ -4653,27 +4657,27 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
+          <t>Estudiantes de Medicina anunciaron protesta y Gustavo Petro les respondió: habría plantón en 17 ciudades - Infobae</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4688,7 +4692,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOckVuZWpkQV9QTnd6UzZmSXdvNl9xX3plZHNIRkV1X2liZTJmYjRHY05uVDc5M09nekFlMDVwVS01WWtsZmstN1VtZkc3M0E5d0xGd1lRMzh5c0Qtc09iei1pVmdSekozWUVLenM5YVRtTms0R3BJdEZocU9YVE5wUEo0UVdLRnQ3cENPWm1ETmhsbjFULThLTVRKanQwSTVvM2hCQW5VODlJejZkRkpYUHpzREpEeDY1M29UaV82cUZQVFp6OEpmRVlxRTBzQzFUcWlPbTVWOVQwSG9LVF9KcGhiejZzTWt2S05KYzdyeDgzbThZMmhkdUNQZTBBdGNHN2RletIBnwJBVV95cUxPOTVVOXMyRFBNN21yQnZ5RHkzMTZOMVYybU0xXzNzczIycm95cHdBcEFKc0d0VVlLT25PYWJkVDhnbUVMdlQwTHktNlJqNG9EeXFDQ1RSaG51Tnc4ZXlsWXpVYzZSZWl1MXVRQVdabXI5ZTRUYXdQblUzWmN5NEE3VW1PRF8yNWdHcjVsdXZ3STF2cUJlenZHbTluZkpKYzRvSlhDZVlNVWdnVjBqZEFuSHpuQnNwdUVMMjBkMm5JNUZVZkFfOHFUMHFpeEdLWGFzZ0Q0V0pZdzdrMXdpUkRsRVZQRVppU3hnTXZlU05GRWZlZ3hKUnBKdFlWdy02cXJRdE1YWUFsSDRZTXctSDRhSkRMMV95QlRPUkJIVV92Yw?oc=5</t>
         </is>
       </c>
       <c r="I95" t="inlineStr"/>
@@ -4696,17 +4700,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
+          <t>Accidente de estudiantes del Liceo Antioqueño: bus iba con el 97% de su capacidad, sin cinturones y con fallas graves de seguridad - Infobae</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Noticias Caracol</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -4716,7 +4720,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -4731,7 +4735,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNZGtNeVVBeHQta1Zhc2Z5YVpZR09qcnJZdnZCOGJ1TGdwbEktWVQ1UElPWmI2bEFEZUlOUGI5Z1J5U053TlBHcHkxclNnYlA2VU8zaWMwN3ZXdW9kdW1wTEJ5akcwcC1kZXk1eFZnQTlNT3JsUnRlRGNwTFpuNFZ4SnowUW5qQnhacGxHSTlCUXdRWDBXRjdHQUd1RGtkUjFJOXZhNmZkWXdfd0I3WGdYcWllRThlRkR4LXdQa1JNbDBlN2pyOUtJSU1zbGhob1cxUWhjeE03aXVJYWpLaTh4QmpyZGpXOVQ4dHJURUd2MWdtb01wd3hISTladGdKbDV1NmfSAZwCQVVfeXFMTmlvd2VmT04wQVNQWEh2LVQ3WXF6M0hZZU4wa3RKa3dUMEU3c3NPQmhONUoxbGNQNnJPR1dsUWp3d3pVT19vM1JoUnZNTWZIR1hWcjZXYXBNcVQ5OVN4dGR2S2dfbXZWclFFeU9GNUM2eEY3OWR5OWo5OUZTeXVSMWhKTHV0VGx6RFc4eVktSGFXdGJwa0FNWTd4b3hyakQxRWNJMXlOUjhiaEhtbXZhWkhDUmZ3ZVVTNGNfTEdUZjl3Z3VPT0VwVjZ5OHBOT0tEVmlZbTFKVUtXcU5JaWN0MnVpNWFLdmVtZTlaQV9Cd0Y3RUc3eXI1R3hrNnRXVnZELVliZTRrVUNaYXNsdFJ1Q2ZkRFpRSnhYcjl3NGE?oc=5</t>
         </is>
       </c>
       <c r="I96" t="inlineStr"/>
@@ -4739,27 +4743,27 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
+          <t>¿El alemán será materia obligatoria en colegios públicos? Esto dice el Mineducación - El Espectador</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -4774,7 +4778,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNZFh6ZDVETFROR255WTE1dm1uNXhtaXg4aGNjOUtZblZDbU9RbnFhLU81Z29yVDZzeG1HcFpjeS12UFJNX1lSaXRRVWIyWUFyWkMyaDJobmNReFhjRzREcTFBTGFsX3RwNDRnUHhydUtWdEcyR0VFeVRXUlg5c0hJZlhydURCVG0zcmd0SkNVbk5qak8tbkJGWnducXNZV1hOUFEtSHRWbmVvOFRXSFM4aG5zbU9SOWJ2Y1RTRGNB0gHSAUFVX3lxTE5jTVU1LW82UDhqRVdjVnNNQ29LZXpEdTM1a2NiRlNUaVBBUnVCZ25hamlJM3RiZW9DNzBMYWNBanJaemVuaEdzUUMyOFljN0t3SU1ac0ZRNnBLWm1LNjAycG8yUFRTZllRWVIwTWV0dTN2TTM3WEt5ZWNNWFlia2VvMFdnNEZtMTlDSWhwX1ZLc3hCTDlvT20zd3ZJUEE2UVJVc1Z3bGpnOENxSWNYcExDX0hiaGxTMnE2dXBSaEJnRE9Od2VQdk1vQmVCUy1PdjlSZw?oc=5</t>
         </is>
       </c>
       <c r="I97" t="inlineStr"/>
@@ -4782,17 +4786,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
+          <t>El nuevo idioma que tendrían que aprender estudiantes de colegios públicos desde 2026 - Noticias Caracol</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Noticias Caracol</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -4802,22 +4806,22 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNRENPX0xEVmxGRDFJallZVDY3UmlXZ0Q0bzVWX2kzSFBISXNlMWZ3eWM0Q1R3eE5KdUF3ZWpRcEFRSG5Rbl9wbnZoeTQyckpBX0VuQ0s2aTFoc2lOblVkd1V0b2FGU0tRNnBsUldGLUdoTGJwVFpTZkcyenB5blpDVi11Y3g3Y3JVQ1lUNVpTZTYwZXVmY3ZhR1ozUUNYMDl0bm5PeFRETzZFTlhIamc0LVZXMWhyNnFqNGpSTXBGOGdONDc5UWJRRTZpc19vczJ0LXFV0gHgAUFVX3lxTE40d0Y3d0Y1VDdvd0FnQWpvdGhBTjl2T3Jsc2dkQnlxSF9OQjhiaVM2VkNLckhhSWZpczU2TTlySGx2RHBadTZJT0E3MTdyZU9ZOTQ4cHIzTW5HZ2FXZ182TjJrdm1xeVAwWVVOZmR1SzktLUl0cGl3dEdyZHlUakYtOHFEMVo3NF9PdzdwZXdSR0FiWDJVQm5FcDBhQ3c2T1ZRXzdFeVZDdkJfYms2UFpHM3lKTk15Y0JFWVNGellIekRvUWpPZFFGOTNBQlkxZmhLR2wxV01yOEtWUTh2cmFY?oc=5</t>
         </is>
       </c>
       <c r="I98" t="inlineStr"/>
@@ -4825,12 +4829,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
+          <t>La SIC impuso medidas a Rappi, Dislicores y Éxito: buscan evitar venta de vapeadores a menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4850,7 +4854,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -4860,7 +4864,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQTDZ6dnN2WnNvMEl4WDlXUjRsY2tRVjUwNDlUekJ3TDl2YWZ1dVQwVjR1bVFYUTQ4d2F1VmRnTG1QQm9GY3NudHZscjVvOXRRaGZHaG53NWVNbkZOWlpvYVR3Ry1ZV3B3TkxmTEVBM19VQXowNEk4V2dwNWJ2YkU5MUNDSDhoejhNeTZ2OWs3bkJoZmktdVdzMHpIMnlLb1AzUWt0OWFiTTAwakNlZGR3ZUhNckstTXB1eGI1ajVvTFZXSjd0Q3kteHJESU50UW5NTGEtR1ptNW1ueHdHTEFKVWpOLWZDRGtibEtidG04TVpLQlYyTlR3NVRPX1drUGh00gGbAkFVX3lxTFBUMk1tdnRwODNzcE02RVVvbWtQd3BjajRfWlQ5aVdScUNHOFNSSlU4cHhZQXJVajJZcEc1aWZBZU9OakE1RXc5cFg0cTJwN3E2RmZBQ21sX3h1YUg0a3d1YjBJdWY4aGl1VU9lTXJKNlphR2FVaU9WVlRuMzJJVGFyX09SNzMyWE5sV0E5THZWd3RWVTF0bVUza0gwWml4U2ExRG1mYmlyMU44RVNCLXZjc1dIcXZESXF2eHRQOWtMLWlQdXlHa05qaFhnMjVQVFQ1elh4MC1VenZKcHV4UzBoRTZ6N0JhN0dPV1FiQjVSSTZ5YmNQV0x0cWpwaVQwMEswTUN5SEw5b2M4VXVUREVnd0IwdTlkaW1fT3M?oc=5</t>
         </is>
       </c>
       <c r="I99" t="inlineStr"/>
@@ -4868,74 +4872,70 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
+          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Política pública</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
-        </is>
-      </c>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2025-11-13</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
+          <t>Tras el envenenamiento con talio de menores en Bogotá, Zulma Guzmán confesó la relación que tuvo con padre de una de las niñas fallecidas - Infobae</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -4950,24 +4950,20 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
-        </is>
-      </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOYmZ3Tm9XR3FoMXBaa25la2NlYWFPWjFqejhhY0VyWU8yb2VOampHZXIxMlRrVU8wTG9NOTZla1NXeHZsRW9kSWJnaE1QUjFCemJ2bHJWejlMeHlwcHZTOE1Yc2dsY21MUUJ2cGpMX1V0UEVpeDhzRFo4YmwxR2gwaHRVNWJab0N1NnBxaF9HR0VBc2xxUWNSZUhLSXJ6TjRkX1ppT01jQ1YyOXlsSmhWd2lnNXdxQ0xKR19iWF90dC1zY2Jobnk4T0VZRU1yZjJRN1VJT1BNT3l4dW10REVFbWlNd1JPVm5KaFF4NzF5RXlxeU5TUlNpTUFlWdIBlgJBVV95cUxQSUt2Nmk1NTYtZzNZdjYtdzhFV2Ezal9OWEhoY2hjczBUV19UN2UxN3dfYmw5SW5iMEJBY1B1ZUowZlN0a3NpQWROcTR3WjRsRThBV25QU3FLbllrWWxIOUpLamxLNDJUdzU3elVEYzRqbGc1SE5PeDZ1dmNvMmtVZUlCSWNMOTlrcVUzdFlkcThpUmQ0THBTZGEyNkJZUl9UYnFhanVEdlNmaWdNSHNxWTVSVHRLQk1MaElEOWxNUzFZeWczRkdpbHM2bVlZQUdjQ0xkdDJqckNfR2tSckVtQW9hYzlZSTlpS1BwX1pWNXpJa1R2MS1ZSU5rWDRZX1lQVzRud1hoRmk4aXZ3SFRxc2FwdjRpdw?oc=5</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2025-11-07</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
+          <t>La localidad de Usaquén tiene una Casa de Juventud para beneficiar a más de 100.000 jóvenes</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4982,7 +4978,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Política pública</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -4997,24 +4993,24 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#74871d874f</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
+          <t>●Bogotá abre un nuevo espacio para las y los jóvenes de la localidad, ubicado en la calle 155 #7-45, con acto protocolario y participación de autoridades y representantes juveniles. ●Esta casa amplía la cobertura territorial del servicio Casas de...</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2025-10-16</t>
+          <t>2025-11-13</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
+          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -5029,7 +5025,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -5044,24 +5040,24 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
+          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2025-10-09</t>
+          <t>2025-11-07</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
+          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -5076,7 +5072,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -5091,24 +5087,24 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
+          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2025-09-23</t>
+          <t>2025-10-16</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
+          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -5138,24 +5134,24 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2025-09-19</t>
+          <t>2025-10-09</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
+          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -5185,24 +5181,24 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
+          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2025-09-13</t>
+          <t>2025-09-23</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
+          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -5232,24 +5228,24 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2025-09-19</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+          <t>Últimos días para inscribirse y obtener una beca en formación técnico laboral de la Agencia Atenea</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -5264,7 +5260,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -5279,24 +5275,24 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#d7dc735e17</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+          <t>•Son 1.500 cupos y se cubre el 100 % de la matrícula, apoyo económico por semestre y acompañamiento en la ruta educativa y laboral. • La convocatoria se cierra el domingo 21 de septiembre a las 11 y 59 de la noche</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2025-09-09</t>
+          <t>2025-09-13</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -5326,57 +5322,151 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2025-09-09</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>SDIS - Juventud</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>institucional</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
           <t>2025-09-06</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr">
+      <c r="B112" t="inlineStr">
         <is>
           <t>El Frailejón abre sus puertas: Usme estrena nueva Casa de la Juventud</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
+      <c r="C112" t="inlineStr">
         <is>
           <t>SDIS - Juventud</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr">
+      <c r="D112" t="inlineStr">
         <is>
           <t>institucional</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
+      <c r="E112" t="inlineStr">
         <is>
           <t>Otra</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr">
+      <c r="F112" t="inlineStr">
         <is>
           <t>Bogotá</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr">
+      <c r="G112" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr">
+      <c r="H112" t="inlineStr">
         <is>
           <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c7eca5d4bd</t>
         </is>
       </c>
-      <c r="I110" t="inlineStr">
+      <c r="I112" t="inlineStr">
         <is>
           <t>• Aunque ya existía una Casa de la Juventud en Usme, la sede se traslada y reinaugura para ofrecer mejores condiciones, ampliar servicios y fortalecer la atención a los jóvenes. • La reapertura se desarrolló con el acompañamiento de la Plataforma...</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-03-20
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I112"/>
+  <dimension ref="A1:I114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,12 +478,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Condenaron en Miami a hombre que viajó a Medellín a abusar sexualmente de una menor de edad</t>
+          <t>Balacera en Barranquilla dejó tres personas heridas y tres capturadas</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -498,12 +498,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -513,24 +513,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/medellin/condenaron-en-miami-a-hombre-que-viajo-a-medellin-a-abusar-sexualmente-de-una-menor-de-edad/</t>
+          <t>https://www.elespectador.com/colombia/barranquilla/balacera-en-barranquilla-dejo-tres-personas-heridas-y-tres-capturadas/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Declarado culpable en Miami hombre que viajó a Medellín a abusar sexualmente de una menor.</t>
+          <t>Una balacera, al parecer entre miembros de Pepes y Costeños, dejó tres heridos y tres capturados, entre ellos un menor de edad.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Insólito pedido de familia de David Acosta luego de que el joven apareciera con vida en Bogotá</t>
+          <t>Dos menores de edad murieron en grave accidente de tránsito entre moto y tractocamión</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -550,17 +550,17 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/caso-david-acosta-familia-pide-cerrar-investigacion-falsa-desaparicion-PP5103111</t>
+          <t>https://www.pulzo.com/nacion/dos-menores-edad-murieron-grave-accidente-transito-caldas-PP5103822A</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -568,59 +568,55 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Adolescente de 14 años murió en riña entre menores de edad fuera de un colegio en Cali</t>
+          <t>Insólito pedido de familia de David Acosta luego de que el joven apareciera con vida en Bogotá</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/adolescente-de-14-anos-murio-en-rina-entre-menores-de-edad-fuera-de-un-colegio-en-cali/</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Adolescente de 14 años murió en riña entre menores afuera de un colegio en Cali. ¿Qué dicen las autoridades?</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/bogota/caso-david-acosta-familia-pide-cerrar-investigacion-falsa-desaparicion-PP5103111</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Por explotación sexual, capturaron a estadounidense en hotel del norte de Barranquilla</t>
+          <t>Condenaron en Miami a hombre que viajó a Medellín a abusar sexualmente de una menor de edad</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -635,12 +631,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Barranquilla</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -650,12 +646,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/barranquilla/por-explotacion-sexual-capturaron-a-estadounidense-en-hotel-del-norte-de-barranquilla/</t>
+          <t>https://www.elespectador.com/colombia/medellin/condenaron-en-miami-a-hombre-que-viajo-a-medellin-a-abusar-sexualmente-de-una-menor-de-edad/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Las autoridades capturaron a un extranjero y a una joven de 19 años por explotación sexual de menor de edad y proxenetismo.</t>
+          <t>Declarado culpable en Miami hombre que viajó a Medellín a abusar sexualmente de una menor.</t>
         </is>
       </c>
     </row>
@@ -705,32 +701,32 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Estudiantes de un colegio en La Ceja, Antioquia, impidieron la construcción de un hospital sobre un humedal</t>
+          <t>Adolescente de 14 años murió en riña entre menores de edad fuera de un colegio en Cali</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -740,91 +736,91 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/estudiantes-de-un-colegio-en-la-ceja-antioquia-impidieron-la-construccion-de-un-hospital-sobre-un-humedal/</t>
+          <t>https://www.elespectador.com/colombia/cali/adolescente-de-14-anos-murio-en-rina-entre-menores-de-edad-fuera-de-un-colegio-en-cali/</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Estudiantes y docentes del Bernardo Uribe Londoño marchan en defensa de su humedal. Un conflicto entre la salud y el equilibrio ambiental sacude a La CejaEl artículoEstudiantes de un colegio en La Ceja, Antioquia, impidieron la construcción de un...</t>
+          <t>Adolescente de 14 años murió en riña entre menores afuera de un colegio en Cali. ¿Qué dicen las autoridades?</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Mafe Carrascal explicó por qué la bancada del Pacto Histórico por Bogotá no asistió a encuentro con el alcalde Carlos Fernando Galán</t>
+          <t>Por explotación sexual, capturaron a estadounidense en hotel del norte de Barranquilla</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/17/mafe-carrascal-explico-por-que-la-bancada-del-pacto-historico-por-bogota-no-asistio-a-encuentro-con-el-alcalde-carlos-fernando-galan/</t>
+          <t>https://www.elespectador.com/colombia/barranquilla/por-explotacion-sexual-capturaron-a-estadounidense-en-hotel-del-norte-de-barranquilla/</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>La representante indicó que la reunión se realizaría a puerta cerrada y que esta decisión contradice los intereses de su partido. Además, afirmó que al gobierno local le falta implementar políticas dirigidas a los jóvenes y a la prevención de...</t>
+          <t>Las autoridades capturaron a un extranjero y a una joven de 19 años por explotación sexual de menor de edad y proxenetismo.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Asesinan a joven de 15 años en Cartagena; su padre resultó herido al intentar defenderlo</t>
+          <t>Estudiantes de un colegio en La Ceja, Antioquia, impidieron la construcción de un hospital sobre un humedal</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -834,29 +830,29 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/asesinan-a-menor-de-15-anos-en-cartagena-su-padre-resulto-herido-al-intentar-defenderlo/</t>
+          <t>https://www.las2orillas.co/estudiantes-de-un-colegio-en-la-ceja-antioquia-impidieron-la-construccion-de-un-hospital-sobre-un-humedal/</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>El presunto homicida ya fue localizado y detenido.</t>
+          <t>Estudiantes y docentes del Bernardo Uribe Londoño marchan en defensa de su humedal. Un conflicto entre la salud y el equilibrio ambiental sacude a La CejaEl artículoEstudiantes de un colegio en La Ceja, Antioquia, impidieron la construcción de un...</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Joven de 29 años ignoró síntomas creyendo que era TDAH, pero un accidente reveló un cáncer cerebral: 'Solo pedía llegar a los 30'</t>
+          <t>Mafe Carrascal explicó por qué la bancada del Pacto Histórico por Bogotá no asistió a encuentro con el alcalde Carlos Fernando Galán</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Diario ADN</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -866,39 +862,39 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.diarioadn.co/seccion/vida</t>
+          <t>https://www.infobae.com/colombia/2026/03/17/mafe-carrascal-explico-por-que-la-bancada-del-pacto-historico-por-bogota-no-asistio-a-encuentro-con-el-alcalde-carlos-fernando-galan/</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Cuando los médicos le informaron del hallazgo en su cerebro, Lauren aseguró que muchas piezas encajaron de repente. "Fue casi un alivio", señaló.</t>
+          <t>La representante indicó que la reunión se realizaría a puerta cerrada y que esta decisión contradice los intereses de su partido. Además, afirmó que al gobierno local le falta implementar políticas dirigidas a los jóvenes y a la prevención de...</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dos jóvenes fueron detenidos por presunta extorsión en Santo Tomás, Atlántico</t>
+          <t>Asesinan a joven de 15 años en Cartagena; su padre resultó herido al intentar defenderlo</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -918,7 +914,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -928,34 +924,34 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/dos-jovenes-fueron-detenidos-por-presunta-extorsion-en-santo-tomas-atlantico/</t>
+          <t>https://www.elespectador.com/colombia/asesinan-a-menor-de-15-anos-en-cartagena-su-padre-resulto-herido-al-intentar-defenderlo/</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>La investigación señala que los implicados habrían intimidado a un conductor de furgón.</t>
+          <t>El presunto homicida ya fue localizado y detenido.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Hallan el cuerpo de una adolescente en vivienda de Sahagún, Córdoba; autoridades investigan</t>
+          <t>Joven de 29 años ignoró síntomas creyendo que era TDAH, pero un accidente reveló un cáncer cerebral: 'Solo pedía llegar a los 30'</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Diario ADN</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -975,12 +971,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/hallan-el-cuerpo-de-una-menor-en-una-vivienda-de-sahagun-cordoba-autoridades-investigan/</t>
+          <t>https://www.diarioadn.co/seccion/vida</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>En lo que va de este año, este sería el tercer caso de una mujer asesinada en el municipio y el cuarto en el departamento.</t>
+          <t>Cuando los médicos le informaron del hallazgo en su cerebro, Lauren aseguró que muchas piezas encajaron de repente. "Fue casi un alivio", señaló.</t>
         </is>
       </c>
     </row>
@@ -992,27 +988,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Compensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo lograron?</t>
+          <t>Dos jóvenes fueron detenidos por presunta extorsión en Santo Tomás, Atlántico</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1022,34 +1018,34 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/compensar-firmo-un-sorprendente-acuerdo-con-una-de-las-mejores-ligas-de-futbol-del-mundo-quienes-lo-lograron/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/dos-jovenes-fueron-detenidos-por-presunta-extorsion-en-santo-tomas-atlantico/</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>La Liga española acepto hacer una alianza con la solida caja de copensacion familiar para fortalecer la formación de jóvenes talentosEl artículoCompensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo...</t>
+          <t>La investigación señala que los implicados habrían intimidado a un conductor de furgón.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pese a todo, la IA podría potenciar el criterio político de la juventud</t>
+          <t>Hallan el cuerpo de una adolescente en vivienda de Sahagún, Córdoba; autoridades investigan</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1069,29 +1065,29 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/red-de-expertos/red-de-democracia-y-tecnologia/pese-a-todo-la-ia-podria-potenciar-el-criterio-politico-de-la-juventud/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/hallan-el-cuerpo-de-una-menor-en-una-vivienda-de-sahagun-cordoba-autoridades-investigan/</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Aunque la IA genera inquietudes en el ámbito educativo, también puede formar la conciencia política e histórica entre la juventud.The postPese a todo, la IA podría potenciar el criterio político de la juventudappeared first onLa Silla Vacía.</t>
+          <t>En lo que va de este año, este sería el tercer caso de una mujer asesinada en el municipio y el cuarto en el departamento.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Murió el influencer colombiano Alejo Little a los 33 años: estos fueron los quebrantos de salud que presentó en los últimos meses</t>
+          <t>Compensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo lograron?</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1101,7 +1097,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1116,12 +1112,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/14/murio-el-influencer-colombiano-alejo-little-a-los-33-anos-estos-fueron-los-quebrantos-de-salud-que-presento-en-los-ultimos-meses/</t>
+          <t>https://www.las2orillas.co/compensar-firmo-un-sorprendente-acuerdo-con-una-de-las-mejores-ligas-de-futbol-del-mundo-quienes-lo-lograron/</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>El creador de contenido compartió experiencias sobre el acoso escolar y promovió la aceptación personal a través de sus redes sociales y charlas en instituciones educativas</t>
+          <t>La Liga española acepto hacer una alianza con la solida caja de copensacion familiar para fortalecer la formación de jóvenes talentosEl artículoCompensar firmó un sorprendente acuerdo con una de las mejores ligas de fútbol del mundo ¿Quiénes lo...</t>
         </is>
       </c>
     </row>
@@ -1133,12 +1129,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Con $86 mil millones de regalías, Bolívar construirá universidad en Montes de María y otros dos proyectos educativos</t>
+          <t>Pese a todo, la IA podría potenciar el criterio político de la juventud</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1148,12 +1144,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1163,12 +1159,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/con-86-mil-millones-de-regalias-bolivar-construira-universidad-en-montes-de-maria-y-otros-dos-proyectos-educativos/</t>
+          <t>https://www.lasillavacia.com/red-de-expertos/red-de-democracia-y-tecnologia/pese-a-todo-la-ia-podria-potenciar-el-criterio-politico-de-la-juventud/</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Los proyectos impulsados por Yamil Arana buscan, entre otras cosas, abrir más de 4 mil cupos para jóvenes de una región que durante años fue escenario de conflictoEl artículoCon $86 mil millones de regalías, Bolívar construirá universidad en Montes...</t>
+          <t>Aunque la IA genera inquietudes en el ámbito educativo, también puede formar la conciencia política e histórica entre la juventud.The postPese a todo, la IA podría potenciar el criterio político de la juventudappeared first onLa Silla Vacía.</t>
         </is>
       </c>
     </row>
@@ -1180,12 +1176,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Los therian: un fenómeno que alarma</t>
+          <t>Murió el influencer colombiano Alejo Little a los 33 años: estos fueron los quebrantos de salud que presentó en los últimos meses</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1210,29 +1206,29 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/los-therian-un-fenomeno-que-alarma/</t>
+          <t>https://www.infobae.com/colombia/2026/03/14/murio-el-influencer-colombiano-alejo-little-a-los-33-anos-estos-fueron-los-quebrantos-de-salud-que-presento-en-los-ultimos-meses/</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Cuando la identificación con un animal es persistente. se recomienda orientación psicológica para ayudar al joven en el desarrollo de una identidad saludableEl artículoLos therian: un fenómeno que alarmafue publicado originalmente enLas2orillas.co:...</t>
+          <t>El creador de contenido compartió experiencias sobre el acoso escolar y promovió la aceptación personal a través de sus redes sociales y charlas en instituciones educativas</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Figura de Independiente Medellín dedicó su gol en la clasificación del equipo en la Copa Libertadores a una persona que “está en tratamiento”</t>
+          <t>Con $86 mil millones de regalías, Bolívar construirá universidad en Montes de María y otros dos proyectos educativos</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1242,12 +1238,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1257,44 +1253,44 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/13/figura-de-independiente-medellin-dedico-su-gol-en-la-clasificacion-del-equipo-en-la-copa-libertadores-a-una-persona-que-esta-en-tratamiento/</t>
+          <t>https://www.las2orillas.co/con-86-mil-millones-de-regalias-bolivar-construira-universidad-en-montes-de-maria-y-otros-dos-proyectos-educativos/</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>El equipo dirigido por Alejandro Restrepo venció 2-1 a Juventud de Uruguay ante 12.000 hinchas y clasificó a la fase de grupos, donde acompañará a Deportes Tolima, Junior y Santa Fe en el torneo continental</t>
+          <t>Los proyectos impulsados por Yamil Arana buscan, entre otras cosas, abrir más de 4 mil cupos para jóvenes de una región que durante años fue escenario de conflictoEl artículoCon $86 mil millones de regalías, Bolívar construirá universidad en Montes...</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Abren 200 becas para jóvenes del Pacífico que lideren proyectos en sus territorios</t>
+          <t>Los therian: un fenómeno que alarma</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1304,44 +1300,44 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/abren-200-becas-para-jovenes-del-pacifico-que-lideren-proyectos-en-sus-territorios/</t>
+          <t>https://www.las2orillas.co/los-therian-un-fenomeno-que-alarma/</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>El programa DALE lidera Pacífico ofrecerá formación, mentorías y acompañamiento a jóvenes que impulsen iniciativas comunitarias en litoral.</t>
+          <t>Cuando la identificación con un animal es persistente. se recomienda orientación psicológica para ayudar al joven en el desarrollo de una identidad saludableEl artículoLos therian: un fenómeno que alarmafue publicado originalmente enLas2orillas.co:...</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
+          <t>Abren 200 becas para jóvenes del Pacífico que lideren proyectos en sus territorios</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1351,25 +1347,29 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abren-200-becas-para-jovenes-del-pacifico-que-lideren-proyectos-en-sus-territorios/</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>El programa DALE lidera Pacífico ofrecerá formación, mentorías y acompañamiento a jóvenes que impulsen iniciativas comunitarias en litoral.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
+          <t>Figura de Independiente Medellín dedicó su gol en la clasificación del equipo en la Copa Libertadores a una persona que “está en tratamiento”</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1379,12 +1379,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1394,10 +1394,14 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/deportes/2026/03/13/figura-de-independiente-medellin-dedico-su-gol-en-la-clasificacion-del-equipo-en-la-copa-libertadores-a-una-persona-que-esta-en-tratamiento/</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>El equipo dirigido por Alejandro Restrepo venció 2-1 a Juventud de Uruguay ante 12.000 hinchas y clasificó a la fase de grupos, donde acompañará a Deportes Tolima, Junior y Santa Fe en el torneo continental</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1407,12 +1411,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>La travesía del gigante telescopio que Rodolfo Llinás le regaló al histórico Observatorio de la Universidad Nacional</t>
+          <t>Solo 1 de cada 4 estudiantes colombianos logra el nivel avanzado en educación media: ¿por qué importa?</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1437,14 +1441,10 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-travesia-del-gigante-telescopio-que-rodolfo-llinas-le-regalo-al-historico-observatorio-de-la-universidad-nacional/</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>En medio del paro de la Nacional, el cientifico donó su telescopio personal, el más grande instalado en Colombia, ahora al servicio de estudiantes e investigadoresEl artículoLa travesía del gigante telescopio que Rodolfo Llinás le regaló al...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/desigualdad-en-la-educacion-media-en-colombia-solo-el-13-de-estudiantes-logra-competencias-clave-PP5091242A</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
+          <t>La travesía del gigante telescopio que Rodolfo Llinás le regaló al histórico Observatorio de la Universidad Nacional</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1484,12 +1484,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
+          <t>https://www.las2orillas.co/la-travesia-del-gigante-telescopio-que-rodolfo-llinas-le-regalo-al-historico-observatorio-de-la-universidad-nacional/</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
+          <t>En medio del paro de la Nacional, el cientifico donó su telescopio personal, el más grande instalado en Colombia, ahora al servicio de estudiantes e investigadoresEl artículoLa travesía del gigante telescopio que Rodolfo Llinás le regaló al...</t>
         </is>
       </c>
     </row>
@@ -1501,12 +1501,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Estudiantes de colegios públicos en Bogotá que tendrían que reponer clase el sábado</t>
+          <t>Gobierno geolocaliza casi 1.000 colegios en La Guajira que eran “invisibles”: no figuraban en el mapa</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1521,45 +1521,49 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/estudiantes-colegios-publicos-bogota-que-tendrian-que-reponer-clase-PP5091931A</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/03/12/gobierno-geolocaliza-casi-1000-colegios-en-la-guajira-que-eran-invisibles-no-figuraban-en-el-mapa/</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Los pocos planteles educativos con geolocalización en plataformas de ubicación están en las cabeceras municipales del departamento</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
+          <t>Estudiantes de colegios públicos en Bogotá que tendrían que reponer clase el sábado</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1574,29 +1578,25 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/bogota/estudiantes-colegios-publicos-bogota-que-tendrian-que-reponer-clase-PP5091931A</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Independiente Medellín vs. Juventud: hora y dónde ver el partido decisivo del Poderoso en la Copa Libertadores</t>
+          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1606,12 +1606,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1621,14 +1621,10 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/03/11/independiente-medellin-vs-juventud-hora-y-donde-ver-el-partido-decisivo-del-poderoso-en-la-copa-libertadores/</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>El rojo paisa quiere estar entre los 32 mejores equipos de América para la edición del 2026</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1638,22 +1634,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
+          <t>Por paro de docentes en Bogotá: Secretaría de Educación advirtió que los profesores tendrían que trabajar en sábado</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1668,12 +1664,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/paro-de-docentes-en-bogota-secretaria-de-educacion-confirmo-reposicion-de-clases-si-el-profesor-se-ausenta/</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
+          <t>Una estrategia coordinada busca que los centros escolares registren y reporten detalladamente las asistencias, horarios y participación de docentes y estudiantes, a fin de garantizar el desarrollo normal de contenidos curriculares</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1681,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
+          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1700,12 +1696,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Valledupar</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1715,12 +1711,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
+          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
         </is>
       </c>
     </row>
@@ -1732,42 +1728,42 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Prosperidad Social inicia entrega de transferencia monetaria de Jóvenes en Paz</t>
+          <t>La crisi